<commit_message>
Add Claude Code -> Hermes parity tab; log passcode-sharing event without the value
New 14_Claude_Code_Parity tab tracks, per Claude Code capability used on this
project, what Hermes-native capability would need to exist for Hermes to do it
instead -- the concrete breakdown behind GV-02's bootstrap-sunset goal. Also
escalated SV-13 (human-side passcode storage policy) to Risk after today's vault
passphrase was shared directly in chat; the literal value is not stored anywhere,
only the fact that the gap it points to is real.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Hermes_Way.xlsx
+++ b/Hermes_Way.xlsx
@@ -24,6 +24,7 @@
     <sheet name="11_Cost_Subscriptions" sheetId="15" state="visible" r:id="rId15"/>
     <sheet name="12_Security_Hardening" sheetId="16" state="visible" r:id="rId16"/>
     <sheet name="13_Governance_Change_Mgmt" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet name="14_Claude_Code_Parity" sheetId="18" state="visible" r:id="rId18"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -611,7 +612,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A57"/>
+  <dimension ref="A1:A58"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -989,6 +990,13 @@
       <c r="A57" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">  13_Governance_Change_Mgmt      how this stays coherent as it grows</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  14_Claude_Code_Parity         what Claude Code does today, mapped to the Hermes-native capability needed to retire it</t>
         </is>
       </c>
     </row>
@@ -4427,7 +4435,11 @@
           <t>Hermes Design Specialist</t>
         </is>
       </c>
-      <c r="J6" s="8" t="inlineStr"/>
+      <c r="J6" s="8" t="inlineStr">
+        <is>
+          <t>See 14_Claude_Code_Parity for the concrete per-capability breakdown of what this actually requires</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="8" t="inlineStr">
@@ -4618,6 +4630,679 @@
     <mergeCell ref="A2:J2"/>
   </mergeCells>
   <conditionalFormatting sqref="E5:E10">
+    <cfRule type="cellIs" priority="1" operator="equal" dxfId="3">
+      <formula>"Done"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="2" operator="equal" dxfId="4">
+      <formula>"Partial"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="3" operator="equal" dxfId="5">
+      <formula>"Not Started"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="4" operator="equal" dxfId="6">
+      <formula>"Risk"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="5" operator="equal" dxfId="7">
+      <formula>"Violation"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="000E7C7B"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J18"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="8" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="54" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="42" customWidth="1" min="6" max="6"/>
+    <col width="7" customWidth="1" min="7" max="7"/>
+    <col width="10" customWidth="1" min="8" max="8"/>
+    <col width="22" customWidth="1" min="9" max="9"/>
+    <col width="44" customWidth="1" min="10" max="10"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="22" customHeight="1">
+      <c r="A1" s="6" t="inlineStr">
+        <is>
+          <t>Claude Code → Hermes Parity</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="16" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>The replacement lens: for everything Claude Code does on this project today, what Hermes-native capability would need to do it instead — so Claude Code can actually be retired, not just described as temporary.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="7" t="inlineStr">
+        <is>
+          <t>ID</t>
+        </is>
+      </c>
+      <c r="B4" s="7" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="C4" s="7" t="inlineStr">
+        <is>
+          <t>Description (execution level)</t>
+        </is>
+      </c>
+      <c r="D4" s="7" t="inlineStr">
+        <is>
+          <t>Must Live On</t>
+        </is>
+      </c>
+      <c r="E4" s="7" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="F4" s="7" t="inlineStr">
+        <is>
+          <t>Evidence / Location</t>
+        </is>
+      </c>
+      <c r="G4" s="7" t="inlineStr">
+        <is>
+          <t>Points</t>
+        </is>
+      </c>
+      <c r="H4" s="7" t="inlineStr">
+        <is>
+          <t>Points Earned</t>
+        </is>
+      </c>
+      <c r="I4" s="7" t="inlineStr">
+        <is>
+          <t>Owner Role</t>
+        </is>
+      </c>
+      <c r="J4" s="7" t="inlineStr">
+        <is>
+          <t>Notes / Next Action</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="8" t="inlineStr">
+        <is>
+          <t>CCP-01</t>
+        </is>
+      </c>
+      <c r="B5" s="8" t="inlineStr">
+        <is>
+          <t>Catalog read/write parity</t>
+        </is>
+      </c>
+      <c r="C5" s="8" t="inlineStr">
+        <is>
+          <t>Claude Code drives catalog_mcp.py by hand each session. The tool itself already runs on hermes-vps (TM-01) — the gap is usage, not capability: Hermes isn't the one calling it as part of its own memory loop yet.</t>
+        </is>
+      </c>
+      <c r="D5" s="8" t="inlineStr">
+        <is>
+          <t>Hermes-VPS</t>
+        </is>
+      </c>
+      <c r="E5" s="8" t="inlineStr">
+        <is>
+          <t>Partial</t>
+        </is>
+      </c>
+      <c r="F5" s="8" t="inlineStr">
+        <is>
+          <t>TM-01</t>
+        </is>
+      </c>
+      <c r="G5" s="8" t="n">
+        <v>5</v>
+      </c>
+      <c r="H5" s="8">
+        <f>IF(E5="Done",G5,IF(E5="Partial",G5*0.5,0))</f>
+        <v/>
+      </c>
+      <c r="I5" s="8" t="inlineStr">
+        <is>
+          <t>Hermes Design Specialist</t>
+        </is>
+      </c>
+      <c r="J5" s="8" t="inlineStr">
+        <is>
+          <t>Tool parity exists; usage parity doesn't</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="8" t="inlineStr">
+        <is>
+          <t>CCP-02</t>
+        </is>
+      </c>
+      <c r="B6" s="8" t="inlineStr">
+        <is>
+          <t>Vault secret access parity</t>
+        </is>
+      </c>
+      <c r="C6" s="8" t="inlineStr">
+        <is>
+          <t>Same gap as CCP-01, blocked further by the 4x vault_mcp.py duplication.</t>
+        </is>
+      </c>
+      <c r="D6" s="8" t="inlineStr">
+        <is>
+          <t>Hermes-VPS</t>
+        </is>
+      </c>
+      <c r="E6" s="8" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F6" s="8" t="inlineStr">
+        <is>
+          <t>TM-06 / SV-12</t>
+        </is>
+      </c>
+      <c r="G6" s="8" t="n">
+        <v>5</v>
+      </c>
+      <c r="H6" s="8">
+        <f>IF(E6="Done",G6,IF(E6="Partial",G6*0.5,0))</f>
+        <v/>
+      </c>
+      <c r="I6" s="8" t="inlineStr">
+        <is>
+          <t>Secrets Custodian</t>
+        </is>
+      </c>
+      <c r="J6" s="8" t="inlineStr">
+        <is>
+          <t>Consolidate first, then shift usage to Hermes</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="8" t="inlineStr">
+        <is>
+          <t>CCP-03</t>
+        </is>
+      </c>
+      <c r="B7" s="8" t="inlineStr">
+        <is>
+          <t>Salt/infra command parity</t>
+        </is>
+      </c>
+      <c r="C7" s="8" t="inlineStr">
+        <is>
+          <t>infra_mcp.py already registered on hermes-vps (TM-04) — same usage-parity gap as CCP-01.</t>
+        </is>
+      </c>
+      <c r="D7" s="8" t="inlineStr">
+        <is>
+          <t>Hermes-VPS</t>
+        </is>
+      </c>
+      <c r="E7" s="8" t="inlineStr">
+        <is>
+          <t>Partial</t>
+        </is>
+      </c>
+      <c r="F7" s="8" t="inlineStr">
+        <is>
+          <t>TM-04</t>
+        </is>
+      </c>
+      <c r="G7" s="8" t="n">
+        <v>5</v>
+      </c>
+      <c r="H7" s="8">
+        <f>IF(E7="Done",G7,IF(E7="Partial",G7*0.5,0))</f>
+        <v/>
+      </c>
+      <c r="I7" s="8" t="inlineStr">
+        <is>
+          <t>Home-Network Liaison</t>
+        </is>
+      </c>
+      <c r="J7" s="8" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="8" t="inlineStr">
+        <is>
+          <t>CCP-04</t>
+        </is>
+      </c>
+      <c r="B8" s="8" t="inlineStr">
+        <is>
+          <t>Git repository upkeep (commit/push)</t>
+        </is>
+      </c>
+      <c r="C8" s="8" t="inlineStr">
+        <is>
+          <t>Claude Code commits/pushes to this repo via direct shell git commands on this laptop. No Hermes-native equivalent exists at all — Hermes would need a git/GitHub-aware tool (wrapping gh/git with its own deploy key) reachable from hermes-vps.</t>
+        </is>
+      </c>
+      <c r="D8" s="8" t="inlineStr">
+        <is>
+          <t>Either / Bridge</t>
+        </is>
+      </c>
+      <c r="E8" s="8" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F8" s="8" t="inlineStr"/>
+      <c r="G8" s="8" t="n">
+        <v>8</v>
+      </c>
+      <c r="H8" s="8">
+        <f>IF(E8="Done",G8,IF(E8="Partial",G8*0.5,0))</f>
+        <v/>
+      </c>
+      <c r="I8" s="8" t="inlineStr">
+        <is>
+          <t>Hermes Design Specialist</t>
+        </is>
+      </c>
+      <c r="J8" s="8" t="inlineStr">
+        <is>
+          <t>Real gap, not just a usage shift — nothing lets Hermes itself touch this repo today</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="8" t="inlineStr">
+        <is>
+          <t>CCP-05</t>
+        </is>
+      </c>
+      <c r="B9" s="8" t="inlineStr">
+        <is>
+          <t>Repo file editing / code changes</t>
+        </is>
+      </c>
+      <c r="C9" s="8" t="inlineStr">
+        <is>
+          <t>Claude Code edits this project's files directly via local tools. Hermes-native equivalent would be one of its sandboxed execution backends (local/Docker/SSH/Modal) pointed at the repo.</t>
+        </is>
+      </c>
+      <c r="D9" s="8" t="inlineStr">
+        <is>
+          <t>Either / Bridge</t>
+        </is>
+      </c>
+      <c r="E9" s="8" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F9" s="8" t="inlineStr"/>
+      <c r="G9" s="8" t="n">
+        <v>8</v>
+      </c>
+      <c r="H9" s="8">
+        <f>IF(E9="Done",G9,IF(E9="Partial",G9*0.5,0))</f>
+        <v/>
+      </c>
+      <c r="I9" s="8" t="inlineStr">
+        <is>
+          <t>Hermes Design Specialist</t>
+        </is>
+      </c>
+      <c r="J9" s="8" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="8" t="inlineStr">
+        <is>
+          <t>CCP-06</t>
+        </is>
+      </c>
+      <c r="B10" s="8" t="inlineStr">
+        <is>
+          <t>Document / spreadsheet generation</t>
+        </is>
+      </c>
+      <c r="C10" s="8" t="inlineStr">
+        <is>
+          <t>This very workbook was built with openpyxl in a local venv. No Hermes-native equivalent — would need a scripting execution backend (Modal job or Dokploy-hosted script) capable of the same generation step.</t>
+        </is>
+      </c>
+      <c r="D10" s="8" t="inlineStr">
+        <is>
+          <t>Hermes-VPS</t>
+        </is>
+      </c>
+      <c r="E10" s="8" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F10" s="8" t="inlineStr"/>
+      <c r="G10" s="8" t="n">
+        <v>5</v>
+      </c>
+      <c r="H10" s="8">
+        <f>IF(E10="Done",G10,IF(E10="Partial",G10*0.5,0))</f>
+        <v/>
+      </c>
+      <c r="I10" s="8" t="inlineStr">
+        <is>
+          <t>Platform/SRE</t>
+        </is>
+      </c>
+      <c r="J10" s="8" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="8" t="inlineStr">
+        <is>
+          <t>CCP-07</t>
+        </is>
+      </c>
+      <c r="B11" s="8" t="inlineStr">
+        <is>
+          <t>Shareable web output</t>
+        </is>
+      </c>
+      <c r="C11" s="8" t="inlineStr">
+        <is>
+          <t>Claude Code used Claude.ai's own Artifact tool for the earlier status page. The direct Hermes-native analogue is already tracked as CR-08 (Hermes-hosted web presence) — this row just names the Claude-Code-specific trigger for closing it.</t>
+        </is>
+      </c>
+      <c r="D11" s="8" t="inlineStr">
+        <is>
+          <t>Hermes-VPS</t>
+        </is>
+      </c>
+      <c r="E11" s="8" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F11" s="8" t="inlineStr">
+        <is>
+          <t>CR-08</t>
+        </is>
+      </c>
+      <c r="G11" s="8" t="n">
+        <v>3</v>
+      </c>
+      <c r="H11" s="8">
+        <f>IF(E11="Done",G11,IF(E11="Partial",G11*0.5,0))</f>
+        <v/>
+      </c>
+      <c r="I11" s="8" t="inlineStr">
+        <is>
+          <t>Hermes Design Specialist</t>
+        </is>
+      </c>
+      <c r="J11" s="8" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="8" t="inlineStr">
+        <is>
+          <t>CCP-08</t>
+        </is>
+      </c>
+      <c r="B12" s="8" t="inlineStr">
+        <is>
+          <t>Web search / page fetch</t>
+        </is>
+      </c>
+      <c r="C12" s="8" t="inlineStr">
+        <is>
+          <t>Claude Code has its own WebSearch/WebFetch tools; Hermes's search_mcp.py (TM-02) is the preferred native path and already works.</t>
+        </is>
+      </c>
+      <c r="D12" s="8" t="inlineStr">
+        <is>
+          <t>Hermes-VPS</t>
+        </is>
+      </c>
+      <c r="E12" s="8" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F12" s="8" t="inlineStr">
+        <is>
+          <t>TM-02</t>
+        </is>
+      </c>
+      <c r="G12" s="8" t="n">
+        <v>3</v>
+      </c>
+      <c r="H12" s="8">
+        <f>IF(E12="Done",G12,IF(E12="Partial",G12*0.5,0))</f>
+        <v/>
+      </c>
+      <c r="I12" s="8" t="inlineStr">
+        <is>
+          <t>Platform/SRE</t>
+        </is>
+      </c>
+      <c r="J12" s="8" t="inlineStr">
+        <is>
+          <t>Tool parity already achieved here</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="8" t="inlineStr">
+        <is>
+          <t>CCP-09</t>
+        </is>
+      </c>
+      <c r="B13" s="8" t="inlineStr">
+        <is>
+          <t>Browser automation</t>
+        </is>
+      </c>
+      <c r="C13" s="8" t="inlineStr">
+        <is>
+          <t>Claude Code has dedicated browser tools; Nous's native Tool Gateway advertises browser automation too, but it's unconfirmed/uncredentialed (same item as TM-07).</t>
+        </is>
+      </c>
+      <c r="D13" s="8" t="inlineStr">
+        <is>
+          <t>Hermes-VPS</t>
+        </is>
+      </c>
+      <c r="E13" s="8" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F13" s="8" t="inlineStr">
+        <is>
+          <t>TM-07</t>
+        </is>
+      </c>
+      <c r="G13" s="8" t="n">
+        <v>3</v>
+      </c>
+      <c r="H13" s="8">
+        <f>IF(E13="Done",G13,IF(E13="Partial",G13*0.5,0))</f>
+        <v/>
+      </c>
+      <c r="I13" s="8" t="inlineStr">
+        <is>
+          <t>Platform/SRE</t>
+        </is>
+      </c>
+      <c r="J13" s="8" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="8" t="inlineStr">
+        <is>
+          <t>CCP-10</t>
+        </is>
+      </c>
+      <c r="B14" s="8" t="inlineStr">
+        <is>
+          <t>Scheduled / recurring tasks</t>
+        </is>
+      </c>
+      <c r="C14" s="8" t="inlineStr">
+        <is>
+          <t>Claude Code's environment can schedule wakeups/cron jobs for this kind of work; whether hermes-agent exposes an equivalent internal scheduler is unconfirmed.</t>
+        </is>
+      </c>
+      <c r="D14" s="8" t="inlineStr">
+        <is>
+          <t>Hermes-VPS</t>
+        </is>
+      </c>
+      <c r="E14" s="8" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F14" s="8" t="inlineStr"/>
+      <c r="G14" s="8" t="n">
+        <v>5</v>
+      </c>
+      <c r="H14" s="8">
+        <f>IF(E14="Done",G14,IF(E14="Partial",G14*0.5,0))</f>
+        <v/>
+      </c>
+      <c r="I14" s="8" t="inlineStr">
+        <is>
+          <t>Hermes Design Specialist</t>
+        </is>
+      </c>
+      <c r="J14" s="8" t="inlineStr">
+        <is>
+          <t>Needed for things like secret-rotation reminders or nightly backup checks once those exist</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="8" t="inlineStr">
+        <is>
+          <t>CCP-11</t>
+        </is>
+      </c>
+      <c r="B15" s="8" t="inlineStr">
+        <is>
+          <t>Session / multi-step task tracking</t>
+        </is>
+      </c>
+      <c r="C15" s="8" t="inlineStr">
+        <is>
+          <t>Claude Code tracks its own task lists mid-session; unconfirmed whether hermes-agent has anything similar for tracking its own multi-step work.</t>
+        </is>
+      </c>
+      <c r="D15" s="8" t="inlineStr">
+        <is>
+          <t>Hermes-VPS</t>
+        </is>
+      </c>
+      <c r="E15" s="8" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F15" s="8" t="inlineStr"/>
+      <c r="G15" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="H15" s="8">
+        <f>IF(E15="Done",G15,IF(E15="Partial",G15*0.5,0))</f>
+        <v/>
+      </c>
+      <c r="I15" s="8" t="inlineStr">
+        <is>
+          <t>Hermes Design Specialist</t>
+        </is>
+      </c>
+      <c r="J15" s="8" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="8" t="inlineStr">
+        <is>
+          <t>CCP-12</t>
+        </is>
+      </c>
+      <c r="B16" s="8" t="inlineStr">
+        <is>
+          <t>Full bootstrap retirement criterion</t>
+        </is>
+      </c>
+      <c r="C16" s="8" t="inlineStr">
+        <is>
+          <t>The actual 'replace Claude Code with Hermes' finish line: every row above at parity, AND Hermes can perform this project's real maintenance (memory, git, infra) without Claude Code ever being opened.</t>
+        </is>
+      </c>
+      <c r="D16" s="8" t="inlineStr">
+        <is>
+          <t>N/A (process/doc)</t>
+        </is>
+      </c>
+      <c r="E16" s="8" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F16" s="8" t="inlineStr"/>
+      <c r="G16" s="8" t="n">
+        <v>10</v>
+      </c>
+      <c r="H16" s="8">
+        <f>IF(E16="Done",G16,IF(E16="Partial",G16*0.5,0))</f>
+        <v/>
+      </c>
+      <c r="I16" s="8" t="inlineStr">
+        <is>
+          <t>Hermes Design Specialist</t>
+        </is>
+      </c>
+      <c r="J16" s="8" t="inlineStr">
+        <is>
+          <t>This is GV-02's concrete success criterion</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="B18" s="16" t="inlineStr">
+        <is>
+          <t>TAB TOTAL</t>
+        </is>
+      </c>
+      <c r="G18" s="16">
+        <f>SUM(G5:G16)</f>
+        <v/>
+      </c>
+      <c r="H18" s="16">
+        <f>SUM(H5:H16)</f>
+        <v/>
+      </c>
+      <c r="I18" s="16">
+        <f>TEXT(H18/G18,"0%")&amp;" complete"</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:J1"/>
+    <mergeCell ref="A2:J2"/>
+  </mergeCells>
+  <conditionalFormatting sqref="E5:E16">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="3">
       <formula>"Done"</formula>
     </cfRule>
@@ -5381,7 +6066,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E39"/>
+  <dimension ref="A1:E41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -5745,195 +6430,182 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="12" t="inlineStr">
+      <c r="A18" s="10" t="inlineStr">
+        <is>
+          <t>14_Claude_Code_Parity</t>
+        </is>
+      </c>
+      <c r="B18" s="10" t="inlineStr">
+        <is>
+          <t>Claude Code → Hermes Parity</t>
+        </is>
+      </c>
+      <c r="C18" s="10">
+        <f>SUM(14_Claude_Code_Parity!G5:G16)</f>
+        <v/>
+      </c>
+      <c r="D18" s="10">
+        <f>SUM(14_Claude_Code_Parity!H5:H16)</f>
+        <v/>
+      </c>
+      <c r="E18" s="11">
+        <f>IFERROR(D18/C18,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="12" t="inlineStr">
         <is>
           <t>GRAND TOTAL</t>
         </is>
       </c>
-      <c r="B18" s="13" t="n"/>
-      <c r="C18" s="12">
-        <f>SUM(C5:C17)</f>
-        <v/>
-      </c>
-      <c r="D18" s="12">
-        <f>SUM(D5:D17)</f>
-        <v/>
-      </c>
-      <c r="E18" s="14">
-        <f>IFERROR(D18/C18,0)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="15" t="inlineStr">
+      <c r="B19" s="13" t="n"/>
+      <c r="C19" s="12">
+        <f>SUM(C5:C18)</f>
+        <v/>
+      </c>
+      <c r="D19" s="12">
+        <f>SUM(D5:D18)</f>
+        <v/>
+      </c>
+      <c r="E19" s="14">
+        <f>IFERROR(D19/C19,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="15" t="inlineStr">
         <is>
           <t>FINISH LINE</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="3" t="inlineStr">
-        <is>
-          <t>Hermes is 'fully realized' when ALL of the following are true at once — not just an overall percentage:</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">  1. Grand Total % Complete above is 100%, or every remaining open row is a deliberately-accepted Risk (not a Not Started).</t>
+          <t>Hermes is 'fully realized' when ALL of the following are true at once — not just an overall percentage:</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">  2. Zero rows anywhere are still status = Violation.</t>
+          <t xml:space="preserve">  1. Grand Total % Complete above is 100%, or every remaining open row is a deliberately-accepted Risk (not a Not Started).</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">  3. 03_Model_Routing_Resilience row MR-05 (WireGuard-down fire drill) is Done — this is the actual proof of the core promise.</t>
+          <t xml:space="preserve">  2. Zero rows anywhere are still status = Violation.</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">  4. 02_Identity_Memory rows IM-01 through IM-04 are Done — same Hermes, every interface, every location.</t>
+          <t xml:space="preserve">  3. 03_Model_Routing_Resilience row MR-05 (WireGuard-down fire drill) is Done — this is the actual proof of the core promise.</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="3" t="inlineStr">
         <is>
+          <t xml:space="preserve">  4. 02_Identity_Memory rows IM-01 through IM-04 are Done — same Hermes, every interface, every location.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="3" t="inlineStr">
+        <is>
           <t xml:space="preserve">  5. Only then: 11_Cost_Subscriptions CS-03 (cancel Claude Pro) gets executed.</t>
         </is>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="15" t="inlineStr">
+      <c r="A28" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  6. 14_Claude_Code_Parity row CCP-12 is Done — Hermes can maintain this project itself, so Claude Code's bootstrap role actually ends, not just gets described as temporary.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="15" t="inlineStr">
         <is>
           <t>LEGACY GOALS (catalog G1-G9) MAPPED TO THIS WORKBOOK</t>
         </is>
       </c>
     </row>
-    <row r="29">
-      <c r="A29" s="9" t="inlineStr">
+    <row r="31">
+      <c r="A31" s="9" t="inlineStr">
         <is>
           <t>Goal</t>
         </is>
       </c>
-      <c r="B29" s="9" t="inlineStr">
+      <c r="B31" s="9" t="inlineStr">
         <is>
           <t>Catalog status</t>
         </is>
       </c>
-      <c r="C29" s="9" t="inlineStr">
+      <c r="C31" s="9" t="inlineStr">
         <is>
           <t>What it actually required</t>
         </is>
       </c>
-      <c r="D29" s="9" t="inlineStr">
+      <c r="D31" s="9" t="inlineStr">
         <is>
           <t>Where that lives now</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="8" t="inlineStr">
-        <is>
-          <t>G1 — Hermes &lt;-&gt; local model, one real exchange</t>
-        </is>
-      </c>
-      <c r="B31" s="8" t="inlineStr">
-        <is>
-          <t>in_progress</t>
-        </is>
-      </c>
-      <c r="C31" s="8" t="inlineStr">
-        <is>
-          <t>Confirmed reachable + one real exchange with the local model.</t>
-        </is>
-      </c>
-      <c r="D31" s="8" t="inlineStr">
-        <is>
-          <t>03_Model_Routing_Resilience (will need re-verification once 07_Local_Inference's runtime changes)</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="8" t="inlineStr">
-        <is>
-          <t>G2 — local runtime serving multiple models concurrently</t>
-        </is>
-      </c>
-      <c r="B32" s="8" t="inlineStr">
-        <is>
-          <t>done (stale)</t>
-        </is>
-      </c>
-      <c r="C32" s="8" t="inlineStr">
-        <is>
-          <t>Verified on Ollama, multiple qwen3-vl variants loaded.</t>
-        </is>
-      </c>
-      <c r="D32" s="8" t="inlineStr">
-        <is>
-          <t>07_Local_Inference LI-03/LI-04 — must be re-proven on whichever runtime replaces Ollama</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="8" t="inlineStr">
         <is>
-          <t>G3 — VPS provisioned, hermes serve running</t>
+          <t>G1 — Hermes &lt;-&gt; local model, one real exchange</t>
         </is>
       </c>
       <c r="B33" s="8" t="inlineStr">
         <is>
-          <t>done</t>
+          <t>in_progress</t>
         </is>
       </c>
       <c r="C33" s="8" t="inlineStr">
         <is>
-          <t>Box up, agent process live.</t>
+          <t>Confirmed reachable + one real exchange with the local model.</t>
         </is>
       </c>
       <c r="D33" s="8" t="inlineStr">
         <is>
-          <t>01_Core_Runtime CR-01 to CR-03</t>
+          <t>03_Model_Routing_Resilience (will need re-verification once 07_Local_Inference's runtime changes)</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="8" t="inlineStr">
         <is>
-          <t>G4 — WireGuard tunnel, LAN reachable from VPS</t>
+          <t>G2 — local runtime serving multiple models concurrently</t>
         </is>
       </c>
       <c r="B34" s="8" t="inlineStr">
         <is>
-          <t>done</t>
+          <t>done (stale)</t>
         </is>
       </c>
       <c r="C34" s="8" t="inlineStr">
         <is>
-          <t>Tunnel + subnet routing, verified end-to-end.</t>
+          <t>Verified on Ollama, multiple qwen3-vl variants loaded.</t>
         </is>
       </c>
       <c r="D34" s="8" t="inlineStr">
         <is>
-          <t>06_Home_Network_Boundary HN-01/HN-02</t>
+          <t>07_Local_Inference LI-03/LI-04 — must be re-proven on whichever runtime replaces Ollama</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="8" t="inlineStr">
         <is>
-          <t>G5 — ChatGPT Plus linked, Codex used for real task</t>
+          <t>G3 — VPS provisioned, hermes serve running</t>
         </is>
       </c>
       <c r="B35" s="8" t="inlineStr">
@@ -5943,115 +6615,160 @@
       </c>
       <c r="C35" s="8" t="inlineStr">
         <is>
-          <t>Native link+code flow, one real coding task.</t>
+          <t>Box up, agent process live.</t>
         </is>
       </c>
       <c r="D35" s="8" t="inlineStr">
         <is>
-          <t>03_Model_Routing_Resilience MR-01</t>
+          <t>01_Core_Runtime CR-01 to CR-03</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="8" t="inlineStr">
         <is>
-          <t>G6 — Hermes Desktop on laptop, same experience 2 locations</t>
+          <t>G4 — WireGuard tunnel, LAN reachable from VPS</t>
         </is>
       </c>
       <c r="B36" s="8" t="inlineStr">
         <is>
-          <t>not_started</t>
+          <t>done</t>
         </is>
       </c>
       <c r="C36" s="8" t="inlineStr">
         <is>
-          <t>Desktop pointed at VPS backend, proven identical from two places.</t>
+          <t>Tunnel + subnet routing, verified end-to-end.</t>
         </is>
       </c>
       <c r="D36" s="8" t="inlineStr">
         <is>
-          <t>08_Interfaces_Access IA-03/IA-04, blocked on 02_Identity_Memory IM-03</t>
+          <t>06_Home_Network_Boundary HN-01/HN-02</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="8" t="inlineStr">
         <is>
-          <t>G7 — Signal/Telegram wired up</t>
+          <t>G5 — ChatGPT Plus linked, Codex used for real task</t>
         </is>
       </c>
       <c r="B37" s="8" t="inlineStr">
         <is>
-          <t>not_started</t>
+          <t>done</t>
         </is>
       </c>
       <c r="C37" s="8" t="inlineStr">
         <is>
-          <t>A real messaging channel on top of hermes-gateway.</t>
+          <t>Native link+code flow, one real coding task.</t>
         </is>
       </c>
       <c r="D37" s="8" t="inlineStr">
         <is>
-          <t>08_Interfaces_Access IA-05</t>
+          <t>03_Model_Routing_Resilience MR-01</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="8" t="inlineStr">
         <is>
-          <t>G8 — local-first routing verified end-to-end</t>
+          <t>G6 — Hermes Desktop on laptop, same experience 2 locations</t>
         </is>
       </c>
       <c r="B38" s="8" t="inlineStr">
         <is>
-          <t>not_started (likely already true, never marked)</t>
+          <t>not_started</t>
         </is>
       </c>
       <c r="C38" s="8" t="inlineStr">
         <is>
-          <t>One prompt stays local, one escalates, both observed.</t>
+          <t>Desktop pointed at VPS backend, proven identical from two places.</t>
         </is>
       </c>
       <c r="D38" s="8" t="inlineStr">
         <is>
-          <t>03_Model_Routing_Resilience — router-llm-as-judge-rebuild-2026-09-28 log entry already shows this; update the catalog goal status</t>
+          <t>08_Interfaces_Access IA-03/IA-04, blocked on 02_Identity_Memory IM-03</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="8" t="inlineStr">
         <is>
+          <t>G7 — Signal/Telegram wired up</t>
+        </is>
+      </c>
+      <c r="B39" s="8" t="inlineStr">
+        <is>
+          <t>not_started</t>
+        </is>
+      </c>
+      <c r="C39" s="8" t="inlineStr">
+        <is>
+          <t>A real messaging channel on top of hermes-gateway.</t>
+        </is>
+      </c>
+      <c r="D39" s="8" t="inlineStr">
+        <is>
+          <t>08_Interfaces_Access IA-05</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="8" t="inlineStr">
+        <is>
+          <t>G8 — local-first routing verified end-to-end</t>
+        </is>
+      </c>
+      <c r="B40" s="8" t="inlineStr">
+        <is>
+          <t>not_started (likely already true, never marked)</t>
+        </is>
+      </c>
+      <c r="C40" s="8" t="inlineStr">
+        <is>
+          <t>One prompt stays local, one escalates, both observed.</t>
+        </is>
+      </c>
+      <c r="D40" s="8" t="inlineStr">
+        <is>
+          <t>03_Model_Routing_Resilience — router-llm-as-judge-rebuild-2026-09-28 log entry already shows this; update the catalog goal status</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="8" t="inlineStr">
+        <is>
           <t>G9 — Claude Pro canceled</t>
         </is>
       </c>
-      <c r="B39" s="8" t="inlineStr">
+      <c r="B41" s="8" t="inlineStr">
         <is>
           <t>not_started</t>
         </is>
       </c>
-      <c r="C39" s="8" t="inlineStr">
+      <c r="C41" s="8" t="inlineStr">
         <is>
           <t>Cancel once ChatGPT Plus/Codex covers the same ground.</t>
         </is>
       </c>
-      <c r="D39" s="8" t="inlineStr">
+      <c r="D41" s="8" t="inlineStr">
         <is>
           <t>11_Cost_Subscriptions CS-03 — the literal finish line</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="8">
-    <mergeCell ref="A21:E21"/>
+  <mergeCells count="9">
     <mergeCell ref="A26:E26"/>
     <mergeCell ref="A24:E24"/>
     <mergeCell ref="A2:E2"/>
     <mergeCell ref="A25:E25"/>
+    <mergeCell ref="A28:E28"/>
     <mergeCell ref="A1:E1"/>
     <mergeCell ref="A23:E23"/>
     <mergeCell ref="A22:E22"/>
+    <mergeCell ref="A27:E27"/>
   </mergeCells>
-  <conditionalFormatting sqref="E5:E18">
+  <conditionalFormatting sqref="E5:E19">
     <cfRule type="dataBar" priority="1">
       <dataBar>
         <cfvo type="num" val="0"/>
@@ -9260,7 +9977,7 @@
       </c>
       <c r="C17" s="8" t="inlineStr">
         <is>
-          <t>How you yourself keep the vault passcode safe is currently undefined.</t>
+          <t>How you yourself keep the vault/Salt passcode safe is currently undefined — underscored 2026-10-03 when it was shared directly in a chat session rather than pulled from a password manager. Not persisted in plaintext anywhere by Claude; this row exists so it doesn't need to be re-typed in conversation again.</t>
         </is>
       </c>
       <c r="D17" s="8" t="inlineStr">
@@ -9270,12 +9987,16 @@
       </c>
       <c r="E17" s="8" t="inlineStr">
         <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F17" s="8" t="inlineStr"/>
+          <t>Risk</t>
+        </is>
+      </c>
+      <c r="F17" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-03 chat session</t>
+        </is>
+      </c>
       <c r="G17" s="8" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="H17" s="8">
         <f>IF(E17="Done",G17,IF(E17="Partial",G17*0.5,0))</f>
@@ -9286,7 +10007,11 @@
           <t>Product Owner (Mark)</t>
         </is>
       </c>
-      <c r="J17" s="8" t="inlineStr"/>
+      <c r="J17" s="8" t="inlineStr">
+        <is>
+          <t>Adopt a password manager / vault-native entry point so the passcode never needs to be typed into a chat again</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="B19" s="16" t="inlineStr">

</xml_diff>

<commit_message>
Drop Risk/Violation from the workbook's Status column; features only
Status now tracks completion state only (Done/Partial/Not Started). The
workbook is a feature backlog the user wants built, not an audit log Claude
runs against it on its own judgment -- context about exposure or scope creep
belongs in the Notes column, not in Status. Converted every former Risk/
Violation row accordingly and removed the now-unused color mapping.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Hermes_Way.xlsx
+++ b/Hermes_Way.xlsx
@@ -162,7 +162,7 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
   </cellStyles>
-  <dxfs count="8">
+  <dxfs count="6">
     <dxf>
       <fill>
         <patternFill patternType="solid">
@@ -220,32 +220,6 @@
       <fill>
         <patternFill patternType="solid">
           <fgColor rgb="00ECEBEC"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <name val="Arial"/>
-        <b val="1"/>
-        <color rgb="00B3412A"/>
-        <sz val="10"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="00F8E6E0"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <name val="Arial"/>
-        <b val="1"/>
-        <color rgb="009A2E13"/>
-        <sz val="10"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="00F6D9CF"/>
         </patternFill>
       </fill>
     </dxf>
@@ -792,9 +766,9 @@
       <c r="A27" s="3" t="inlineStr"/>
     </row>
     <row r="28">
-      <c r="A28" s="4" t="inlineStr">
-        <is>
-          <t>STATUS DEFINITIONS</t>
+      <c r="A28" s="3" t="inlineStr">
+        <is>
+          <t>STATUS DEFINITIONS (feature-completion only — not an audit log)</t>
         </is>
       </c>
     </row>
@@ -822,14 +796,14 @@
     <row r="32">
       <c r="A32" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Risk        exists and is live, but is a known exposure/problem by itself (not just 'missing')</t>
+          <t xml:space="preserve">  Anything worth flagging about WHY a row matters or what's exposed in the meantime belongs in Notes/Next</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Violation    actively contradicts a Hermes Way standard (see 00_Hermes_Way_Standards) right now</t>
+          <t xml:space="preserve">  Action, not in Status — Status only ever answers 'is this feature built yet.'</t>
         </is>
       </c>
     </row>
@@ -1196,7 +1170,7 @@
       </c>
       <c r="C7" s="8" t="inlineStr">
         <is>
-          <t>User's own 2026-09-23 decision was to shrink home-network involvement to just the VPN-accessed local model — Salt + MeshCentral have since been added on top, which is scope creep against that decision, not a new idea.</t>
+          <t>User's own 2026-09-23 decision was to shrink home-network involvement to just the VPN-accessed local model. Salt + MeshCentral have since been added on top — decide whether to ratify that as an intentional exception or roll it back.</t>
         </is>
       </c>
       <c r="D7" s="8" t="inlineStr">
@@ -1206,7 +1180,7 @@
       </c>
       <c r="E7" s="8" t="inlineStr">
         <is>
-          <t>Violation</t>
+          <t>Not Started</t>
         </is>
       </c>
       <c r="F7" s="8" t="inlineStr">
@@ -1296,7 +1270,7 @@
       </c>
       <c r="E9" s="8" t="inlineStr">
         <is>
-          <t>Risk</t>
+          <t>Not Started</t>
         </is>
       </c>
       <c r="F9" s="8" t="inlineStr">
@@ -1318,7 +1292,7 @@
       </c>
       <c r="J9" s="8" t="inlineStr">
         <is>
-          <t>CRITICAL</t>
+          <t>High priority — add an allowlist or disable ALLOW_ALL_USERS</t>
         </is>
       </c>
     </row>
@@ -1478,12 +1452,6 @@
     </cfRule>
     <cfRule type="cellIs" priority="3" operator="equal" dxfId="5">
       <formula>"Not Started"</formula>
-    </cfRule>
-    <cfRule type="cellIs" priority="4" operator="equal" dxfId="6">
-      <formula>"Risk"</formula>
-    </cfRule>
-    <cfRule type="cellIs" priority="5" operator="equal" dxfId="7">
-      <formula>"Violation"</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2116,12 +2084,6 @@
     <cfRule type="cellIs" priority="3" operator="equal" dxfId="5">
       <formula>"Not Started"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="4" operator="equal" dxfId="6">
-      <formula>"Risk"</formula>
-    </cfRule>
-    <cfRule type="cellIs" priority="5" operator="equal" dxfId="7">
-      <formula>"Violation"</formula>
-    </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2441,7 +2403,7 @@
       </c>
       <c r="C10" s="8" t="inlineStr">
         <is>
-          <t>Both still-open asks point the opposite direction from the 'ordinary traffic only' design — never closed out.</t>
+          <t>Both still-open asks point the opposite direction from the 'ordinary traffic only' design — a decision either way closes this out.</t>
         </is>
       </c>
       <c r="D10" s="8" t="inlineStr">
@@ -2451,7 +2413,7 @@
       </c>
       <c r="E10" s="8" t="inlineStr">
         <is>
-          <t>Risk</t>
+          <t>Not Started</t>
         </is>
       </c>
       <c r="F10" s="8" t="inlineStr">
@@ -2629,12 +2591,6 @@
     </cfRule>
     <cfRule type="cellIs" priority="3" operator="equal" dxfId="5">
       <formula>"Not Started"</formula>
-    </cfRule>
-    <cfRule type="cellIs" priority="4" operator="equal" dxfId="6">
-      <formula>"Risk"</formula>
-    </cfRule>
-    <cfRule type="cellIs" priority="5" operator="equal" dxfId="7">
-      <formula>"Violation"</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -3017,12 +2973,6 @@
     <cfRule type="cellIs" priority="3" operator="equal" dxfId="5">
       <formula>"Not Started"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="4" operator="equal" dxfId="6">
-      <formula>"Risk"</formula>
-    </cfRule>
-    <cfRule type="cellIs" priority="5" operator="equal" dxfId="7">
-      <formula>"Violation"</formula>
-    </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -3403,12 +3353,6 @@
     </cfRule>
     <cfRule type="cellIs" priority="3" operator="equal" dxfId="5">
       <formula>"Not Started"</formula>
-    </cfRule>
-    <cfRule type="cellIs" priority="4" operator="equal" dxfId="6">
-      <formula>"Risk"</formula>
-    </cfRule>
-    <cfRule type="cellIs" priority="5" operator="equal" dxfId="7">
-      <formula>"Violation"</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -3787,12 +3731,6 @@
     <cfRule type="cellIs" priority="3" operator="equal" dxfId="5">
       <formula>"Not Started"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="4" operator="equal" dxfId="6">
-      <formula>"Risk"</formula>
-    </cfRule>
-    <cfRule type="cellIs" priority="5" operator="equal" dxfId="7">
-      <formula>"Violation"</formula>
-    </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -3950,7 +3888,7 @@
       </c>
       <c r="E6" s="8" t="inlineStr">
         <is>
-          <t>Risk</t>
+          <t>Not Started</t>
         </is>
       </c>
       <c r="F6" s="8" t="inlineStr"/>
@@ -3968,7 +3906,7 @@
       </c>
       <c r="J6" s="8" t="inlineStr">
         <is>
-          <t>CRITICAL, duplicate of HN-05 by design</t>
+          <t>Duplicate of HN-05 by design</t>
         </is>
       </c>
     </row>
@@ -3995,7 +3933,7 @@
       </c>
       <c r="E7" s="8" t="inlineStr">
         <is>
-          <t>Risk</t>
+          <t>Not Started</t>
         </is>
       </c>
       <c r="F7" s="8" t="inlineStr"/>
@@ -4013,7 +3951,7 @@
       </c>
       <c r="J7" s="8" t="inlineStr">
         <is>
-          <t>CRITICAL, duplicate of SV-08 by design</t>
+          <t>Duplicate of SV-08 by design</t>
         </is>
       </c>
     </row>
@@ -4255,12 +4193,6 @@
     </cfRule>
     <cfRule type="cellIs" priority="3" operator="equal" dxfId="5">
       <formula>"Not Started"</formula>
-    </cfRule>
-    <cfRule type="cellIs" priority="4" operator="equal" dxfId="6">
-      <formula>"Risk"</formula>
-    </cfRule>
-    <cfRule type="cellIs" priority="5" operator="equal" dxfId="7">
-      <formula>"Violation"</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -4639,12 +4571,6 @@
     <cfRule type="cellIs" priority="3" operator="equal" dxfId="5">
       <formula>"Not Started"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="4" operator="equal" dxfId="6">
-      <formula>"Risk"</formula>
-    </cfRule>
-    <cfRule type="cellIs" priority="5" operator="equal" dxfId="7">
-      <formula>"Violation"</formula>
-    </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -5312,12 +5238,6 @@
     <cfRule type="cellIs" priority="3" operator="equal" dxfId="5">
       <formula>"Not Started"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="4" operator="equal" dxfId="6">
-      <formula>"Risk"</formula>
-    </cfRule>
-    <cfRule type="cellIs" priority="5" operator="equal" dxfId="7">
-      <formula>"Violation"</formula>
-    </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -5378,7 +5298,7 @@
       </c>
       <c r="E4" s="7" t="inlineStr">
         <is>
-          <t>Where it's violated today</t>
+          <t>Current gap, if any</t>
         </is>
       </c>
       <c r="F4" s="7" t="inlineStr">
@@ -6066,7 +5986,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E41"/>
+  <dimension ref="A1:E40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -6490,28 +6410,28 @@
     <row r="23">
       <c r="A23" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">  1. Grand Total % Complete above is 100%, or every remaining open row is a deliberately-accepted Risk (not a Not Started).</t>
+          <t xml:space="preserve">  1. Grand Total % Complete above is 100%, or every remaining open row has a deliberate, written decision to leave it for later.</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">  2. Zero rows anywhere are still status = Violation.</t>
+          <t xml:space="preserve">  2. 03_Model_Routing_Resilience row MR-05 (WireGuard-down fire drill) is Done — this is the actual proof of the core promise.</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">  3. 03_Model_Routing_Resilience row MR-05 (WireGuard-down fire drill) is Done — this is the actual proof of the core promise.</t>
+          <t xml:space="preserve">  3. 02_Identity_Memory rows IM-01 through IM-04 are Done — same Hermes, every interface, every location.</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">  4. 02_Identity_Memory rows IM-01 through IM-04 are Done — same Hermes, every interface, every location.</t>
+          <t xml:space="preserve">  4. 14_Claude_Code_Parity row CCP-12 is Done — Hermes can maintain this project itself, so Claude Code's bootstrap role actually ends, not just gets described as temporary.</t>
         </is>
       </c>
     </row>
@@ -6522,90 +6442,105 @@
         </is>
       </c>
     </row>
-    <row r="28">
-      <c r="A28" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  6. 14_Claude_Code_Parity row CCP-12 is Done — Hermes can maintain this project itself, so Claude Code's bootstrap role actually ends, not just gets described as temporary.</t>
+    <row r="29">
+      <c r="A29" s="15" t="inlineStr">
+        <is>
+          <t>LEGACY GOALS (catalog G1-G9) MAPPED TO THIS WORKBOOK</t>
         </is>
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="15" t="inlineStr">
-        <is>
-          <t>LEGACY GOALS (catalog G1-G9) MAPPED TO THIS WORKBOOK</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="9" t="inlineStr">
+      <c r="A30" s="9" t="inlineStr">
         <is>
           <t>Goal</t>
         </is>
       </c>
-      <c r="B31" s="9" t="inlineStr">
+      <c r="B30" s="9" t="inlineStr">
         <is>
           <t>Catalog status</t>
         </is>
       </c>
-      <c r="C31" s="9" t="inlineStr">
+      <c r="C30" s="9" t="inlineStr">
         <is>
           <t>What it actually required</t>
         </is>
       </c>
-      <c r="D31" s="9" t="inlineStr">
+      <c r="D30" s="9" t="inlineStr">
         <is>
           <t>Where that lives now</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="8" t="inlineStr">
+        <is>
+          <t>G1 — Hermes &lt;-&gt; local model, one real exchange</t>
+        </is>
+      </c>
+      <c r="B32" s="8" t="inlineStr">
+        <is>
+          <t>in_progress</t>
+        </is>
+      </c>
+      <c r="C32" s="8" t="inlineStr">
+        <is>
+          <t>Confirmed reachable + one real exchange with the local model.</t>
+        </is>
+      </c>
+      <c r="D32" s="8" t="inlineStr">
+        <is>
+          <t>03_Model_Routing_Resilience (will need re-verification once 07_Local_Inference's runtime changes)</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="8" t="inlineStr">
         <is>
-          <t>G1 — Hermes &lt;-&gt; local model, one real exchange</t>
+          <t>G2 — local runtime serving multiple models concurrently</t>
         </is>
       </c>
       <c r="B33" s="8" t="inlineStr">
         <is>
-          <t>in_progress</t>
+          <t>done (stale)</t>
         </is>
       </c>
       <c r="C33" s="8" t="inlineStr">
         <is>
-          <t>Confirmed reachable + one real exchange with the local model.</t>
+          <t>Verified on Ollama, multiple qwen3-vl variants loaded.</t>
         </is>
       </c>
       <c r="D33" s="8" t="inlineStr">
         <is>
-          <t>03_Model_Routing_Resilience (will need re-verification once 07_Local_Inference's runtime changes)</t>
+          <t>07_Local_Inference LI-03/LI-04 — must be re-proven on whichever runtime replaces Ollama</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="8" t="inlineStr">
         <is>
-          <t>G2 — local runtime serving multiple models concurrently</t>
+          <t>G3 — VPS provisioned, hermes serve running</t>
         </is>
       </c>
       <c r="B34" s="8" t="inlineStr">
         <is>
-          <t>done (stale)</t>
+          <t>done</t>
         </is>
       </c>
       <c r="C34" s="8" t="inlineStr">
         <is>
-          <t>Verified on Ollama, multiple qwen3-vl variants loaded.</t>
+          <t>Box up, agent process live.</t>
         </is>
       </c>
       <c r="D34" s="8" t="inlineStr">
         <is>
-          <t>07_Local_Inference LI-03/LI-04 — must be re-proven on whichever runtime replaces Ollama</t>
+          <t>01_Core_Runtime CR-01 to CR-03</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="8" t="inlineStr">
         <is>
-          <t>G3 — VPS provisioned, hermes serve running</t>
+          <t>G4 — WireGuard tunnel, LAN reachable from VPS</t>
         </is>
       </c>
       <c r="B35" s="8" t="inlineStr">
@@ -6615,19 +6550,19 @@
       </c>
       <c r="C35" s="8" t="inlineStr">
         <is>
-          <t>Box up, agent process live.</t>
+          <t>Tunnel + subnet routing, verified end-to-end.</t>
         </is>
       </c>
       <c r="D35" s="8" t="inlineStr">
         <is>
-          <t>01_Core_Runtime CR-01 to CR-03</t>
+          <t>06_Home_Network_Boundary HN-01/HN-02</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="8" t="inlineStr">
         <is>
-          <t>G4 — WireGuard tunnel, LAN reachable from VPS</t>
+          <t>G5 — ChatGPT Plus linked, Codex used for real task</t>
         </is>
       </c>
       <c r="B36" s="8" t="inlineStr">
@@ -6637,41 +6572,41 @@
       </c>
       <c r="C36" s="8" t="inlineStr">
         <is>
-          <t>Tunnel + subnet routing, verified end-to-end.</t>
+          <t>Native link+code flow, one real coding task.</t>
         </is>
       </c>
       <c r="D36" s="8" t="inlineStr">
         <is>
-          <t>06_Home_Network_Boundary HN-01/HN-02</t>
+          <t>03_Model_Routing_Resilience MR-01</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="8" t="inlineStr">
         <is>
-          <t>G5 — ChatGPT Plus linked, Codex used for real task</t>
+          <t>G6 — Hermes Desktop on laptop, same experience 2 locations</t>
         </is>
       </c>
       <c r="B37" s="8" t="inlineStr">
         <is>
-          <t>done</t>
+          <t>not_started</t>
         </is>
       </c>
       <c r="C37" s="8" t="inlineStr">
         <is>
-          <t>Native link+code flow, one real coding task.</t>
+          <t>Desktop pointed at VPS backend, proven identical from two places.</t>
         </is>
       </c>
       <c r="D37" s="8" t="inlineStr">
         <is>
-          <t>03_Model_Routing_Resilience MR-01</t>
+          <t>08_Interfaces_Access IA-03/IA-04, blocked on 02_Identity_Memory IM-03</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="8" t="inlineStr">
         <is>
-          <t>G6 — Hermes Desktop on laptop, same experience 2 locations</t>
+          <t>G7 — Signal/Telegram wired up</t>
         </is>
       </c>
       <c r="B38" s="8" t="inlineStr">
@@ -6681,88 +6616,65 @@
       </c>
       <c r="C38" s="8" t="inlineStr">
         <is>
-          <t>Desktop pointed at VPS backend, proven identical from two places.</t>
+          <t>A real messaging channel on top of hermes-gateway.</t>
         </is>
       </c>
       <c r="D38" s="8" t="inlineStr">
         <is>
-          <t>08_Interfaces_Access IA-03/IA-04, blocked on 02_Identity_Memory IM-03</t>
+          <t>08_Interfaces_Access IA-05</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="8" t="inlineStr">
         <is>
-          <t>G7 — Signal/Telegram wired up</t>
+          <t>G8 — local-first routing verified end-to-end</t>
         </is>
       </c>
       <c r="B39" s="8" t="inlineStr">
         <is>
-          <t>not_started</t>
+          <t>not_started (likely already true, never marked)</t>
         </is>
       </c>
       <c r="C39" s="8" t="inlineStr">
         <is>
-          <t>A real messaging channel on top of hermes-gateway.</t>
+          <t>One prompt stays local, one escalates, both observed.</t>
         </is>
       </c>
       <c r="D39" s="8" t="inlineStr">
         <is>
-          <t>08_Interfaces_Access IA-05</t>
+          <t>03_Model_Routing_Resilience — router-llm-as-judge-rebuild-2026-09-28 log entry already shows this; update the catalog goal status</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="8" t="inlineStr">
         <is>
-          <t>G8 — local-first routing verified end-to-end</t>
+          <t>G9 — Claude Pro canceled</t>
         </is>
       </c>
       <c r="B40" s="8" t="inlineStr">
         <is>
-          <t>not_started (likely already true, never marked)</t>
+          <t>not_started</t>
         </is>
       </c>
       <c r="C40" s="8" t="inlineStr">
         <is>
-          <t>One prompt stays local, one escalates, both observed.</t>
+          <t>Cancel once ChatGPT Plus/Codex covers the same ground.</t>
         </is>
       </c>
       <c r="D40" s="8" t="inlineStr">
         <is>
-          <t>03_Model_Routing_Resilience — router-llm-as-judge-rebuild-2026-09-28 log entry already shows this; update the catalog goal status</t>
-        </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" s="8" t="inlineStr">
-        <is>
-          <t>G9 — Claude Pro canceled</t>
-        </is>
-      </c>
-      <c r="B41" s="8" t="inlineStr">
-        <is>
-          <t>not_started</t>
-        </is>
-      </c>
-      <c r="C41" s="8" t="inlineStr">
-        <is>
-          <t>Cancel once ChatGPT Plus/Codex covers the same ground.</t>
-        </is>
-      </c>
-      <c r="D41" s="8" t="inlineStr">
-        <is>
           <t>11_Cost_Subscriptions CS-03 — the literal finish line</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="9">
+  <mergeCells count="8">
     <mergeCell ref="A26:E26"/>
     <mergeCell ref="A24:E24"/>
     <mergeCell ref="A2:E2"/>
     <mergeCell ref="A25:E25"/>
-    <mergeCell ref="A28:E28"/>
     <mergeCell ref="A1:E1"/>
     <mergeCell ref="A23:E23"/>
     <mergeCell ref="A22:E22"/>
@@ -7252,7 +7164,7 @@
       </c>
       <c r="E13" s="8" t="inlineStr">
         <is>
-          <t>Violation</t>
+          <t>Not Started</t>
         </is>
       </c>
       <c r="F13" s="8" t="inlineStr">
@@ -7524,12 +7436,6 @@
     </cfRule>
     <cfRule type="cellIs" priority="3" operator="equal" dxfId="5">
       <formula>"Not Started"</formula>
-    </cfRule>
-    <cfRule type="cellIs" priority="4" operator="equal" dxfId="6">
-      <formula>"Risk"</formula>
-    </cfRule>
-    <cfRule type="cellIs" priority="5" operator="equal" dxfId="7">
-      <formula>"Violation"</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -8002,12 +7908,6 @@
     <cfRule type="cellIs" priority="3" operator="equal" dxfId="5">
       <formula>"Not Started"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="4" operator="equal" dxfId="6">
-      <formula>"Risk"</formula>
-    </cfRule>
-    <cfRule type="cellIs" priority="5" operator="equal" dxfId="7">
-      <formula>"Violation"</formula>
-    </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -8650,12 +8550,6 @@
     </cfRule>
     <cfRule type="cellIs" priority="3" operator="equal" dxfId="5">
       <formula>"Not Started"</formula>
-    </cfRule>
-    <cfRule type="cellIs" priority="4" operator="equal" dxfId="6">
-      <formula>"Risk"</formula>
-    </cfRule>
-    <cfRule type="cellIs" priority="5" operator="equal" dxfId="7">
-      <formula>"Violation"</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -8848,12 +8742,12 @@
       </c>
       <c r="B7" s="8" t="inlineStr">
         <is>
-          <t>fetch_page tool-recognition bug</t>
+          <t>fetch_page tool-recognition fixed</t>
         </is>
       </c>
       <c r="C7" s="8" t="inlineStr">
         <is>
-          <t>Model inconsistently recognizes the tool exists across invocation modes (chat -q vs -z --cli) — root cause not isolated.</t>
+          <t>Model inconsistently recognizes the tool exists across invocation modes (chat -q vs -z --cli) — root cause not isolated yet.</t>
         </is>
       </c>
       <c r="D7" s="8" t="inlineStr">
@@ -8863,7 +8757,7 @@
       </c>
       <c r="E7" s="8" t="inlineStr">
         <is>
-          <t>Risk</t>
+          <t>Not Started</t>
         </is>
       </c>
       <c r="F7" s="8" t="inlineStr">
@@ -8998,7 +8892,7 @@
       </c>
       <c r="E10" s="8" t="inlineStr">
         <is>
-          <t>Violation</t>
+          <t>Not Started</t>
         </is>
       </c>
       <c r="F10" s="8" t="inlineStr">
@@ -9348,12 +9242,6 @@
     </cfRule>
     <cfRule type="cellIs" priority="3" operator="equal" dxfId="5">
       <formula>"Not Started"</formula>
-    </cfRule>
-    <cfRule type="cellIs" priority="4" operator="equal" dxfId="6">
-      <formula>"Risk"</formula>
-    </cfRule>
-    <cfRule type="cellIs" priority="5" operator="equal" dxfId="7">
-      <formula>"Violation"</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -9751,7 +9639,7 @@
       </c>
       <c r="B12" s="8" t="inlineStr">
         <is>
-          <t>/Dockers share plaintext .env exposure</t>
+          <t>/Dockers share plaintext .env exposure remediated</t>
         </is>
       </c>
       <c r="C12" s="8" t="inlineStr">
@@ -9766,7 +9654,7 @@
       </c>
       <c r="E12" s="8" t="inlineStr">
         <is>
-          <t>Risk</t>
+          <t>Not Started</t>
         </is>
       </c>
       <c r="F12" s="8" t="inlineStr">
@@ -9932,7 +9820,7 @@
       </c>
       <c r="C16" s="8" t="inlineStr">
         <is>
-          <t>Same violation as TM-06 — tracked here because it's fundamentally a secrets-handling problem, not just a tooling one.</t>
+          <t>Same item as TM-06 — tracked here because it's fundamentally a secrets-handling problem, not just a tooling one.</t>
         </is>
       </c>
       <c r="D16" s="8" t="inlineStr">
@@ -9942,7 +9830,7 @@
       </c>
       <c r="E16" s="8" t="inlineStr">
         <is>
-          <t>Violation</t>
+          <t>Not Started</t>
         </is>
       </c>
       <c r="F16" s="8" t="inlineStr">
@@ -9977,7 +9865,7 @@
       </c>
       <c r="C17" s="8" t="inlineStr">
         <is>
-          <t>How you yourself keep the vault/Salt passcode safe is currently undefined — underscored 2026-10-03 when it was shared directly in a chat session rather than pulled from a password manager. Not persisted in plaintext anywhere by Claude; this row exists so it doesn't need to be re-typed in conversation again.</t>
+          <t>Define how the vault/Salt passcode is stored and retrieved on the human side (e.g. a password manager entry) so it never needs to be typed into a chat session.</t>
         </is>
       </c>
       <c r="D17" s="8" t="inlineStr">
@@ -9987,14 +9875,10 @@
       </c>
       <c r="E17" s="8" t="inlineStr">
         <is>
-          <t>Risk</t>
-        </is>
-      </c>
-      <c r="F17" s="8" t="inlineStr">
-        <is>
-          <t>2026-10-03 chat session</t>
-        </is>
-      </c>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F17" s="8" t="inlineStr"/>
       <c r="G17" s="8" t="n">
         <v>5</v>
       </c>
@@ -10009,7 +9893,7 @@
       </c>
       <c r="J17" s="8" t="inlineStr">
         <is>
-          <t>Adopt a password manager / vault-native entry point so the passcode never needs to be typed into a chat again</t>
+          <t>Passcode was typed directly in chat on 2026-10-03; not persisted anywhere by Claude, but this feature would make that unnecessary going forward</t>
         </is>
       </c>
     </row>
@@ -10047,12 +9931,6 @@
     <cfRule type="cellIs" priority="3" operator="equal" dxfId="5">
       <formula>"Not Started"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="4" operator="equal" dxfId="6">
-      <formula>"Risk"</formula>
-    </cfRule>
-    <cfRule type="cellIs" priority="5" operator="equal" dxfId="7">
-      <formula>"Violation"</formula>
-    </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Lock in Qwen3.6-35B-A3B, log sister's separate Hermes, migrate catalog/vault
- LI-04: Qwen3.6-35B-A3B locked in after comparing Qwen3.8-27B (dense),
  Qwen3.8-Flash-Next (oversized), and a community Qwen3.8 distill (worse
  on real agentic tasks).
- CR-15/CR-16: sister gets a fully separate Hermes on its own $12/mo Vultr
  instance, not shared access -- local-model sharing left as an open question.
- SV-14/SV-15: the VPS self-sufficiency rule decided this session makes
  catalog+vault living on fileserver a rule violation, not just a resilience
  gap -- added SV-15 to track the migration to Vultr Managed Database.
- BD-02: corrected after checking the Vultr console directly -- Auto Backups
  is actually enabled (full-disk snapshot), not "nothing" as previously
  tracked.
- IM-01/IM-05: fixed SOUL.md -> MEMORY.md naming (the real file hermes-agent
  reads), and named Hindsight as the concrete extended-memory candidate.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Hermes_Way.xlsx
+++ b/Hermes_Way.xlsx
@@ -348,8 +348,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="tbl_01_Core_Runtime" displayName="tbl_01_Core_Runtime" ref="A4:J48" headerRowCount="1">
-  <autoFilter ref="A4:J48"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="tbl_01_Core_Runtime" displayName="tbl_01_Core_Runtime" ref="A4:J50" headerRowCount="1">
+  <autoFilter ref="A4:J50"/>
   <tableColumns count="10">
     <tableColumn id="1" name="ID"/>
     <tableColumn id="2" name="Feature"/>
@@ -538,8 +538,8 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="tbl_05_Secrets_Vault" displayName="tbl_05_Secrets_Vault" ref="A4:J48" headerRowCount="1">
-  <autoFilter ref="A4:J48"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="tbl_05_Secrets_Vault" displayName="tbl_05_Secrets_Vault" ref="A4:J49" headerRowCount="1">
+  <autoFilter ref="A4:J49"/>
   <tableColumns count="10">
     <tableColumn id="1" name="ID"/>
     <tableColumn id="2" name="Feature"/>
@@ -1243,7 +1243,7 @@
     <row r="49">
       <c r="A49" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">  02_Identity_Memory            SOUL.md/USER.md, cross-interface continuity</t>
+          <t xml:space="preserve">  02_Identity_Memory            MEMORY.md/USER.md, extended memory providers, cross-interface continuity</t>
         </is>
       </c>
     </row>
@@ -2507,7 +2507,7 @@
       </c>
       <c r="C8" s="8" t="inlineStr">
         <is>
-          <t>Qwen3.6-35B-A3B floated as a candidate, unbenchmarked, not pulled.</t>
+          <t>Locked in 2026-10-04: Qwen3.6-35B-A3B. Compared against Qwen3.8-27B (dense, rejected — forfeits MoE RAM-offload), Qwen3.8-Flash-Next (MoE but ~2x oversized for this RAM/VRAM budget), and a community Qwen3.8-distilled 35B-A3B (same shape, but scored worse on real agentic tasks: 10/20 vs 16/20). Chosen, not yet pulled or benchmarked.</t>
         </is>
       </c>
       <c r="D8" s="8" t="inlineStr">
@@ -2517,10 +2517,14 @@
       </c>
       <c r="E8" s="8" t="inlineStr">
         <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F8" s="8" t="inlineStr"/>
+          <t>Partial</t>
+        </is>
+      </c>
+      <c r="F8" s="8" t="inlineStr">
+        <is>
+          <t>hermes-local-model-locked-qwen3.6-35b-a3b-2026-10-04</t>
+        </is>
+      </c>
       <c r="G8" s="8" t="n">
         <v>8</v>
       </c>
@@ -2533,7 +2537,11 @@
           <t>Model/Routing Engineer</t>
         </is>
       </c>
-      <c r="J8" s="8" t="inlineStr"/>
+      <c r="J8" s="8" t="inlineStr">
+        <is>
+          <t>Pulling + benchmarking (LI-07) is the remaining step</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="8" t="inlineStr">
@@ -5300,7 +5308,7 @@
       </c>
       <c r="C6" s="8" t="inlineStr">
         <is>
-          <t>One ad hoc 306.5MB snapshot exists (taken 2026-09-29, before the install-channel migration) — but nothing recurring/scheduled backs up config.yaml, SOUL/USER.md, or MCP venvs on an ongoing basis.</t>
+          <t>Confirmed 2026-10-04 via the Vultr console: Auto Backups is Enabled on hermes-vps — a full-disk snapshot at the infrastructure level, broader than the earlier one-off app backup. Covers config.yaml/MEMORY.md/MCP venvs automatically.</t>
         </is>
       </c>
       <c r="D6" s="8" t="inlineStr">
@@ -5310,12 +5318,12 @@
       </c>
       <c r="E6" s="8" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F6" s="8" t="inlineStr">
         <is>
-          <t>hermes-migrated-to-supported-install-2026-09-29</t>
+          <t>hermes-vps-vultr-auto-backups-enabled-2026-10-04</t>
         </is>
       </c>
       <c r="G6" s="8" t="n">
@@ -5330,7 +5338,11 @@
           <t>Platform/SRE</t>
         </is>
       </c>
-      <c r="J6" s="8" t="inlineStr"/>
+      <c r="J6" s="8" t="inlineStr">
+        <is>
+          <t>Worth confirming restore has actually been tested (BD-05) despite backup existing</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="8" t="inlineStr">
@@ -10869,7 +10881,7 @@
       </c>
       <c r="E5" s="8" t="inlineStr">
         <is>
-          <t>02_Identity_Memory — session store not confirmed single, SOUL.md/USER.md not even committed yet</t>
+          <t>02_Identity_Memory — session store not confirmed single, MEMORY.md/USER.md not even committed yet</t>
         </is>
       </c>
       <c r="F5" s="8" t="inlineStr">
@@ -11590,11 +11602,11 @@
         </is>
       </c>
       <c r="C5" s="10">
-        <f>SUM('01_Core_Runtime'!G5:G48)</f>
+        <f>SUM('01_Core_Runtime'!G5:G50)</f>
         <v/>
       </c>
       <c r="D5" s="10">
-        <f>SUM('01_Core_Runtime'!H5:H48)</f>
+        <f>SUM('01_Core_Runtime'!H5:H50)</f>
         <v/>
       </c>
       <c r="E5" s="11">
@@ -11686,11 +11698,11 @@
         </is>
       </c>
       <c r="C9" s="10">
-        <f>SUM('05_Secrets_Vault'!G5:G48)</f>
+        <f>SUM('05_Secrets_Vault'!G5:G49)</f>
         <v/>
       </c>
       <c r="D9" s="10">
-        <f>SUM('05_Secrets_Vault'!H5:H48)</f>
+        <f>SUM('05_Secrets_Vault'!H5:H49)</f>
         <v/>
       </c>
       <c r="E9" s="11">
@@ -12245,7 +12257,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J50"/>
+  <dimension ref="A1:J52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -12949,34 +12961,94 @@
       <c r="J18" s="8" t="inlineStr"/>
     </row>
     <row r="19">
-      <c r="A19" s="8" t="n"/>
-      <c r="B19" s="8" t="n"/>
-      <c r="C19" s="8" t="n"/>
-      <c r="D19" s="8" t="n"/>
-      <c r="E19" s="8" t="n"/>
-      <c r="F19" s="8" t="n"/>
-      <c r="G19" s="8" t="n"/>
+      <c r="A19" s="8" t="inlineStr">
+        <is>
+          <t>CR-15</t>
+        </is>
+      </c>
+      <c r="B19" s="8" t="inlineStr">
+        <is>
+          <t>Sister's Hermes — separate VPS provisioned</t>
+        </is>
+      </c>
+      <c r="C19" s="8" t="inlineStr">
+        <is>
+          <t>Decided 2026-10-04: full separation, not a restricted-user account on this instance, so memory/context never bleeds between the two. Vultr High Performance AMD, 1 vCPU / 2GB RAM / 50GB NVMe, $12/mo, HermesAgent marketplace image — same pattern as hermes-vps.</t>
+        </is>
+      </c>
+      <c r="D19" s="8" t="inlineStr">
+        <is>
+          <t>Hermes-VPS</t>
+        </is>
+      </c>
+      <c r="E19" s="8" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F19" s="8" t="inlineStr">
+        <is>
+          <t>hermes-sister-separate-agent-2026-10-04</t>
+        </is>
+      </c>
+      <c r="G19" s="8" t="n">
+        <v>8</v>
+      </c>
       <c r="H19" s="8">
         <f>IF(E19="Done",G19,IF(E19="Partial",G19*0.5,0))</f>
         <v/>
       </c>
-      <c r="I19" s="8" t="n"/>
-      <c r="J19" s="8" t="n"/>
+      <c r="I19" s="8" t="inlineStr">
+        <is>
+          <t>Product Owner (Mark)</t>
+        </is>
+      </c>
+      <c r="J19" s="8" t="inlineStr">
+        <is>
+          <t>A second, independent deployment — not a feature of this Hermes instance</t>
+        </is>
+      </c>
     </row>
     <row r="20">
-      <c r="A20" s="8" t="n"/>
-      <c r="B20" s="8" t="n"/>
-      <c r="C20" s="8" t="n"/>
-      <c r="D20" s="8" t="n"/>
-      <c r="E20" s="8" t="n"/>
-      <c r="F20" s="8" t="n"/>
-      <c r="G20" s="8" t="n"/>
+      <c r="A20" s="8" t="inlineStr">
+        <is>
+          <t>CR-16</t>
+        </is>
+      </c>
+      <c r="B20" s="8" t="inlineStr">
+        <is>
+          <t>Sister's Hermes — local-model access decided</t>
+        </is>
+      </c>
+      <c r="C20" s="8" t="inlineStr">
+        <is>
+          <t>Open question from the planning conversation: does her instance get access to w_workstation's local model, or stay Codex/cloud-only? One RTX A4000 can't serve two simultaneous agents without one waiting on the other.</t>
+        </is>
+      </c>
+      <c r="D20" s="8" t="inlineStr">
+        <is>
+          <t>Either / Bridge</t>
+        </is>
+      </c>
+      <c r="E20" s="8" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F20" s="8" t="inlineStr"/>
+      <c r="G20" s="8" t="n">
+        <v>3</v>
+      </c>
       <c r="H20" s="8">
         <f>IF(E20="Done",G20,IF(E20="Partial",G20*0.5,0))</f>
         <v/>
       </c>
-      <c r="I20" s="8" t="n"/>
-      <c r="J20" s="8" t="n"/>
+      <c r="I20" s="8" t="inlineStr">
+        <is>
+          <t>Product Owner (Mark)</t>
+        </is>
+      </c>
+      <c r="J20" s="8" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" s="8" t="n"/>
@@ -13398,22 +13470,52 @@
       <c r="I48" s="8" t="n"/>
       <c r="J48" s="8" t="n"/>
     </row>
+    <row r="49">
+      <c r="A49" s="8" t="n"/>
+      <c r="B49" s="8" t="n"/>
+      <c r="C49" s="8" t="n"/>
+      <c r="D49" s="8" t="n"/>
+      <c r="E49" s="8" t="n"/>
+      <c r="F49" s="8" t="n"/>
+      <c r="G49" s="8" t="n"/>
+      <c r="H49" s="8">
+        <f>IF(E49="Done",G49,IF(E49="Partial",G49*0.5,0))</f>
+        <v/>
+      </c>
+      <c r="I49" s="8" t="n"/>
+      <c r="J49" s="8" t="n"/>
+    </row>
     <row r="50">
-      <c r="B50" s="20" t="inlineStr">
+      <c r="A50" s="8" t="n"/>
+      <c r="B50" s="8" t="n"/>
+      <c r="C50" s="8" t="n"/>
+      <c r="D50" s="8" t="n"/>
+      <c r="E50" s="8" t="n"/>
+      <c r="F50" s="8" t="n"/>
+      <c r="G50" s="8" t="n"/>
+      <c r="H50" s="8">
+        <f>IF(E50="Done",G50,IF(E50="Partial",G50*0.5,0))</f>
+        <v/>
+      </c>
+      <c r="I50" s="8" t="n"/>
+      <c r="J50" s="8" t="n"/>
+    </row>
+    <row r="52">
+      <c r="B52" s="20" t="inlineStr">
         <is>
           <t>TAB TOTAL (includes blank headroom rows above for future additions)</t>
         </is>
       </c>
-      <c r="G50" s="20">
-        <f>SUM(G5:G48)</f>
-        <v/>
-      </c>
-      <c r="H50" s="20">
-        <f>SUM(H5:H48)</f>
-        <v/>
-      </c>
-      <c r="I50" s="20">
-        <f>IFERROR(TEXT(H50/G50,"0%")&amp;" complete","0% complete")</f>
+      <c r="G52" s="20">
+        <f>SUM(G5:G50)</f>
+        <v/>
+      </c>
+      <c r="H52" s="20">
+        <f>SUM(H5:H50)</f>
+        <v/>
+      </c>
+      <c r="I52" s="20">
+        <f>IFERROR(TEXT(H52/G52,"0%")&amp;" complete","0% complete")</f>
         <v/>
       </c>
     </row>
@@ -13422,7 +13524,7 @@
     <mergeCell ref="A1:J1"/>
     <mergeCell ref="A2:J2"/>
   </mergeCells>
-  <conditionalFormatting sqref="E5:E48">
+  <conditionalFormatting sqref="E5:E50">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="3">
       <formula>"Done"</formula>
     </cfRule>
@@ -13536,12 +13638,12 @@
       </c>
       <c r="B5" s="8" t="inlineStr">
         <is>
-          <t>SOUL.md committed to hermes-vps</t>
+          <t>MEMORY.md committed to hermes-vps</t>
         </is>
       </c>
       <c r="C5" s="8" t="inlineStr">
         <is>
-          <t>Drafted in conversation, never actually written to the box.</t>
+          <t>Earlier plan called this SOUL.md — the real file hermes-agent reads is MEMORY.md (file-backed, 2,200-char cap, built in). Drafted in conversation, never actually written to the box.</t>
         </is>
       </c>
       <c r="D5" s="8" t="inlineStr">
@@ -13717,7 +13819,7 @@
       </c>
       <c r="C9" s="8" t="inlineStr">
         <is>
-          <t>Decision/context memory currently lives in Claude Code's bootstrap catalog habit, not in Hermes itself — per CLAUDE.md this role is meant to move into Hermes eventually.</t>
+          <t>Decision/context memory currently lives in Claude Code's bootstrap catalog habit, not in Hermes itself. Researched 2026-10-04: Hermes supports pluggable memory providers (Hindsight, Supermemory, Mnemosyne); Hindsight's local Docker mode (own Postgres, no cloud dependency) is the best fit — and if it can point at the same database as the catalog/vault once SV-15 migrates them, Hermes's memory and the project's memory become one store instead of two.</t>
         </is>
       </c>
       <c r="D9" s="8" t="inlineStr">
@@ -13732,7 +13834,7 @@
       </c>
       <c r="F9" s="8" t="inlineStr">
         <is>
-          <t>catalog (temporary) -&gt; Hermes (target)</t>
+          <t>catalog (temporary) -&gt; Hindsight (target)</t>
         </is>
       </c>
       <c r="G9" s="8" t="n">
@@ -13747,7 +13849,11 @@
           <t>Hermes Design Specialist</t>
         </is>
       </c>
-      <c r="J9" s="8" t="inlineStr"/>
+      <c r="J9" s="8" t="inlineStr">
+        <is>
+          <t>Depends on SV-15 (catalog/vault migration) landing first for the shared-database option</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="8" t="inlineStr">
@@ -16612,7 +16718,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J50"/>
+  <dimension ref="A1:J51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -17222,7 +17328,7 @@
       </c>
       <c r="C17" s="8" t="inlineStr">
         <is>
-          <t>catalog_mcp.py and vault_mcp.py on hermes-vps both call out to fileserver:3003 over the WireGuard tunnel. 03_Model_Routing_Resilience's MR-05 fire drill only covers the local model falling back to Codex — it does NOT cover what happens to Hermes's memory and secrets access if the same tunnel is down. Define whether that's an acceptable degradation (Hermes keeps answering via Codex but can't log/recall catalog memory or fetch new secrets until the tunnel's back) or whether a VPS-local cache/replica is needed.</t>
+          <t>catalog_mcp.py and vault_mcp.py on hermes-vps both call out to fileserver:3003 over the WireGuard tunnel. 03_Model_Routing_Resilience's MR-05 fire drill only covers the local model falling back to Codex — it does NOT cover what happens to Hermes's memory and secrets access if the same tunnel is down. SUPERSEDED by the 2026-10-04 VPS self-sufficiency rule: the answer isn't 'define acceptable degradation,' it's 'this dependency on the home network isn't allowed to exist' — see SV-15.</t>
         </is>
       </c>
       <c r="D17" s="8" t="inlineStr">
@@ -17250,29 +17356,29 @@
       </c>
       <c r="J17" s="8" t="inlineStr">
         <is>
-          <t>Scope gap found reviewing SV-01 — this is arguably as load-bearing as MR-05 itself</t>
+          <t>Resolved in principle by SV-15; this row closes once that migration lands</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="8" t="inlineStr">
         <is>
-          <t>SV-13</t>
+          <t>SV-15</t>
         </is>
       </c>
       <c r="B18" s="8" t="inlineStr">
         <is>
-          <t>Human-side passcode storage policy</t>
+          <t>Catalog + vault migrated off fileserver</t>
         </is>
       </c>
       <c r="C18" s="8" t="inlineStr">
         <is>
-          <t>Define how the vault/Salt passcode is stored and retrieved on the human side (e.g. a password manager entry) so it never needs to be typed into a chat session.</t>
+          <t>Required by the 2026-10-04 VPS self-sufficiency rule: hermes-vps must be able to do everything except run the local LLM without depending on the home network. Catalog + vault currently live on fileserver, which violates this. Target: Vultr Managed Database (Postgres, supports pgvector for free) — also solves IM-05's memory-provider storage need in the same move.</t>
         </is>
       </c>
       <c r="D18" s="8" t="inlineStr">
         <is>
-          <t>N/A (process/doc)</t>
+          <t>Hermes-VPS</t>
         </is>
       </c>
       <c r="E18" s="8" t="inlineStr">
@@ -17280,9 +17386,13 @@
           <t>Not Started</t>
         </is>
       </c>
-      <c r="F18" s="8" t="inlineStr"/>
+      <c r="F18" s="8" t="inlineStr">
+        <is>
+          <t>hermes-catalog-vault-migration-required-2026-10-04</t>
+        </is>
+      </c>
       <c r="G18" s="8" t="n">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="H18" s="8">
         <f>IF(E18="Done",G18,IF(E18="Partial",G18*0.5,0))</f>
@@ -17290,29 +17400,59 @@
       </c>
       <c r="I18" s="8" t="inlineStr">
         <is>
-          <t>Product Owner (Mark)</t>
+          <t>Hermes Design Specialist</t>
         </is>
       </c>
       <c r="J18" s="8" t="inlineStr">
         <is>
-          <t>Passcode was typed directly in chat on 2026-10-03; not persisted anywhere by Claude, but this feature would make that unnecessary going forward</t>
+          <t>Closes SV-14 entirely once done; also unblocks IM-05's Hindsight shared-database option</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="8" t="n"/>
-      <c r="B19" s="8" t="n"/>
-      <c r="C19" s="8" t="n"/>
-      <c r="D19" s="8" t="n"/>
-      <c r="E19" s="8" t="n"/>
-      <c r="F19" s="8" t="n"/>
-      <c r="G19" s="8" t="n"/>
+      <c r="A19" s="8" t="inlineStr">
+        <is>
+          <t>SV-13</t>
+        </is>
+      </c>
+      <c r="B19" s="8" t="inlineStr">
+        <is>
+          <t>Human-side passcode storage policy</t>
+        </is>
+      </c>
+      <c r="C19" s="8" t="inlineStr">
+        <is>
+          <t>Define how the vault/Salt passcode is stored and retrieved on the human side (e.g. a password manager entry) so it never needs to be typed into a chat session.</t>
+        </is>
+      </c>
+      <c r="D19" s="8" t="inlineStr">
+        <is>
+          <t>N/A (process/doc)</t>
+        </is>
+      </c>
+      <c r="E19" s="8" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F19" s="8" t="inlineStr"/>
+      <c r="G19" s="8" t="n">
+        <v>5</v>
+      </c>
       <c r="H19" s="8">
         <f>IF(E19="Done",G19,IF(E19="Partial",G19*0.5,0))</f>
         <v/>
       </c>
-      <c r="I19" s="8" t="n"/>
-      <c r="J19" s="8" t="n"/>
+      <c r="I19" s="8" t="inlineStr">
+        <is>
+          <t>Product Owner (Mark)</t>
+        </is>
+      </c>
+      <c r="J19" s="8" t="inlineStr">
+        <is>
+          <t>Passcode was typed directly in chat on 2026-10-03; not persisted anywhere by Claude, but this feature would make that unnecessary going forward</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="8" t="n"/>
@@ -17749,22 +17889,37 @@
       <c r="I48" s="8" t="n"/>
       <c r="J48" s="8" t="n"/>
     </row>
-    <row r="50">
-      <c r="B50" s="20" t="inlineStr">
+    <row r="49">
+      <c r="A49" s="8" t="n"/>
+      <c r="B49" s="8" t="n"/>
+      <c r="C49" s="8" t="n"/>
+      <c r="D49" s="8" t="n"/>
+      <c r="E49" s="8" t="n"/>
+      <c r="F49" s="8" t="n"/>
+      <c r="G49" s="8" t="n"/>
+      <c r="H49" s="8">
+        <f>IF(E49="Done",G49,IF(E49="Partial",G49*0.5,0))</f>
+        <v/>
+      </c>
+      <c r="I49" s="8" t="n"/>
+      <c r="J49" s="8" t="n"/>
+    </row>
+    <row r="51">
+      <c r="B51" s="20" t="inlineStr">
         <is>
           <t>TAB TOTAL (includes blank headroom rows above for future additions)</t>
         </is>
       </c>
-      <c r="G50" s="20">
-        <f>SUM(G5:G48)</f>
-        <v/>
-      </c>
-      <c r="H50" s="20">
-        <f>SUM(H5:H48)</f>
-        <v/>
-      </c>
-      <c r="I50" s="20">
-        <f>IFERROR(TEXT(H50/G50,"0%")&amp;" complete","0% complete")</f>
+      <c r="G51" s="20">
+        <f>SUM(G5:G49)</f>
+        <v/>
+      </c>
+      <c r="H51" s="20">
+        <f>SUM(H5:H49)</f>
+        <v/>
+      </c>
+      <c r="I51" s="20">
+        <f>IFERROR(TEXT(H51/G51,"0%")&amp;" complete","0% complete")</f>
         <v/>
       </c>
     </row>
@@ -17773,7 +17928,7 @@
     <mergeCell ref="A1:J1"/>
     <mergeCell ref="A2:J2"/>
   </mergeCells>
-  <conditionalFormatting sqref="E5:E48">
+  <conditionalFormatting sqref="E5:E49">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="3">
       <formula>"Done"</formula>
     </cfRule>

</xml_diff>

<commit_message>
Add D1_Vultr_Services_Audit discovery tab; price out Serverless Inference
New discovery-tab pattern: brown-tabbed, D-prefixed, reference research kept
separate from the tracked 01-15 action-item tabs so an execution-phase reader
isn't wading through research prose to find what to actually do.

First installment: full Vultr product catalog mapped against Hermes's needs.
Headline findings -- Managed Database is the fix for SV-15 (catalog/vault
migration), Cloud Firewall could close the gateway exposure (HN-05/SH-02) at
the network layer as a second line of defense, VPC becomes relevant once the
sister's-agent VPS and/or Managed Database exist.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Hermes_Way.xlsx
+++ b/Hermes_Way.xlsx
@@ -26,6 +26,7 @@
     <sheet name="13_Governance_Change_Mgmt" sheetId="17" state="visible" r:id="rId17"/>
     <sheet name="14_Claude_Code_Parity" sheetId="18" state="visible" r:id="rId18"/>
     <sheet name="15_Productivity_And_Acceptance" sheetId="19" state="visible" r:id="rId19"/>
+    <sheet name="D1_Vultr_Services_Audit" sheetId="20" state="visible" r:id="rId20"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -480,6 +481,20 @@
 </table>
 </file>
 
+<file path=xl/tables/table16.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="16" name="tbl_D1_Vultr_Services_Audit" displayName="tbl_D1_Vultr_Services_Audit" ref="A4:E18" headerRowCount="1">
+  <autoFilter ref="A4:E18"/>
+  <tableColumns count="5">
+    <tableColumn id="1" name="Service"/>
+    <tableColumn id="2" name="What it does"/>
+    <tableColumn id="3" name="Relevant to Hermes?"/>
+    <tableColumn id="4" name="Why"/>
+    <tableColumn id="5" name="Priority"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleLight11" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="tbl_02_Identity_Memory" displayName="tbl_02_Identity_Memory" ref="A4:J42" headerRowCount="1">
   <autoFilter ref="A4:J42"/>
@@ -922,7 +937,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A62"/>
+  <dimension ref="A1:A66"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -1335,6 +1350,30 @@
       <c r="A62" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">  15_Productivity_And_Acceptance  everyday usefulness (Google office, deliverables, long-running work) and how to actually prove any of it works</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="3" t="inlineStr"/>
+    </row>
+    <row r="64">
+      <c r="A64" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  DISCOVERY TABS (prefixed D#, brown tab color) — reference research, not a tracked backlog. Resulting</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  action items get added to the 01-15 tabs above, not tracked for completion here.</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  D1_Vultr_Services_Audit       what Vultr offers vs. what Hermes should actually use</t>
         </is>
       </c>
     </row>
@@ -11270,6 +11309,454 @@
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="008A5A2E"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E18"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="40" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="48" customWidth="1" min="4" max="4"/>
+    <col width="34" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="22" customHeight="1">
+      <c r="A1" s="6" t="inlineStr">
+        <is>
+          <t>Discovery — Vultr Services Audit</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="16" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>What Vultr actually offers, researched 2026-10-04, mapped against whether Hermes should use it. Reference material, not a tracked backlog — the resulting action items live in the 01-15 tabs, not here.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="7" t="inlineStr">
+        <is>
+          <t>Service</t>
+        </is>
+      </c>
+      <c r="B4" s="7" t="inlineStr">
+        <is>
+          <t>What it does</t>
+        </is>
+      </c>
+      <c r="C4" s="7" t="inlineStr">
+        <is>
+          <t>Relevant to Hermes?</t>
+        </is>
+      </c>
+      <c r="D4" s="7" t="inlineStr">
+        <is>
+          <t>Why</t>
+        </is>
+      </c>
+      <c r="E4" s="7" t="inlineStr">
+        <is>
+          <t>Priority</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="8" t="inlineStr">
+        <is>
+          <t>Cloud Compute (High Performance AMD)</t>
+        </is>
+      </c>
+      <c r="B5" s="8" t="inlineStr">
+        <is>
+          <t>VPS tiers — the box Hermes itself runs on.</t>
+        </is>
+      </c>
+      <c r="C5" s="8" t="inlineStr">
+        <is>
+          <t>Already using</t>
+        </is>
+      </c>
+      <c r="D5" s="8" t="inlineStr">
+        <is>
+          <t>hermes-vps is this; sister's agent (CR-15) will be a second one.</t>
+        </is>
+      </c>
+      <c r="E5" s="8" t="inlineStr">
+        <is>
+          <t>N/A — in use</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="8" t="inlineStr">
+        <is>
+          <t>Managed Database (Postgres, MySQL, Valkey, Kafka)</t>
+        </is>
+      </c>
+      <c r="B6" s="8" t="inlineStr">
+        <is>
+          <t>Fully-managed DB, $3.50/mo+, pgvector support free.</t>
+        </is>
+      </c>
+      <c r="C6" s="8" t="inlineStr">
+        <is>
+          <t>Yes — high priority</t>
+        </is>
+      </c>
+      <c r="D6" s="8" t="inlineStr">
+        <is>
+          <t>Direct fix for SV-15 (catalog/vault migration off fileserver) and a possible shared store for Hindsight (IM-05).</t>
+        </is>
+      </c>
+      <c r="E6" s="8" t="inlineStr">
+        <is>
+          <t>High — tracked as SV-15</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="8" t="inlineStr">
+        <is>
+          <t>Serverless Inference</t>
+        </is>
+      </c>
+      <c r="B7" s="8" t="inlineStr">
+        <is>
+          <t>Pay-per-token hosted LLMs, pre-configured on hermes-vps already.</t>
+        </is>
+      </c>
+      <c r="C7" s="8" t="inlineStr">
+        <is>
+          <t>Already using (idle)</t>
+        </is>
+      </c>
+      <c r="D7" s="8" t="inlineStr">
+        <is>
+          <t>Real fallback tier between free-local and paid-Codex — priced out this session.</t>
+        </is>
+      </c>
+      <c r="E7" s="8" t="inlineStr">
+        <is>
+          <t>Medium — reactivate as a fallback</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="8" t="inlineStr">
+        <is>
+          <t>Object Storage (S3-compatible)</t>
+        </is>
+      </c>
+      <c r="B8" s="8" t="inlineStr">
+        <is>
+          <t>Cheap unstructured storage, multiple tiers.</t>
+        </is>
+      </c>
+      <c r="C8" s="8" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D8" s="8" t="inlineStr">
+        <is>
+          <t>Natural backup destination for BD-02/BD-06.</t>
+        </is>
+      </c>
+      <c r="E8" s="8" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="8" t="inlineStr">
+        <is>
+          <t>Cloud Firewall</t>
+        </is>
+      </c>
+      <c r="B9" s="8" t="inlineStr">
+        <is>
+          <t>Managed network-level firewall, separate from the VPS's own ufw.</t>
+        </is>
+      </c>
+      <c r="C9" s="8" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D9" s="8" t="inlineStr">
+        <is>
+          <t>Could close HN-05/SH-02 (gateway shell exposure) at the network layer, not just the app config layer — a second line of defense.</t>
+        </is>
+      </c>
+      <c r="E9" s="8" t="inlineStr">
+        <is>
+          <t>High — security-relevant</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="8" t="inlineStr">
+        <is>
+          <t>VPC (private networking)</t>
+        </is>
+      </c>
+      <c r="B10" s="8" t="inlineStr">
+        <is>
+          <t>Private network between your Vultr instances, no public IP needed between them.</t>
+        </is>
+      </c>
+      <c r="C10" s="8" t="inlineStr">
+        <is>
+          <t>Yes, once there's &gt;1 instance</t>
+        </is>
+      </c>
+      <c r="D10" s="8" t="inlineStr">
+        <is>
+          <t>Once sister's VPS (CR-15) and/or a Managed Database (SV-15) exist, VPC lets them talk to hermes-vps privately instead of over the public internet.</t>
+        </is>
+      </c>
+      <c r="E10" s="8" t="inlineStr">
+        <is>
+          <t>Medium — do alongside SV-15/CR-15</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="8" t="inlineStr">
+        <is>
+          <t>Block Storage</t>
+        </is>
+      </c>
+      <c r="B11" s="8" t="inlineStr">
+        <is>
+          <t>Expandable disk volumes you attach to a VPS.</t>
+        </is>
+      </c>
+      <c r="C11" s="8" t="inlineStr">
+        <is>
+          <t>Maybe</t>
+        </is>
+      </c>
+      <c r="D11" s="8" t="inlineStr">
+        <is>
+          <t>hermes-vps's 100GB NVMe could get tight once memory providers/skills accumulate data; not urgent yet.</t>
+        </is>
+      </c>
+      <c r="E11" s="8" t="inlineStr">
+        <is>
+          <t>Low — watch CR-12 (resource headroom)</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="8" t="inlineStr">
+        <is>
+          <t>Cloud GPU / Bare Metal (GPU options)</t>
+        </is>
+      </c>
+      <c r="B12" s="8" t="inlineStr">
+        <is>
+          <t>On-demand or dedicated GPU instances.</t>
+        </is>
+      </c>
+      <c r="C12" s="8" t="inlineStr">
+        <is>
+          <t>Worth knowing, not recommended now</t>
+        </is>
+      </c>
+      <c r="D12" s="8" t="inlineStr">
+        <is>
+          <t>Could theoretically host the local model on Vultr instead of w_workstation, which would fully remove the WireGuard-down dependency (MR-05) — but at real GPU-instance cost, undercutting the whole 'free local inference' point of using owned hardware.</t>
+        </is>
+      </c>
+      <c r="E12" s="8" t="inlineStr">
+        <is>
+          <t>Low — only if the home-GPU approach is abandoned later</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="8" t="inlineStr">
+        <is>
+          <t>Kubernetes (VKE)</t>
+        </is>
+      </c>
+      <c r="B13" s="8" t="inlineStr">
+        <is>
+          <t>Managed container orchestration, free control plane.</t>
+        </is>
+      </c>
+      <c r="C13" s="8" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="D13" s="8" t="inlineStr">
+        <is>
+          <t>Overkill for one VPS running one agent; relevant only if Hermes sprawls into many containerized services.</t>
+        </is>
+      </c>
+      <c r="E13" s="8" t="inlineStr">
+        <is>
+          <t>Not now</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="8" t="inlineStr">
+        <is>
+          <t>Container Registry</t>
+        </is>
+      </c>
+      <c r="B14" s="8" t="inlineStr">
+        <is>
+          <t>Stores container images Hermes/Dokploy might build.</t>
+        </is>
+      </c>
+      <c r="C14" s="8" t="inlineStr">
+        <is>
+          <t>Already tracked (TM-07 area)</t>
+        </is>
+      </c>
+      <c r="D14" s="8" t="inlineStr">
+        <is>
+          <t>Free tier (10GB) covers this until custom images become a real need.</t>
+        </is>
+      </c>
+      <c r="E14" s="8" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="8" t="inlineStr">
+        <is>
+          <t>CDN</t>
+        </is>
+      </c>
+      <c r="B15" s="8" t="inlineStr">
+        <is>
+          <t>Edge caching for static assets.</t>
+        </is>
+      </c>
+      <c r="C15" s="8" t="inlineStr">
+        <is>
+          <t>Minor</t>
+        </is>
+      </c>
+      <c r="D15" s="8" t="inlineStr">
+        <is>
+          <t>Only relevant once CR-08 (Hermes-hosted web presence) exists and has real traffic.</t>
+        </is>
+      </c>
+      <c r="E15" s="8" t="inlineStr">
+        <is>
+          <t>Low — revisit after CR-08</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="8" t="inlineStr">
+        <is>
+          <t>DNS</t>
+        </is>
+      </c>
+      <c r="B16" s="8" t="inlineStr">
+        <is>
+          <t>Vultr's own DNS hosting.</t>
+        </is>
+      </c>
+      <c r="C16" s="8" t="inlineStr">
+        <is>
+          <t>Optional</t>
+        </is>
+      </c>
+      <c r="D16" s="8" t="inlineStr">
+        <is>
+          <t>DuckDNS already works for the existing domain; moving DNS to Vultr is a 'prefer Vultr' nice-to-have, not a need.</t>
+        </is>
+      </c>
+      <c r="E16" s="8" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="8" t="inlineStr">
+        <is>
+          <t>Marketplace one-click apps</t>
+        </is>
+      </c>
+      <c r="B17" s="8" t="inlineStr">
+        <is>
+          <t>Pre-built app images (Easypanel, CloudPanel, WireGuard, etc.)</t>
+        </is>
+      </c>
+      <c r="C17" s="8" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="D17" s="8" t="inlineStr">
+        <is>
+          <t>Dokploy already covers the container-hosting role; the WireGuard app doesn't apply since the tunnel's home-side endpoint must stay physically at home by definition.</t>
+        </is>
+      </c>
+      <c r="E17" s="8" t="inlineStr">
+        <is>
+          <t>Not applicable</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="8" t="inlineStr">
+        <is>
+          <t>Load Balancers / NAT Gateway / Direct Connect</t>
+        </is>
+      </c>
+      <c r="B18" s="8" t="inlineStr">
+        <is>
+          <t>HA traffic distribution, private hybrid-cloud links.</t>
+        </is>
+      </c>
+      <c r="C18" s="8" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="D18" s="8" t="inlineStr">
+        <is>
+          <t>Enterprise/multi-instance-at-scale features; nothing here operates at that scale.</t>
+        </is>
+      </c>
+      <c r="E18" s="8" t="inlineStr">
+        <is>
+          <t>Not applicable</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A2:E2"/>
+    <mergeCell ref="A1:E1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <tableParts count="1">
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  </tableParts>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
Correct SOUL.md/MEMORY.md conflation; deepen memory+soul discovery
A prior same-session edit wrongly concluded SOUL.md wasn't real and renamed
it to MEMORY.md. It is real and distinct: SOUL.md (~/.hermes/SOUL.md, 2200
chars) defines WHO the agent is; MEMORY.md (same cap, separate file) defines
WHAT it has learned. Restored IM-01 to SOUL.md, added IM-09 for MEMORY.md.

Enriched IM-05 (extended memory) and IM-07 (retention policy) with the real
mechanics found: agent-curated capture via self-prompts ("should I persist
this?"), a stated policy (facts aggressively, preferences once proven,
nothing sensitive ever), and Hindsight's reflect operation as the direct
technical answer to "broad scope but curated, not raw total recall."

Flagged two more of Nous's "Five Pillars" (Crons, Self-Improvement) as
zero-coverage gaps in the Read_Me so they don't get lost after Skills.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Hermes_Way.xlsx
+++ b/Hermes_Way.xlsx
@@ -496,8 +496,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="tbl_02_Identity_Memory" displayName="tbl_02_Identity_Memory" ref="A4:J42" headerRowCount="1">
-  <autoFilter ref="A4:J42"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="tbl_02_Identity_Memory" displayName="tbl_02_Identity_Memory" ref="A4:J43" headerRowCount="1">
+  <autoFilter ref="A4:J43"/>
   <tableColumns count="10">
     <tableColumn id="1" name="ID"/>
     <tableColumn id="2" name="Feature"/>
@@ -937,7 +937,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A66"/>
+  <dimension ref="A1:A72"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -1258,7 +1258,7 @@
     <row r="49">
       <c r="A49" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">  02_Identity_Memory            MEMORY.md/USER.md, extended memory providers, cross-interface continuity</t>
+          <t xml:space="preserve">  02_Identity_Memory            SOUL.md/MEMORY.md/USER.md, extended memory providers, cross-interface continuity</t>
         </is>
       </c>
     </row>
@@ -1374,6 +1374,44 @@
       <c r="A66" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">  D1_Vultr_Services_Audit       what Vultr offers vs. what Hermes should actually use</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="3" t="inlineStr"/>
+    </row>
+    <row r="68">
+      <c r="A68" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Found 2026-10-04: Nous's own framing is 'Five Pillars' -- Memory, Skills, Soul, Crons, Self-</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Improvement. Memory+Soul covered in 02_Identity_Memory. Skills queued next. Crons (built-in</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  scheduler: hermes cron list/remove/run) and Self-Improvement (the learn-from-work loop) are</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  real pillars with zero coverage anywhere in this workbook yet -- not yet researched, flagging</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  so they don't get forgotten once Skills is done.</t>
         </is>
       </c>
     </row>
@@ -10920,7 +10958,7 @@
       </c>
       <c r="E5" s="8" t="inlineStr">
         <is>
-          <t>02_Identity_Memory — session store not confirmed single, MEMORY.md/USER.md not even committed yet</t>
+          <t>02_Identity_Memory — session store not confirmed single, SOUL.md/MEMORY.md/USER.md not even committed yet</t>
         </is>
       </c>
       <c r="F5" s="8" t="inlineStr">
@@ -12113,11 +12151,11 @@
         </is>
       </c>
       <c r="C6" s="10">
-        <f>SUM('02_Identity_Memory'!G5:G42)</f>
+        <f>SUM('02_Identity_Memory'!G5:G43)</f>
         <v/>
       </c>
       <c r="D6" s="10">
-        <f>SUM('02_Identity_Memory'!H5:H42)</f>
+        <f>SUM('02_Identity_Memory'!H5:H43)</f>
         <v/>
       </c>
       <c r="E6" s="11">
@@ -14036,7 +14074,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J44"/>
+  <dimension ref="A1:J45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -14125,12 +14163,12 @@
       </c>
       <c r="B5" s="8" t="inlineStr">
         <is>
-          <t>MEMORY.md committed to hermes-vps</t>
+          <t>SOUL.md committed to hermes-vps</t>
         </is>
       </c>
       <c r="C5" s="8" t="inlineStr">
         <is>
-          <t>Earlier plan called this SOUL.md — the real file hermes-agent reads is MEMORY.md (file-backed, 2,200-char cap, built in). Drafted in conversation, never actually written to the box.</t>
+          <t>CORRECTION 2026-10-04: an earlier pass here wrongly claimed SOUL.md wasn't real — it is, and it's distinct from MEMORY.md (see IM-09). Lives at ~/.hermes/SOUL.md, 2,200-char cap, defines WHO the agent is — persona, tone, values, boundaries, judgment style. First slot in the system prompt. Auto-created with a generic default if missing; the version drafted in conversation was never actually written to the box.</t>
         </is>
       </c>
       <c r="D5" s="8" t="inlineStr">
@@ -14145,7 +14183,7 @@
       </c>
       <c r="F5" s="8" t="inlineStr">
         <is>
-          <t>hermes-vps filesystem</t>
+          <t>hermes-agent docs: user-guide/features/personality</t>
         </is>
       </c>
       <c r="G5" s="8" t="n">
@@ -14175,7 +14213,7 @@
       </c>
       <c r="C6" s="8" t="inlineStr">
         <is>
-          <t>Same status — drafted, never committed.</t>
+          <t>User profile/preferences, 1,375-char cap, distinct from both SOUL.md and MEMORY.md. Same status — drafted, never committed.</t>
         </is>
       </c>
       <c r="D6" s="8" t="inlineStr">
@@ -14301,12 +14339,12 @@
       </c>
       <c r="B9" s="8" t="inlineStr">
         <is>
-          <t>Hermes-native long-term memory</t>
+          <t>Hermes-native long-term memory (extended provider)</t>
         </is>
       </c>
       <c r="C9" s="8" t="inlineStr">
         <is>
-          <t>Decision/context memory currently lives in Claude Code's bootstrap catalog habit, not in Hermes itself. Researched 2026-10-04: Hermes supports pluggable memory providers (Hindsight, Supermemory, Mnemosyne); Hindsight's local Docker mode (own Postgres, no cloud dependency) is the best fit — and if it can point at the same database as the catalog/vault once SV-15 migrates them, Hermes's memory and the project's memory become one store instead of two.</t>
+          <t>Decision/context memory currently lives in Claude Code's bootstrap catalog habit, not in Hermes itself. Researched 2026-10-04: Hermes supports pluggable providers (Hindsight, Supermemory, Mnemosyne, others). User's actual requirement: broad scope ('anything is fair game,' Hermes = main AI tool going forward) but genuinely curated, not raw total recall ('remembering everything means remembering nothing'). Hindsight's reflect operation is built for exactly this — it reasons across all stored memories with an LLM to produce a synthesized answer, not a ranked dump; its retain operation also does entity resolution so facts link to canonical people/projects instead of floating as disconnected rows. Local Docker mode keeps this on-box, no cloud dependency, and could share a database with the migrated catalog/vault (SV-15).</t>
         </is>
       </c>
       <c r="D9" s="8" t="inlineStr">
@@ -14338,7 +14376,7 @@
       </c>
       <c r="J9" s="8" t="inlineStr">
         <is>
-          <t>Depends on SV-15 (catalog/vault migration) landing first for the shared-database option</t>
+          <t>Depends on SV-15 landing first for the shared-database option</t>
         </is>
       </c>
     </row>
@@ -14396,7 +14434,7 @@
       </c>
       <c r="C11" s="8" t="inlineStr">
         <is>
-          <t>What Hermes keeps forever vs. prunes — not defined anywhere yet.</t>
+          <t>The built-in system already has a real policy, found 2026-10-04: facts/corrections persisted aggressively, preferences/skills only once they prove themselves, nothing sensitive ever. Capture is agent-judged, not automatic — periodic self-prompts ask 'should I persist this?' (solves humans forgetting to flag what matters). Still undefined: what the SAME policy should be for an extended provider (IM-05) once it exists, which has no built-in character cap forcing curation the way MEMORY.md's 2,200-char limit does.</t>
         </is>
       </c>
       <c r="D11" s="8" t="inlineStr">
@@ -14406,10 +14444,14 @@
       </c>
       <c r="E11" s="8" t="inlineStr">
         <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F11" s="8" t="inlineStr"/>
+          <t>Partial</t>
+        </is>
+      </c>
+      <c r="F11" s="8" t="inlineStr">
+        <is>
+          <t>hermes-agent docs: persistent memory</t>
+        </is>
+      </c>
       <c r="G11" s="8" t="n">
         <v>3</v>
       </c>
@@ -14466,19 +14508,49 @@
       <c r="J12" s="8" t="inlineStr"/>
     </row>
     <row r="13">
-      <c r="A13" s="8" t="n"/>
-      <c r="B13" s="8" t="n"/>
-      <c r="C13" s="8" t="n"/>
-      <c r="D13" s="8" t="n"/>
-      <c r="E13" s="8" t="n"/>
-      <c r="F13" s="8" t="n"/>
-      <c r="G13" s="8" t="n"/>
+      <c r="A13" s="8" t="inlineStr">
+        <is>
+          <t>IM-09</t>
+        </is>
+      </c>
+      <c r="B13" s="8" t="inlineStr">
+        <is>
+          <t>MEMORY.md committed to hermes-vps</t>
+        </is>
+      </c>
+      <c r="C13" s="8" t="inlineStr">
+        <is>
+          <t>Distinct from SOUL.md (IM-01): MEMORY.md holds WHAT the agent has learned — environment facts, conventions, discovered workarounds — not who it is. Same 2,200-char cap; on overflow the agent must consolidate/remove entries before adding more (some nuance gets lost in that process). Human-prunable by hand-editing the file directly; hermes memory compress --older-than 30d also exists for session-level compression.</t>
+        </is>
+      </c>
+      <c r="D13" s="8" t="inlineStr">
+        <is>
+          <t>Hermes-VPS</t>
+        </is>
+      </c>
+      <c r="E13" s="8" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F13" s="8" t="inlineStr">
+        <is>
+          <t>hermes-agent docs: persistent memory</t>
+        </is>
+      </c>
+      <c r="G13" s="8" t="n">
+        <v>8</v>
+      </c>
       <c r="H13" s="8">
         <f>IF(E13="Done",G13,IF(E13="Partial",G13*0.5,0))</f>
         <v/>
       </c>
-      <c r="I13" s="8" t="n"/>
-      <c r="J13" s="8" t="n"/>
+      <c r="I13" s="8" t="inlineStr">
+        <is>
+          <t>Hermes Design Specialist</t>
+        </is>
+      </c>
+      <c r="J13" s="8" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="8" t="n"/>
@@ -14915,22 +14987,37 @@
       <c r="I42" s="8" t="n"/>
       <c r="J42" s="8" t="n"/>
     </row>
-    <row r="44">
-      <c r="B44" s="20" t="inlineStr">
+    <row r="43">
+      <c r="A43" s="8" t="n"/>
+      <c r="B43" s="8" t="n"/>
+      <c r="C43" s="8" t="n"/>
+      <c r="D43" s="8" t="n"/>
+      <c r="E43" s="8" t="n"/>
+      <c r="F43" s="8" t="n"/>
+      <c r="G43" s="8" t="n"/>
+      <c r="H43" s="8">
+        <f>IF(E43="Done",G43,IF(E43="Partial",G43*0.5,0))</f>
+        <v/>
+      </c>
+      <c r="I43" s="8" t="n"/>
+      <c r="J43" s="8" t="n"/>
+    </row>
+    <row r="45">
+      <c r="B45" s="20" t="inlineStr">
         <is>
           <t>TAB TOTAL (includes blank headroom rows above for future additions)</t>
         </is>
       </c>
-      <c r="G44" s="20">
-        <f>SUM(G5:G42)</f>
-        <v/>
-      </c>
-      <c r="H44" s="20">
-        <f>SUM(H5:H42)</f>
-        <v/>
-      </c>
-      <c r="I44" s="20">
-        <f>IFERROR(TEXT(H44/G44,"0%")&amp;" complete","0% complete")</f>
+      <c r="G45" s="20">
+        <f>SUM(G5:G43)</f>
+        <v/>
+      </c>
+      <c r="H45" s="20">
+        <f>SUM(H5:H43)</f>
+        <v/>
+      </c>
+      <c r="I45" s="20">
+        <f>IFERROR(TEXT(H45/G45,"0%")&amp;" complete","0% complete")</f>
         <v/>
       </c>
     </row>
@@ -14939,7 +15026,7 @@
     <mergeCell ref="A1:J1"/>
     <mergeCell ref="A2:J2"/>
   </mergeCells>
-  <conditionalFormatting sqref="E5:E42">
+  <conditionalFormatting sqref="E5:E43">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="3">
       <formula>"Done"</formula>
     </cfRule>

</xml_diff>

<commit_message>
Lock in Hindsight as the extended memory provider
IM-05 updated from researched-candidate to locked decision: Hindsight over
ByteRover, Supermemory, Mem0, Honcho, OpenViking, Holographic, RetainDB, and
Mnemosyne, based on the only independently-reproduced top benchmark
(94.6% LongMemEval) and the reflect operation matching the stated
requirement (broad scope, curated output, not raw total recall).

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Hermes_Way.xlsx
+++ b/Hermes_Way.xlsx
@@ -14339,12 +14339,12 @@
       </c>
       <c r="B9" s="8" t="inlineStr">
         <is>
-          <t>Hermes-native long-term memory (extended provider)</t>
+          <t>Extended memory provider: Hindsight — locked in</t>
         </is>
       </c>
       <c r="C9" s="8" t="inlineStr">
         <is>
-          <t>Decision/context memory currently lives in Claude Code's bootstrap catalog habit, not in Hermes itself. Researched 2026-10-04: Hermes supports pluggable providers (Hindsight, Supermemory, Mnemosyne, others). User's actual requirement: broad scope ('anything is fair game,' Hermes = main AI tool going forward) but genuinely curated, not raw total recall ('remembering everything means remembering nothing'). Hindsight's reflect operation is built for exactly this — it reasons across all stored memories with an LLM to produce a synthesized answer, not a ranked dump; its retain operation also does entity resolution so facts link to canonical people/projects instead of floating as disconnected rows. Local Docker mode keeps this on-box, no cloud dependency, and could share a database with the migrated catalog/vault (SV-15).</t>
+          <t>LOCKED 2026-10-04 after comparing all 8 official Hermes memory plugins (Hindsight, ByteRover, Supermemory, Mem0, Honcho, OpenViking, Holographic, RetainDB) plus Mnemosyne. Hindsight has the best independently-verified benchmark (94.6% LongMemEval, officially reproduced leaderboard result — ByteRover's higher LoCoMo number is vendor-self-reported, not third-party confirmed). Its reflect operation also directly matches the actual requirement: broad scope ('anything is fair game,' Hermes = main AI tool going forward) but genuinely curated ('remembering everything means remembering nothing') — reflect reasons across all stored memories to produce one synthesized answer, not a ranked dump; retain does entity resolution so facts link to canonical people/projects. Local Docker mode, own Postgres, no cloud dependency — could share a database with the migrated catalog/vault (SV-15).</t>
         </is>
       </c>
       <c r="D9" s="8" t="inlineStr">
@@ -14354,12 +14354,12 @@
       </c>
       <c r="E9" s="8" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Partial</t>
         </is>
       </c>
       <c r="F9" s="8" t="inlineStr">
         <is>
-          <t>catalog (temporary) -&gt; Hindsight (target)</t>
+          <t>hermes-memory-provider-locked-hindsight-2026-10-04</t>
         </is>
       </c>
       <c r="G9" s="8" t="n">
@@ -14376,7 +14376,7 @@
       </c>
       <c r="J9" s="8" t="inlineStr">
         <is>
-          <t>Depends on SV-15 landing first for the shared-database option</t>
+          <t>Decided, not yet deployed. Depends on SV-15 landing first for the shared-database option</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Lock in runtime, terminal backend, TTS, Vultr fallback model, and messaging
- LI-03: ik_llama.cpp over vLLM/KTransformers (native Windows build, no WSL2)
- CR-17 (new): terminal.backend=docker, directly mitigates part of HN-05/SH-02
- IA-10 (new): TTS=Edge, the free default, matches voice being a deferred non-goal
- MR-13 (new): Vultr fallback model=DeepSeek-V4-Flash, cheapest of the 8 available
- IA-05: Telegram over Signal (official Bot API vs Signal's unofficial signal-cli)
  -- replaced stale "Signal/Telegram" references throughout with Telegram

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Hermes_Way.xlsx
+++ b/Hermes_Way.xlsx
@@ -349,8 +349,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="tbl_01_Core_Runtime" displayName="tbl_01_Core_Runtime" ref="A4:J50" headerRowCount="1">
-  <autoFilter ref="A4:J50"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="tbl_01_Core_Runtime" displayName="tbl_01_Core_Runtime" ref="A4:J51" headerRowCount="1">
+  <autoFilter ref="A4:J51"/>
   <tableColumns count="10">
     <tableColumn id="1" name="ID"/>
     <tableColumn id="2" name="Feature"/>
@@ -515,8 +515,8 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="tbl_03_Model_Routing_Resilience" displayName="tbl_03_Model_Routing_Resilience" ref="A4:J46" headerRowCount="1">
-  <autoFilter ref="A4:J46"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="tbl_03_Model_Routing_Resilience" displayName="tbl_03_Model_Routing_Resilience" ref="A4:J47" headerRowCount="1">
+  <autoFilter ref="A4:J47"/>
   <tableColumns count="10">
     <tableColumn id="1" name="ID"/>
     <tableColumn id="2" name="Feature"/>
@@ -610,8 +610,8 @@
 </file>
 
 <file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="8" name="tbl_08_Interfaces_Access" displayName="tbl_08_Interfaces_Access" ref="A4:J43" headerRowCount="1">
-  <autoFilter ref="A4:J43"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="8" name="tbl_08_Interfaces_Access" displayName="tbl_08_Interfaces_Access" ref="A4:J44" headerRowCount="1">
+  <autoFilter ref="A4:J44"/>
   <tableColumns count="10">
     <tableColumn id="1" name="ID"/>
     <tableColumn id="2" name="Feature"/>
@@ -1300,7 +1300,7 @@
     <row r="55">
       <c r="A55" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">  08_Interfaces_Access          web UI, Desktop, Signal/Telegram</t>
+          <t xml:space="preserve">  08_Interfaces_Access          web UI, Desktop, Telegram</t>
         </is>
       </c>
     </row>
@@ -2538,12 +2538,12 @@
       </c>
       <c r="B7" s="8" t="inlineStr">
         <is>
-          <t>Runtime chosen</t>
+          <t>Runtime chosen: ik_llama.cpp — locked in</t>
         </is>
       </c>
       <c r="C7" s="8" t="inlineStr">
         <is>
-          <t>vLLM / ik_llama.cpp / llama.cpp (CPU expert offload) / KTransformers — none evaluated on this hardware yet.</t>
+          <t>LOCKED 2026-10-04: ik_llama.cpp over vLLM and KTransformers. vLLM has no official Windows support at all (only unofficial community forks); llama.cpp/ik_llama.cpp has real native Windows builds, no WSL2 needed. ik_llama.cpp specifically exists for this use case: offloading MoE inactive experts to system RAM on consumer hardware.</t>
         </is>
       </c>
       <c r="D7" s="8" t="inlineStr">
@@ -2553,10 +2553,14 @@
       </c>
       <c r="E7" s="8" t="inlineStr">
         <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F7" s="8" t="inlineStr"/>
+          <t>Partial</t>
+        </is>
+      </c>
+      <c r="F7" s="8" t="inlineStr">
+        <is>
+          <t>hermes-five-provider-choices-locked-2026-10-04</t>
+        </is>
+      </c>
       <c r="G7" s="8" t="n">
         <v>10</v>
       </c>
@@ -2569,7 +2573,11 @@
           <t>Model/Routing Engineer</t>
         </is>
       </c>
-      <c r="J7" s="8" t="inlineStr"/>
+      <c r="J7" s="8" t="inlineStr">
+        <is>
+          <t>Decided, not yet installed/benchmarked. Dependencies not yet researched — see D-tab follow-up</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="8" t="inlineStr">
@@ -3451,7 +3459,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J45"/>
+  <dimension ref="A1:J46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -3708,12 +3716,12 @@
       </c>
       <c r="B9" s="8" t="inlineStr">
         <is>
-          <t>Signal/Telegram channel configured</t>
+          <t>Telegram channel configured — locked in</t>
         </is>
       </c>
       <c r="C9" s="8" t="inlineStr">
         <is>
-          <t>hermes-gateway process is running; no channel wired on top of it yet. This is the interface built specifically for the GP 'looks like ordinary traffic' constraint.</t>
+          <t>LOCKED 2026-10-04: Telegram over Signal — official Bot API (reliable) vs. Signal's unofficial signal-cli integration (more brittle). hermes-gateway process is running; no channel wired on top of it yet. This is the interface built specifically for the GP 'looks like ordinary traffic' constraint.</t>
         </is>
       </c>
       <c r="D9" s="8" t="inlineStr">
@@ -3723,12 +3731,12 @@
       </c>
       <c r="E9" s="8" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Partial</t>
         </is>
       </c>
       <c r="F9" s="8" t="inlineStr">
         <is>
-          <t>hermes-gateway</t>
+          <t>hermes-five-provider-choices-locked-2026-10-04</t>
         </is>
       </c>
       <c r="G9" s="8" t="n">
@@ -3743,7 +3751,11 @@
           <t>Interface Engineer</t>
         </is>
       </c>
-      <c r="J9" s="8" t="inlineStr"/>
+      <c r="J9" s="8" t="inlineStr">
+        <is>
+          <t>Needs a Telegram Bot token via BotFather — a new vault-worthy credential, not yet created</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="8" t="inlineStr">
@@ -3885,7 +3897,7 @@
       </c>
       <c r="C13" s="8" t="inlineStr">
         <is>
-          <t>No record of who/when hit the web UI, Desktop, or future Signal channel.</t>
+          <t>No record of who/when hit the web UI, Desktop, or future Telegram channel.</t>
         </is>
       </c>
       <c r="D13" s="8" t="inlineStr">
@@ -3914,19 +3926,53 @@
       <c r="J13" s="8" t="inlineStr"/>
     </row>
     <row r="14">
-      <c r="A14" s="8" t="n"/>
-      <c r="B14" s="8" t="n"/>
-      <c r="C14" s="8" t="n"/>
-      <c r="D14" s="8" t="n"/>
-      <c r="E14" s="8" t="n"/>
-      <c r="F14" s="8" t="n"/>
-      <c r="G14" s="8" t="n"/>
+      <c r="A14" s="8" t="inlineStr">
+        <is>
+          <t>IA-10</t>
+        </is>
+      </c>
+      <c r="B14" s="8" t="inlineStr">
+        <is>
+          <t>TTS provider: Edge — locked in</t>
+        </is>
+      </c>
+      <c r="C14" s="8" t="inlineStr">
+        <is>
+          <t>LOCKED 2026-10-04: Edge TTS, the Hermes default — free, no API key, 322 voices/74 languages. Low-stakes pick since voice is already a deferred non-goal elsewhere in this workbook; not worth more setup effort than the default.</t>
+        </is>
+      </c>
+      <c r="D14" s="8" t="inlineStr">
+        <is>
+          <t>Hermes-VPS</t>
+        </is>
+      </c>
+      <c r="E14" s="8" t="inlineStr">
+        <is>
+          <t>Partial</t>
+        </is>
+      </c>
+      <c r="F14" s="8" t="inlineStr">
+        <is>
+          <t>hermes-five-provider-choices-locked-2026-10-04</t>
+        </is>
+      </c>
+      <c r="G14" s="8" t="n">
+        <v>2</v>
+      </c>
       <c r="H14" s="8">
         <f>IF(E14="Done",G14,IF(E14="Partial",G14*0.5,0))</f>
         <v/>
       </c>
-      <c r="I14" s="8" t="n"/>
-      <c r="J14" s="8" t="n"/>
+      <c r="I14" s="8" t="inlineStr">
+        <is>
+          <t>Interface Engineer</t>
+        </is>
+      </c>
+      <c r="J14" s="8" t="inlineStr">
+        <is>
+          <t>Decided, not yet confirmed configured (it may already be default-active with zero setup needed)</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="8" t="n"/>
@@ -4363,22 +4409,37 @@
       <c r="I43" s="8" t="n"/>
       <c r="J43" s="8" t="n"/>
     </row>
-    <row r="45">
-      <c r="B45" s="20" t="inlineStr">
+    <row r="44">
+      <c r="A44" s="8" t="n"/>
+      <c r="B44" s="8" t="n"/>
+      <c r="C44" s="8" t="n"/>
+      <c r="D44" s="8" t="n"/>
+      <c r="E44" s="8" t="n"/>
+      <c r="F44" s="8" t="n"/>
+      <c r="G44" s="8" t="n"/>
+      <c r="H44" s="8">
+        <f>IF(E44="Done",G44,IF(E44="Partial",G44*0.5,0))</f>
+        <v/>
+      </c>
+      <c r="I44" s="8" t="n"/>
+      <c r="J44" s="8" t="n"/>
+    </row>
+    <row r="46">
+      <c r="B46" s="20" t="inlineStr">
         <is>
           <t>TAB TOTAL (includes blank headroom rows above for future additions)</t>
         </is>
       </c>
-      <c r="G45" s="20">
-        <f>SUM(G5:G43)</f>
-        <v/>
-      </c>
-      <c r="H45" s="20">
-        <f>SUM(H5:H43)</f>
-        <v/>
-      </c>
-      <c r="I45" s="20">
-        <f>IFERROR(TEXT(H45/G45,"0%")&amp;" complete","0% complete")</f>
+      <c r="G46" s="20">
+        <f>SUM(G5:G44)</f>
+        <v/>
+      </c>
+      <c r="H46" s="20">
+        <f>SUM(H5:H44)</f>
+        <v/>
+      </c>
+      <c r="I46" s="20">
+        <f>IFERROR(TEXT(H46/G46,"0%")&amp;" complete","0% complete")</f>
         <v/>
       </c>
     </row>
@@ -4387,7 +4448,7 @@
     <mergeCell ref="A1:J1"/>
     <mergeCell ref="A2:J2"/>
   </mergeCells>
-  <conditionalFormatting sqref="E5:E43">
+  <conditionalFormatting sqref="E5:E44">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="3">
       <formula>"Done"</formula>
     </cfRule>
@@ -10948,7 +11009,7 @@
       </c>
       <c r="C5" s="8" t="inlineStr">
         <is>
-          <t>One memory, one identity, reachable identically from every interface — no split-brain between web UI / Desktop / future Signal.</t>
+          <t>One memory, one identity, reachable identically from every interface — no split-brain between web UI / Desktop / future Telegram.</t>
         </is>
       </c>
       <c r="D5" s="8" t="inlineStr">
@@ -11990,7 +12051,7 @@
       </c>
       <c r="B11" s="8" t="inlineStr">
         <is>
-          <t>Owns every door into Hermes — web UI, Desktop, Signal/Telegram — and that they all lead to the same place.</t>
+          <t>Owns every door into Hermes — web UI, Desktop, Telegram — and that they all lead to the same place.</t>
         </is>
       </c>
       <c r="C11" s="8" t="inlineStr">
@@ -12127,11 +12188,11 @@
         </is>
       </c>
       <c r="C5" s="10">
-        <f>SUM('01_Core_Runtime'!G5:G50)</f>
+        <f>SUM('01_Core_Runtime'!G5:G51)</f>
         <v/>
       </c>
       <c r="D5" s="10">
-        <f>SUM('01_Core_Runtime'!H5:H50)</f>
+        <f>SUM('01_Core_Runtime'!H5:H51)</f>
         <v/>
       </c>
       <c r="E5" s="11">
@@ -12175,11 +12236,11 @@
         </is>
       </c>
       <c r="C7" s="10">
-        <f>SUM('03_Model_Routing_Resilience'!G5:G46)</f>
+        <f>SUM('03_Model_Routing_Resilience'!G5:G47)</f>
         <v/>
       </c>
       <c r="D7" s="10">
-        <f>SUM('03_Model_Routing_Resilience'!H5:H46)</f>
+        <f>SUM('03_Model_Routing_Resilience'!H5:H47)</f>
         <v/>
       </c>
       <c r="E7" s="11">
@@ -12295,11 +12356,11 @@
         </is>
       </c>
       <c r="C12" s="10">
-        <f>SUM('08_Interfaces_Access'!G5:G43)</f>
+        <f>SUM('08_Interfaces_Access'!G5:G44)</f>
         <v/>
       </c>
       <c r="D12" s="10">
-        <f>SUM('08_Interfaces_Access'!H5:H43)</f>
+        <f>SUM('08_Interfaces_Access'!H5:H44)</f>
         <v/>
       </c>
       <c r="E12" s="11">
@@ -12687,7 +12748,7 @@
     <row r="39" ht="44" customHeight="1">
       <c r="A39" s="8" t="inlineStr">
         <is>
-          <t>G7 — Signal/Telegram wired up</t>
+          <t>G7 — Telegram wired up</t>
         </is>
       </c>
       <c r="B39" s="8" t="inlineStr">
@@ -12782,7 +12843,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J52"/>
+  <dimension ref="A1:J53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -13576,19 +13637,53 @@
       <c r="J20" s="8" t="inlineStr"/>
     </row>
     <row r="21">
-      <c r="A21" s="8" t="n"/>
-      <c r="B21" s="8" t="n"/>
-      <c r="C21" s="8" t="n"/>
-      <c r="D21" s="8" t="n"/>
-      <c r="E21" s="8" t="n"/>
-      <c r="F21" s="8" t="n"/>
-      <c r="G21" s="8" t="n"/>
+      <c r="A21" s="8" t="inlineStr">
+        <is>
+          <t>CR-17</t>
+        </is>
+      </c>
+      <c r="B21" s="8" t="inlineStr">
+        <is>
+          <t>Terminal backend: Docker — locked in</t>
+        </is>
+      </c>
+      <c r="C21" s="8" t="inlineStr">
+        <is>
+          <t>LOCKED 2026-10-04: terminal.backend=docker, not local. Directly relevant to HN-05/SH-02 (gateway shell exposure) — switching off 'local' sandboxes every command Hermes runs in a container instead of executing directly on the VPS, containing blast radius even before the allowlist fix lands. Docker's already installed on hermes-vps for Dokploy.</t>
+        </is>
+      </c>
+      <c r="D21" s="8" t="inlineStr">
+        <is>
+          <t>Hermes-VPS</t>
+        </is>
+      </c>
+      <c r="E21" s="8" t="inlineStr">
+        <is>
+          <t>Partial</t>
+        </is>
+      </c>
+      <c r="F21" s="8" t="inlineStr">
+        <is>
+          <t>hermes-five-provider-choices-locked-2026-10-04</t>
+        </is>
+      </c>
+      <c r="G21" s="8" t="n">
+        <v>8</v>
+      </c>
       <c r="H21" s="8">
         <f>IF(E21="Done",G21,IF(E21="Partial",G21*0.5,0))</f>
         <v/>
       </c>
-      <c r="I21" s="8" t="n"/>
-      <c r="J21" s="8" t="n"/>
+      <c r="I21" s="8" t="inlineStr">
+        <is>
+          <t>Security Reviewer</t>
+        </is>
+      </c>
+      <c r="J21" s="8" t="inlineStr">
+        <is>
+          <t>Decided, not yet applied to config.yaml</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="8" t="n"/>
@@ -14025,22 +14120,37 @@
       <c r="I50" s="8" t="n"/>
       <c r="J50" s="8" t="n"/>
     </row>
-    <row r="52">
-      <c r="B52" s="20" t="inlineStr">
+    <row r="51">
+      <c r="A51" s="8" t="n"/>
+      <c r="B51" s="8" t="n"/>
+      <c r="C51" s="8" t="n"/>
+      <c r="D51" s="8" t="n"/>
+      <c r="E51" s="8" t="n"/>
+      <c r="F51" s="8" t="n"/>
+      <c r="G51" s="8" t="n"/>
+      <c r="H51" s="8">
+        <f>IF(E51="Done",G51,IF(E51="Partial",G51*0.5,0))</f>
+        <v/>
+      </c>
+      <c r="I51" s="8" t="n"/>
+      <c r="J51" s="8" t="n"/>
+    </row>
+    <row r="53">
+      <c r="B53" s="20" t="inlineStr">
         <is>
           <t>TAB TOTAL (includes blank headroom rows above for future additions)</t>
         </is>
       </c>
-      <c r="G52" s="20">
-        <f>SUM(G5:G50)</f>
-        <v/>
-      </c>
-      <c r="H52" s="20">
-        <f>SUM(H5:H50)</f>
-        <v/>
-      </c>
-      <c r="I52" s="20">
-        <f>IFERROR(TEXT(H52/G52,"0%")&amp;" complete","0% complete")</f>
+      <c r="G53" s="20">
+        <f>SUM(G5:G51)</f>
+        <v/>
+      </c>
+      <c r="H53" s="20">
+        <f>SUM(H5:H51)</f>
+        <v/>
+      </c>
+      <c r="I53" s="20">
+        <f>IFERROR(TEXT(H53/G53,"0%")&amp;" complete","0% complete")</f>
         <v/>
       </c>
     </row>
@@ -14049,7 +14159,7 @@
     <mergeCell ref="A1:J1"/>
     <mergeCell ref="A2:J2"/>
   </mergeCells>
-  <conditionalFormatting sqref="E5:E50">
+  <conditionalFormatting sqref="E5:E51">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="3">
       <formula>"Done"</formula>
     </cfRule>
@@ -14303,7 +14413,7 @@
       </c>
       <c r="C8" s="8" t="inlineStr">
         <is>
-          <t>Web UI, Hermes Desktop, and (eventually) Signal all resume the same memory, not three separate Hermeses.</t>
+          <t>Web UI, Hermes Desktop, and (eventually) Telegram all resume the same memory, not three separate Hermeses.</t>
         </is>
       </c>
       <c r="D8" s="8" t="inlineStr">
@@ -15051,7 +15161,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J48"/>
+  <dimension ref="A1:J49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -15565,17 +15675,17 @@
     <row r="15">
       <c r="A15" s="8" t="inlineStr">
         <is>
-          <t>MR-11</t>
+          <t>MR-13</t>
         </is>
       </c>
       <c r="B15" s="8" t="inlineStr">
         <is>
-          <t>Retry/backoff policy documented</t>
+          <t>Vultr Serverless Inference fallback model: DeepSeek-V4-Flash — locked in</t>
         </is>
       </c>
       <c r="C15" s="8" t="inlineStr">
         <is>
-          <t>Transient local error vs. hard failure should not be handled identically.</t>
+          <t>LOCKED 2026-10-04: cheapest of the 8 pre-configured models ($0.30/M input, $1.00/M output), fast, general-purpose — right fit for a middle tier meant to be cheap overflow capacity, not a second Codex. Already pre-configured/credentialed on hermes-vps; just needs an explicit fallback_providers entry in config.yaml.</t>
         </is>
       </c>
       <c r="D15" s="8" t="inlineStr">
@@ -15585,12 +15695,16 @@
       </c>
       <c r="E15" s="8" t="inlineStr">
         <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F15" s="8" t="inlineStr"/>
+          <t>Partial</t>
+        </is>
+      </c>
+      <c r="F15" s="8" t="inlineStr">
+        <is>
+          <t>hermes-five-provider-choices-locked-2026-10-04</t>
+        </is>
+      </c>
       <c r="G15" s="8" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="H15" s="8">
         <f>IF(E15="Done",G15,IF(E15="Partial",G15*0.5,0))</f>
@@ -15601,22 +15715,26 @@
           <t>Model/Routing Engineer</t>
         </is>
       </c>
-      <c r="J15" s="8" t="inlineStr"/>
+      <c r="J15" s="8" t="inlineStr">
+        <is>
+          <t>No three-tier routing logic exists yet (judge only knows local-vs-Codex) — this model is configured but not yet reachable by the router</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="8" t="inlineStr">
         <is>
-          <t>MR-12</t>
+          <t>MR-11</t>
         </is>
       </c>
       <c r="B16" s="8" t="inlineStr">
         <is>
-          <t>Routing-decision log retention policy</t>
+          <t>Retry/backoff policy documented</t>
         </is>
       </c>
       <c r="C16" s="8" t="inlineStr">
         <is>
-          <t>complexity_router.log exists and records every verdict, but nothing rotates or retains it deliberately.</t>
+          <t>Transient local error vs. hard failure should not be handled identically.</t>
         </is>
       </c>
       <c r="D16" s="8" t="inlineStr">
@@ -15626,14 +15744,10 @@
       </c>
       <c r="E16" s="8" t="inlineStr">
         <is>
-          <t>Partial</t>
-        </is>
-      </c>
-      <c r="F16" s="8" t="inlineStr">
-        <is>
-          <t>/home/hermes/.hermes/logs/complexity_router.log</t>
-        </is>
-      </c>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F16" s="8" t="inlineStr"/>
       <c r="G16" s="8" t="n">
         <v>3</v>
       </c>
@@ -15643,25 +15757,55 @@
       </c>
       <c r="I16" s="8" t="inlineStr">
         <is>
-          <t>Observability</t>
+          <t>Model/Routing Engineer</t>
         </is>
       </c>
       <c r="J16" s="8" t="inlineStr"/>
     </row>
     <row r="17">
-      <c r="A17" s="8" t="n"/>
-      <c r="B17" s="8" t="n"/>
-      <c r="C17" s="8" t="n"/>
-      <c r="D17" s="8" t="n"/>
-      <c r="E17" s="8" t="n"/>
-      <c r="F17" s="8" t="n"/>
-      <c r="G17" s="8" t="n"/>
+      <c r="A17" s="8" t="inlineStr">
+        <is>
+          <t>MR-12</t>
+        </is>
+      </c>
+      <c r="B17" s="8" t="inlineStr">
+        <is>
+          <t>Routing-decision log retention policy</t>
+        </is>
+      </c>
+      <c r="C17" s="8" t="inlineStr">
+        <is>
+          <t>complexity_router.log exists and records every verdict, but nothing rotates or retains it deliberately.</t>
+        </is>
+      </c>
+      <c r="D17" s="8" t="inlineStr">
+        <is>
+          <t>Hermes-VPS</t>
+        </is>
+      </c>
+      <c r="E17" s="8" t="inlineStr">
+        <is>
+          <t>Partial</t>
+        </is>
+      </c>
+      <c r="F17" s="8" t="inlineStr">
+        <is>
+          <t>/home/hermes/.hermes/logs/complexity_router.log</t>
+        </is>
+      </c>
+      <c r="G17" s="8" t="n">
+        <v>3</v>
+      </c>
       <c r="H17" s="8">
         <f>IF(E17="Done",G17,IF(E17="Partial",G17*0.5,0))</f>
         <v/>
       </c>
-      <c r="I17" s="8" t="n"/>
-      <c r="J17" s="8" t="n"/>
+      <c r="I17" s="8" t="inlineStr">
+        <is>
+          <t>Observability</t>
+        </is>
+      </c>
+      <c r="J17" s="8" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="8" t="n"/>
@@ -16098,22 +16242,37 @@
       <c r="I46" s="8" t="n"/>
       <c r="J46" s="8" t="n"/>
     </row>
-    <row r="48">
-      <c r="B48" s="20" t="inlineStr">
+    <row r="47">
+      <c r="A47" s="8" t="n"/>
+      <c r="B47" s="8" t="n"/>
+      <c r="C47" s="8" t="n"/>
+      <c r="D47" s="8" t="n"/>
+      <c r="E47" s="8" t="n"/>
+      <c r="F47" s="8" t="n"/>
+      <c r="G47" s="8" t="n"/>
+      <c r="H47" s="8">
+        <f>IF(E47="Done",G47,IF(E47="Partial",G47*0.5,0))</f>
+        <v/>
+      </c>
+      <c r="I47" s="8" t="n"/>
+      <c r="J47" s="8" t="n"/>
+    </row>
+    <row r="49">
+      <c r="B49" s="20" t="inlineStr">
         <is>
           <t>TAB TOTAL (includes blank headroom rows above for future additions)</t>
         </is>
       </c>
-      <c r="G48" s="20">
-        <f>SUM(G5:G46)</f>
-        <v/>
-      </c>
-      <c r="H48" s="20">
-        <f>SUM(H5:H46)</f>
-        <v/>
-      </c>
-      <c r="I48" s="20">
-        <f>IFERROR(TEXT(H48/G48,"0%")&amp;" complete","0% complete")</f>
+      <c r="G49" s="20">
+        <f>SUM(G5:G47)</f>
+        <v/>
+      </c>
+      <c r="H49" s="20">
+        <f>SUM(H5:H47)</f>
+        <v/>
+      </c>
+      <c r="I49" s="20">
+        <f>IFERROR(TEXT(H49/G49,"0%")&amp;" complete","0% complete")</f>
         <v/>
       </c>
     </row>
@@ -16122,7 +16281,7 @@
     <mergeCell ref="A1:J1"/>
     <mergeCell ref="A2:J2"/>
   </mergeCells>
-  <conditionalFormatting sqref="E5:E46">
+  <conditionalFormatting sqref="E5:E47">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="3">
       <formula>"Done"</formula>
     </cfRule>

</xml_diff>

<commit_message>
Add D2_Providers_And_Deps: 4 more unchosen providers, real dependencies for the 5 locked
New provider categories found with zero decision yet: STT (separate from TTS),
image generation (FAL.ai, no free/local option unlike everything else chosen
so far), browser automation backend, and embedding provider (resolves the
catalog's long-idle search_similar RPC from the original 2026-09-25 plan).

Also got concrete dependencies for the five locked-in providers: ik_llama.cpp's
Windows build requirements (CUDA 12.6, VS Build Tools 2022, cmake), Docker
terminal backend (likely just a config change, already installed), Telegram's
BotFather token flow (a new vault-worthy credential), Vultr fallback model
(trivial, already credentialed), and Edge TTS (may already be active).

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Hermes_Way.xlsx
+++ b/Hermes_Way.xlsx
@@ -27,6 +27,7 @@
     <sheet name="14_Claude_Code_Parity" sheetId="18" state="visible" r:id="rId18"/>
     <sheet name="15_Productivity_And_Acceptance" sheetId="19" state="visible" r:id="rId19"/>
     <sheet name="D1_Vultr_Services_Audit" sheetId="20" state="visible" r:id="rId20"/>
+    <sheet name="D2_Providers_And_Deps" sheetId="21" state="visible" r:id="rId21"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -495,6 +496,20 @@
 </table>
 </file>
 
+<file path=xl/tables/table17.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="17" name="tbl_D2_Providers_And_Deps" displayName="tbl_D2_Providers_And_Deps" ref="A4:E13" headerRowCount="1">
+  <autoFilter ref="A4:E13"/>
+  <tableColumns count="5">
+    <tableColumn id="1" name="Topic"/>
+    <tableColumn id="2" name="What it is"/>
+    <tableColumn id="3" name="Options found"/>
+    <tableColumn id="4" name="Recommendation / dependency detail"/>
+    <tableColumn id="5" name="Status"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleLight11" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="tbl_02_Identity_Memory" displayName="tbl_02_Identity_Memory" ref="A4:J43" headerRowCount="1">
   <autoFilter ref="A4:J43"/>
@@ -937,7 +952,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A72"/>
+  <dimension ref="A1:A74"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -1378,38 +1393,52 @@
       </c>
     </row>
     <row r="67">
-      <c r="A67" s="3" t="inlineStr"/>
+      <c r="A67" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  D2_Providers_And_Deps  STT/image-gen/browser/embedding providers still unchosen, plus real</t>
+        </is>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Found 2026-10-04: Nous's own framing is 'Five Pillars' -- Memory, Skills, Soul, Crons, Self-</t>
+          <t xml:space="preserve">                                 install dependencies behind the 5 providers already locked in</t>
         </is>
       </c>
     </row>
     <row r="69">
-      <c r="A69" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Improvement. Memory+Soul covered in 02_Identity_Memory. Skills queued next. Crons (built-in</t>
-        </is>
-      </c>
+      <c r="A69" s="3" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">  scheduler: hermes cron list/remove/run) and Self-Improvement (the learn-from-work loop) are</t>
+          <t xml:space="preserve">  Found 2026-10-04: Nous's own framing is 'Five Pillars' -- Memory, Skills, Soul, Crons, Self-</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">  real pillars with zero coverage anywhere in this workbook yet -- not yet researched, flagging</t>
+          <t xml:space="preserve">  Improvement. Memory+Soul covered in 02_Identity_Memory. Skills queued next. Crons (built-in</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  scheduler: hermes cron list/remove/run) and Self-Improvement (the learn-from-work loop) are</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  real pillars with zero coverage anywhere in this workbook yet -- not yet researched, flagging</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">  so they don't get forgotten once Skills is done.</t>
         </is>
@@ -2575,7 +2604,7 @@
       </c>
       <c r="J7" s="8" t="inlineStr">
         <is>
-          <t>Decided, not yet installed/benchmarked. Dependencies not yet researched — see D-tab follow-up</t>
+          <t>Decided, not yet installed/benchmarked. Build dependencies found — see D2_Providers_And_Deps</t>
         </is>
       </c>
     </row>
@@ -11844,6 +11873,319 @@
       <c r="E18" s="8" t="inlineStr">
         <is>
           <t>Not applicable</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A2:E2"/>
+    <mergeCell ref="A1:E1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <tableParts count="1">
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="008A5A2E"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E13"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="34" customWidth="1" min="2" max="2"/>
+    <col width="46" customWidth="1" min="3" max="3"/>
+    <col width="50" customWidth="1" min="4" max="4"/>
+    <col width="20" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="22" customHeight="1">
+      <c r="A1" s="6" t="inlineStr">
+        <is>
+          <t>Discovery — Providers Still Unchosen, and Dependencies of What's Locked</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="16" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Researched 2026-10-04. Two things in one tab: (1) provider categories found that have zero decision yet, (2) the real install/setup dependencies behind the five providers already locked in. Reference material — not a tracked backlog.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="7" t="inlineStr">
+        <is>
+          <t>Topic</t>
+        </is>
+      </c>
+      <c r="B4" s="7" t="inlineStr">
+        <is>
+          <t>What it is</t>
+        </is>
+      </c>
+      <c r="C4" s="7" t="inlineStr">
+        <is>
+          <t>Options found</t>
+        </is>
+      </c>
+      <c r="D4" s="7" t="inlineStr">
+        <is>
+          <t>Recommendation / dependency detail</t>
+        </is>
+      </c>
+      <c r="E4" s="7" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="8" t="inlineStr">
+        <is>
+          <t>STT (speech-to-text)</t>
+        </is>
+      </c>
+      <c r="B5" s="8" t="inlineStr">
+        <is>
+          <t>Separate from TTS — converts your voice input to text. Not yet chosen.</t>
+        </is>
+      </c>
+      <c r="C5" s="8" t="inlineStr">
+        <is>
+          <t>local/faster-whisper (free, on-box), groq (fast cloud), openai, mistral, xai, elevenlabs, telnyx, deepinfra</t>
+        </is>
+      </c>
+      <c r="D5" s="8" t="inlineStr">
+        <is>
+          <t>Recommend local/faster-whisper — free, matches every other 'self-hosted preferred' choice made this session, no new credential needed.</t>
+        </is>
+      </c>
+      <c r="E5" s="8" t="inlineStr">
+        <is>
+          <t>Not chosen — not yet asked about</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="8" t="inlineStr">
+        <is>
+          <t>Image generation</t>
+        </is>
+      </c>
+      <c r="B6" s="8" t="inlineStr">
+        <is>
+          <t>Routed through FAL.ai regardless of which model — not self-hostable.</t>
+        </is>
+      </c>
+      <c r="C6" s="8" t="inlineStr">
+        <is>
+          <t>FLUX 2 Klein/Pro, GPT-Image 1.5/2, Nano Banana Pro, Ideogram V3, Recraft V4 Pro, Qwen, Z-Image Turbo, Krea V2</t>
+        </is>
+      </c>
+      <c r="D6" s="8" t="inlineStr">
+        <is>
+          <t>No free/local option exists for this one, unlike everything else — only relevant if image generation is actually wanted. Needs its own cost conversation if so.</t>
+        </is>
+      </c>
+      <c r="E6" s="8" t="inlineStr">
+        <is>
+          <t>Not chosen — not yet asked about</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="8" t="inlineStr">
+        <is>
+          <t>Browser automation backend</t>
+        </is>
+      </c>
+      <c r="B7" s="8" t="inlineStr">
+        <is>
+          <t>What drives Hermes's browser-use tool capability (TM-07).</t>
+        </is>
+      </c>
+      <c r="C7" s="8" t="inlineStr">
+        <is>
+          <t>Browserbase (cloud), Browser Use (cloud), local Chrome/Brave/Chromium/Edge via CDP, Camofox (local, anti-detection)</t>
+        </is>
+      </c>
+      <c r="D7" s="8" t="inlineStr">
+        <is>
+          <t>Local CDP (e.g. local Chrome) is the free/self-hosted-matching option. Cloud options exist if local browsing proves unreliable.</t>
+        </is>
+      </c>
+      <c r="E7" s="8" t="inlineStr">
+        <is>
+          <t>Not chosen — not yet asked about</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="8" t="inlineStr">
+        <is>
+          <t>Embedding provider</t>
+        </is>
+      </c>
+      <c r="B8" s="8" t="inlineStr">
+        <is>
+          <t>Powers RAG/semantic search — resolves the catalog's long-idle search_similar RPC (mentioned since the original 2026-09-25 local-model plan, nomic-embed-text).</t>
+        </is>
+      </c>
+      <c r="C8" s="8" t="inlineStr">
+        <is>
+          <t>local/fastembed (e.g. all-MiniLM-L6-v2, free), openai, ollama</t>
+        </is>
+      </c>
+      <c r="D8" s="8" t="inlineStr">
+        <is>
+          <t>Recommend local/fastembed — same reasoning as STT. This is also what would let Hindsight (IM-05) or the catalog do real semantic recall instead of exact-match search.</t>
+        </is>
+      </c>
+      <c r="E8" s="8" t="inlineStr">
+        <is>
+          <t>Not chosen — not yet asked about</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="8" t="inlineStr">
+        <is>
+          <t>DEPENDENCY: ik_llama.cpp (LI-03) on Windows</t>
+        </is>
+      </c>
+      <c r="B9" s="8" t="inlineStr">
+        <is>
+          <t>Build requirements for the locked-in runtime.</t>
+        </is>
+      </c>
+      <c r="C9" s="8" t="inlineStr">
+        <is>
+          <t>cmake, C++17 compiler, CUDA 12.6 Toolkit, Visual Studio Build Tools 2022</t>
+        </is>
+      </c>
+      <c r="D9" s="8" t="inlineStr">
+        <is>
+          <t>Env vars needed: VS_DIR, LLVM_DIR, CUDA_DIR (pointing at the CUDA 12.6 install path). Official build docs: github.com/ikawrakow/ik_llama.cpp/blob/main/docs/build.md</t>
+        </is>
+      </c>
+      <c r="E9" s="8" t="inlineStr">
+        <is>
+          <t>Known, not yet done</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="8" t="inlineStr">
+        <is>
+          <t>DEPENDENCY: Docker terminal backend (CR-17)</t>
+        </is>
+      </c>
+      <c r="B10" s="8" t="inlineStr">
+        <is>
+          <t>What the locked-in terminal backend needs.</t>
+        </is>
+      </c>
+      <c r="C10" s="8" t="inlineStr">
+        <is>
+          <t>Docker — already installed on hermes-vps for Dokploy</t>
+        </is>
+      </c>
+      <c r="D10" s="8" t="inlineStr">
+        <is>
+          <t>Likely just a config.yaml change (terminal.backend: docker) plus picking a base image; no new install expected.</t>
+        </is>
+      </c>
+      <c r="E10" s="8" t="inlineStr">
+        <is>
+          <t>Likely low-effort, unconfirmed</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="8" t="inlineStr">
+        <is>
+          <t>DEPENDENCY: Telegram gateway (IA-05)</t>
+        </is>
+      </c>
+      <c r="B11" s="8" t="inlineStr">
+        <is>
+          <t>What the locked-in messaging channel needs.</t>
+        </is>
+      </c>
+      <c r="C11" s="8" t="inlineStr">
+        <is>
+          <t>A BotFather-issued bot token; your own numeric Telegram user ID</t>
+        </is>
+      </c>
+      <c r="D11" s="8" t="inlineStr">
+        <is>
+          <t>5 steps: message @BotFather, /newbot, name it, copy the token (format 123456789:ABC...), get your user ID from @userinfobot, run hermes gateway setup, paste both, start the gateway. Token is a real credential — vault it, don't leave it in config.yaml plaintext.</t>
+        </is>
+      </c>
+      <c r="E11" s="8" t="inlineStr">
+        <is>
+          <t>Known, not yet done — new vault-worthy secret</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="8" t="inlineStr">
+        <is>
+          <t>DEPENDENCY: Vultr fallback model (MR-13)</t>
+        </is>
+      </c>
+      <c r="B12" s="8" t="inlineStr">
+        <is>
+          <t>What DeepSeek-V4-Flash needs beyond what exists.</t>
+        </is>
+      </c>
+      <c r="C12" s="8" t="inlineStr">
+        <is>
+          <t>Already pre-configured/credentialed on hermes-vps</t>
+        </is>
+      </c>
+      <c r="D12" s="8" t="inlineStr">
+        <is>
+          <t>Just needs an explicit fallback_providers entry in config.yaml — no new install or credential.</t>
+        </is>
+      </c>
+      <c r="E12" s="8" t="inlineStr">
+        <is>
+          <t>Trivial, not yet done</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="8" t="inlineStr">
+        <is>
+          <t>DEPENDENCY: Edge TTS (IA-10)</t>
+        </is>
+      </c>
+      <c r="B13" s="8" t="inlineStr">
+        <is>
+          <t>What the locked-in TTS default needs.</t>
+        </is>
+      </c>
+      <c r="C13" s="8" t="inlineStr">
+        <is>
+          <t>None — it's the Hermes default</t>
+        </is>
+      </c>
+      <c r="D13" s="8" t="inlineStr">
+        <is>
+          <t>May already be active with zero configuration. Worth a quick hermes config show to confirm rather than assuming.</t>
+        </is>
+      </c>
+      <c r="E13" s="8" t="inlineStr">
+        <is>
+          <t>Likely already satisfied, unconfirmed</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Lock in Obscura for browser automation
TM-14 (new): Obscura over local Chrome/Camofox (RAM-prohibitive on a 4GB VPS)
and cloud options (paid). Flagged honestly as an unofficial community plugin
-- NousResearch closed the native-support request as not planned -- risk
accepted knowingly rather than glossed over.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Hermes_Way.xlsx
+++ b/Hermes_Way.xlsx
@@ -549,8 +549,8 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="tbl_04_Tool_MCP_Layer" displayName="tbl_04_Tool_MCP_Layer" ref="A4:J47" headerRowCount="1">
-  <autoFilter ref="A4:J47"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="tbl_04_Tool_MCP_Layer" displayName="tbl_04_Tool_MCP_Layer" ref="A4:J48" headerRowCount="1">
+  <autoFilter ref="A4:J48"/>
   <tableColumns count="10">
     <tableColumn id="1" name="ID"/>
     <tableColumn id="2" name="Feature"/>
@@ -12602,11 +12602,11 @@
         </is>
       </c>
       <c r="C8" s="10">
-        <f>SUM('04_Tool_MCP_Layer'!G5:G47)</f>
+        <f>SUM('04_Tool_MCP_Layer'!G5:G48)</f>
         <v/>
       </c>
       <c r="D8" s="10">
-        <f>SUM('04_Tool_MCP_Layer'!H5:H47)</f>
+        <f>SUM('04_Tool_MCP_Layer'!H5:H48)</f>
         <v/>
       </c>
       <c r="E8" s="11">
@@ -16648,7 +16648,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J49"/>
+  <dimension ref="A1:J50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -17295,19 +17295,53 @@
       <c r="J17" s="8" t="inlineStr"/>
     </row>
     <row r="18">
-      <c r="A18" s="8" t="n"/>
-      <c r="B18" s="8" t="n"/>
-      <c r="C18" s="8" t="n"/>
-      <c r="D18" s="8" t="n"/>
-      <c r="E18" s="8" t="n"/>
-      <c r="F18" s="8" t="n"/>
-      <c r="G18" s="8" t="n"/>
+      <c r="A18" s="8" t="inlineStr">
+        <is>
+          <t>TM-14</t>
+        </is>
+      </c>
+      <c r="B18" s="8" t="inlineStr">
+        <is>
+          <t>Browser automation: Obscura — locked in</t>
+        </is>
+      </c>
+      <c r="C18" s="8" t="inlineStr">
+        <is>
+          <t>LOCKED 2026-10-04: Obscura (Rust headless browser, ~30MB/instance) over local Chrome/Camofox (200-400MB+/instance — too heavy for a 4GB VPS already running several services) and cloud options (Browserbase/Browser Use, paid). Known risk, stated plainly: NOT officially supported by hermes-agent core — the integration request was closed as not planned. Only available via the community plugin hermes-plugin-obscura.</t>
+        </is>
+      </c>
+      <c r="D18" s="8" t="inlineStr">
+        <is>
+          <t>Hermes-VPS</t>
+        </is>
+      </c>
+      <c r="E18" s="8" t="inlineStr">
+        <is>
+          <t>Partial</t>
+        </is>
+      </c>
+      <c r="F18" s="8" t="inlineStr">
+        <is>
+          <t>hermes-browser-automation-obscura-2026-10-04</t>
+        </is>
+      </c>
+      <c r="G18" s="8" t="n">
+        <v>5</v>
+      </c>
       <c r="H18" s="8">
         <f>IF(E18="Done",G18,IF(E18="Partial",G18*0.5,0))</f>
         <v/>
       </c>
-      <c r="I18" s="8" t="n"/>
-      <c r="J18" s="8" t="n"/>
+      <c r="I18" s="8" t="inlineStr">
+        <is>
+          <t>Hermes Design Specialist</t>
+        </is>
+      </c>
+      <c r="J18" s="8" t="inlineStr">
+        <is>
+          <t>Install: hermes plugins install SGavrl/hermes-plugin-obscura --enable. Unofficial-plugin risk accepted knowingly, not overlooked</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="8" t="n"/>
@@ -17744,22 +17778,37 @@
       <c r="I47" s="8" t="n"/>
       <c r="J47" s="8" t="n"/>
     </row>
-    <row r="49">
-      <c r="B49" s="20" t="inlineStr">
+    <row r="48">
+      <c r="A48" s="8" t="n"/>
+      <c r="B48" s="8" t="n"/>
+      <c r="C48" s="8" t="n"/>
+      <c r="D48" s="8" t="n"/>
+      <c r="E48" s="8" t="n"/>
+      <c r="F48" s="8" t="n"/>
+      <c r="G48" s="8" t="n"/>
+      <c r="H48" s="8">
+        <f>IF(E48="Done",G48,IF(E48="Partial",G48*0.5,0))</f>
+        <v/>
+      </c>
+      <c r="I48" s="8" t="n"/>
+      <c r="J48" s="8" t="n"/>
+    </row>
+    <row r="50">
+      <c r="B50" s="20" t="inlineStr">
         <is>
           <t>TAB TOTAL (includes blank headroom rows above for future additions)</t>
         </is>
       </c>
-      <c r="G49" s="20">
-        <f>SUM(G5:G47)</f>
-        <v/>
-      </c>
-      <c r="H49" s="20">
-        <f>SUM(H5:H47)</f>
-        <v/>
-      </c>
-      <c r="I49" s="20">
-        <f>IFERROR(TEXT(H49/G49,"0%")&amp;" complete","0% complete")</f>
+      <c r="G50" s="20">
+        <f>SUM(G5:G48)</f>
+        <v/>
+      </c>
+      <c r="H50" s="20">
+        <f>SUM(H5:H48)</f>
+        <v/>
+      </c>
+      <c r="I50" s="20">
+        <f>IFERROR(TEXT(H50/G50,"0%")&amp;" complete","0% complete")</f>
         <v/>
       </c>
     </row>
@@ -17768,7 +17817,7 @@
     <mergeCell ref="A1:J1"/>
     <mergeCell ref="A2:J2"/>
   </mergeCells>
-  <conditionalFormatting sqref="E5:E47">
+  <conditionalFormatting sqref="E5:E48">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="3">
       <formula>"Done"</formula>
     </cfRule>

</xml_diff>

<commit_message>
Research Skills pillar: D3_Skills_System tab, catalog entity
SKILL.md format, storage layout, bundled (87) vs optional (79)
catalogs, self-authored skill creation, and hub/project security
scanning, researched against hermes-agent's official docs. No skill
categories installed yet -- still discovery phase. Crons and
Self-Improvement remain unresearched.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Hermes_Way.xlsx
+++ b/Hermes_Way.xlsx
@@ -28,6 +28,7 @@
     <sheet name="15_Productivity_And_Acceptance" sheetId="19" state="visible" r:id="rId19"/>
     <sheet name="D1_Vultr_Services_Audit" sheetId="20" state="visible" r:id="rId20"/>
     <sheet name="D2_Providers_And_Deps" sheetId="21" state="visible" r:id="rId21"/>
+    <sheet name="D3_Skills_System" sheetId="22" state="visible" r:id="rId22"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -952,7 +953,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A74"/>
+  <dimension ref="A1:A75"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -1407,40 +1408,47 @@
       </c>
     </row>
     <row r="69">
-      <c r="A69" s="3" t="inlineStr"/>
+      <c r="A69" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  D3_Skills_System             how the Skills pillar actually works (SKILL.md, bundled/optional, self-authoring)</t>
+        </is>
+      </c>
     </row>
     <row r="70">
-      <c r="A70" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Found 2026-10-04: Nous's own framing is 'Five Pillars' -- Memory, Skills, Soul, Crons, Self-</t>
-        </is>
-      </c>
+      <c r="A70" s="3" t="inlineStr"/>
     </row>
     <row r="71">
       <c r="A71" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Improvement. Memory+Soul covered in 02_Identity_Memory. Skills queued next. Crons (built-in</t>
+          <t xml:space="preserve">  Found 2026-10-04: Nous's own framing is 'Five Pillars' -- Memory, Skills, Soul, Crons, Self-</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">  scheduler: hermes cron list/remove/run) and Self-Improvement (the learn-from-work loop) are</t>
+          <t xml:space="preserve">  Improvement. Memory+Soul covered in 02_Identity_Memory. Skills researched 2026-10-04 (see</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">  real pillars with zero coverage anywhere in this workbook yet -- not yet researched, flagging</t>
+          <t xml:space="preserve">  D3_Skills_System) -- SKILL.md format, bundled/optional catalogs, self-authored creation,</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">  so they don't get forgotten once Skills is done.</t>
+          <t xml:space="preserve">  security scanning all covered; no categories installed yet, still discovery. Crons and Self-</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Improvement remain real pillars with zero coverage anywhere in this workbook -- not yet researched.</t>
         </is>
       </c>
     </row>
@@ -12201,6 +12209,316 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="008A5A2E"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E13"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="36" customWidth="1" min="2" max="2"/>
+    <col width="50" customWidth="1" min="3" max="3"/>
+    <col width="54" customWidth="1" min="4" max="4"/>
+    <col width="20" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="22" customHeight="1">
+      <c r="A1" s="6" t="inlineStr">
+        <is>
+          <t>Discovery — Skills System (Five Pillars: Skills)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="16" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Researched 2026-10-04. How hermes-agent's Skills pillar actually works: what a skill is, how it's stored/loaded, bundled vs optional, self-authored creation, security scanning. Reference material — not a tracked backlog. Sources: hermes-agent.nousresearch.com/docs (user-guide/features/skills, guides/work-with-skills, reference/skills-catalog, reference/optional-skills-catalog).</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="7" t="inlineStr">
+        <is>
+          <t>Topic</t>
+        </is>
+      </c>
+      <c r="B4" s="7" t="inlineStr">
+        <is>
+          <t>What it is</t>
+        </is>
+      </c>
+      <c r="C4" s="7" t="inlineStr">
+        <is>
+          <t>Options found</t>
+        </is>
+      </c>
+      <c r="D4" s="7" t="inlineStr">
+        <is>
+          <t>Recommendation / dependency detail</t>
+        </is>
+      </c>
+      <c r="E4" s="7" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="8" t="inlineStr">
+        <is>
+          <t>What a skill is</t>
+        </is>
+      </c>
+      <c r="B5" s="8" t="inlineStr">
+        <is>
+          <t>An on-demand knowledge document the agent loads when needed — procedural memory for recurring tasks, not a one-off prompt.</t>
+        </is>
+      </c>
+      <c r="C5" s="8" t="inlineStr">
+        <is>
+          <t>SKILL.md with YAML frontmatter (name, description, version, metadata.hermes: tags/category/platforms/requires_toolsets/config) + body sections (When to Use, Procedure, Pitfalls, Verification). Compatible with the open agentskills.io standard.</t>
+        </is>
+      </c>
+      <c r="D5" s="8" t="inlineStr">
+        <is>
+          <t>Distinct from the Tool/MCP layer (TM-07's Tool Gateway = built-in capabilities like web search/TTS/browser automation). Skills are learned procedures layered on top of whatever tools exist — don't conflate the two rows.</t>
+        </is>
+      </c>
+      <c r="E5" s="8" t="inlineStr">
+        <is>
+          <t>Understood, not yet used</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="8" t="inlineStr">
+        <is>
+          <t>Storage &amp; directory structure</t>
+        </is>
+      </c>
+      <c r="B6" s="8" t="inlineStr">
+        <is>
+          <t>Where skills physically live on hermes-vps.</t>
+        </is>
+      </c>
+      <c r="C6" s="8" t="inlineStr">
+        <is>
+          <t>~/.hermes/skills/&lt;category&gt;/&lt;skill-name&gt;/ containing SKILL.md (required) plus optional references/, templates/, scripts/, examples/, assets/ subfolders.</t>
+        </is>
+      </c>
+      <c r="D6" s="8" t="inlineStr">
+        <is>
+          <t>Primary source of truth is the filesystem, not a database — matches the 'everything on the VPS, self-sufficient' architecture rule already set for this project.</t>
+        </is>
+      </c>
+      <c r="E6" s="8" t="inlineStr">
+        <is>
+          <t>Understood, not yet used</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="8" t="inlineStr">
+        <is>
+          <t>Discovery &amp; invocation</t>
+        </is>
+      </c>
+      <c r="B7" s="8" t="inlineStr">
+        <is>
+          <t>How the agent finds and loads a skill without burning context on all of them upfront.</t>
+        </is>
+      </c>
+      <c r="C7" s="8" t="inlineStr">
+        <is>
+          <t>3-level progressive disclosure: skills_list() (~3k tokens, metadata only) -&gt; skill_view(name) (full SKILL.md) -&gt; skill_view(name, path) (one reference file). Invoked via /skill-name slash commands (stackable: /skill1 /skill2 instruction), or picked up from natural conversation.</t>
+        </is>
+      </c>
+      <c r="D7" s="8" t="inlineStr">
+        <is>
+          <t>Token-cheap by design — matches the economic-router priority already set for this project (LLM-as-judge router logged 2026-10-03).</t>
+        </is>
+      </c>
+      <c r="E7" s="8" t="inlineStr">
+        <is>
+          <t>Understood, not yet used</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="8" t="inlineStr">
+        <is>
+          <t>Bundled vs optional skills</t>
+        </is>
+      </c>
+      <c r="B8" s="8" t="inlineStr">
+        <is>
+          <t>Two tiers of pre-written skills shipping with hermes-agent itself.</t>
+        </is>
+      </c>
+      <c r="C8" s="8" t="inlineStr">
+        <is>
+          <t>166 tracked skills total: 87 bundled (seed automatically on install, tracked via .bundled_manifest, opt out with `hermes skills opt-out`) + 79 optional (live under official/ in the repo, installed on demand with `hermes skills install official/&lt;path&gt;`, skip the third-party community-skill security scan since they're first-party).</t>
+        </is>
+      </c>
+      <c r="D8" s="8" t="inlineStr">
+        <is>
+          <t>Review the bundled set once hermes-vps exists (`hermes skills list`) before assuming anything needs installing — some of what Memory/Soul/Tool-layer already decided may already be covered by a bundled skill.</t>
+        </is>
+      </c>
+      <c r="E8" s="8" t="inlineStr">
+        <is>
+          <t>Not yet reviewed against bundled list</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="8" t="inlineStr">
+        <is>
+          <t>Self-authored skill creation</t>
+        </is>
+      </c>
+      <c r="B9" s="8" t="inlineStr">
+        <is>
+          <t>How the agent writes its *own* new skills during use — the actual 'self-improvement via skills' loop.</t>
+        </is>
+      </c>
+      <c r="C9" s="8" t="inlineStr">
+        <is>
+          <t>Agent calls skill_manage(action=create/patch/patch-with-content/delete/write_file/remove_file). Docs describe it recording a new reusable skill after completing a complex task (~5+ tool calls) with zero human authoring. Writes can be gated: `skills.write_approval: true` stages them under ~/.hermes/pending/skills/ for human review instead of applying immediately.</t>
+        </is>
+      </c>
+      <c r="D9" s="8" t="inlineStr">
+        <is>
+          <t>Recommend `write_approval: true` at least initially — same 'review before trust' posture already applied to the unofficial Obscura plugin. Revisit once the agent's judgment on what's worth turning into a skill has a track record.</t>
+        </is>
+      </c>
+      <c r="E9" s="8" t="inlineStr">
+        <is>
+          <t>Not yet configured</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="8" t="inlineStr">
+        <is>
+          <t>Security &amp; sandboxing</t>
+        </is>
+      </c>
+      <c r="B10" s="8" t="inlineStr">
+        <is>
+          <t>What stops an installed or self-written skill from doing something malicious.</t>
+        </is>
+      </c>
+      <c r="C10" s="8" t="inlineStr">
+        <is>
+          <t>Hub-installed skills get scanned for data exfiltration, prompt injection, destructive commands, and supply-chain signals; an optional NVIDIA SkillEvaluator Tier-1 scan adds PII detection. Project-local skills (.hermes/skills/ inside a git repo) get the same scanner before entering the index, with dangerous findings quarantined. Skills can declare required_environment_variables, which Hermes requests and passes through to execute_code/terminal sandboxes automatically.</t>
+        </is>
+      </c>
+      <c r="D10" s="8" t="inlineStr">
+        <is>
+          <t>The required_environment_variables mechanism is a second place secrets can leak outside the vault (05_Secrets_Vault) if a skill mishandles them — worth a Security Hardening row once any skill actually declares one.</t>
+        </is>
+      </c>
+      <c r="E10" s="8" t="inlineStr">
+        <is>
+          <t>Understood, no mitigating row logged yet</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="8" t="inlineStr">
+        <is>
+          <t>Bundled categories relevant here</t>
+        </is>
+      </c>
+      <c r="B11" s="8" t="inlineStr">
+        <is>
+          <t>Which of the 12 bundled categories actually matter for this project's shape.</t>
+        </is>
+      </c>
+      <c r="C11" s="8" t="inlineStr">
+        <is>
+          <t>Autonomous AI Agents (delegate to Claude Code / Codex / OpenCode, computer automation, Hermes-orchestrates-Hermes), DevOps (lifecycle review, Kanban handoff verification), Productivity (Google Workspace, Office docs, meeting action items), Research (arXiv, competitor monitoring, citation grounding), Email (IMAP/SMTP via Himalaya CLI).</t>
+        </is>
+      </c>
+      <c r="D11" s="8" t="inlineStr">
+        <is>
+          <t>'Autonomous AI Agents' directly overlaps the Codex-as-thinking-tier routing decision already locked (03_Model_Routing_Resilience) — check this category first once hermes-vps exists, it may already implement part of that routing instead of needing custom work.</t>
+        </is>
+      </c>
+      <c r="E11" s="8" t="inlineStr">
+        <is>
+          <t>Not yet cross-checked against 03_Model_Routing_Resilience</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="8" t="inlineStr">
+        <is>
+          <t>Optional categories relevant here</t>
+        </is>
+      </c>
+      <c r="B12" s="8" t="inlineStr">
+        <is>
+          <t>Which of the 23 optional categories are worth installing given this project's actual needs.</t>
+        </is>
+      </c>
+      <c r="C12" s="8" t="inlineStr">
+        <is>
+          <t>smart-home (Philips Hue via OpenHue CLI — only relevant if Hue exists on the home network, unconfirmed), security (1Password, Sherlock account discovery, data-broker removal), devops (Docker container mgmt, SSH tunneling, RSS/JSON API monitoring — overlaps the Docker terminal backend already locked), mcp (build/deploy custom MCP servers, OAuth handling — overlaps the 4 custom MCP servers already in 04_Tool_MCP_Layer), data-science (Jupyter notebook execution).</t>
+        </is>
+      </c>
+      <c r="D12" s="8" t="inlineStr">
+        <is>
+          <t>mcp and devops optional-skill categories are the two with real near-term relevance — they overlap tooling this project is already hand-building (TM-01 through TM-14). Worth checking whether the optional skill replaces hand-rolled work before building more MCP servers manually.</t>
+        </is>
+      </c>
+      <c r="E12" s="8" t="inlineStr">
+        <is>
+          <t>Candidates identified, none installed — needs explicit go-ahead, this is still discovery</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="8" t="inlineStr">
+        <is>
+          <t>Open question for next session</t>
+        </is>
+      </c>
+      <c r="B13" s="8" t="inlineStr">
+        <is>
+          <t>What this discovery pass did NOT resolve.</t>
+        </is>
+      </c>
+      <c r="C13" s="8" t="inlineStr">
+        <is>
+          <t>Whether any home-network device (Hue, etc.) actually exists to make smart-home skills relevant; whether bundled skills already cover gaps currently tracked as custom work in 01-15 tabs; exact behavior of hermes skills opt-out (full vs partial).</t>
+        </is>
+      </c>
+      <c r="D13" s="8" t="inlineStr">
+        <is>
+          <t>Answer by running `hermes skills list` and `hermes skills search &lt;keyword&gt;` directly against hermes-vps once it exists, rather than guessing further from docs alone.</t>
+        </is>
+      </c>
+      <c r="E13" s="8" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A2:E2"/>
+    <mergeCell ref="A1:E1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
@@ -12989,8 +13307,8 @@
           <t>Required: confirmed reachable + one real exchange with the local model. Lives in 03_Model_Routing_Resilience; will need re-verification once 07_Local_Inference's runtime changes.</t>
         </is>
       </c>
-      <c r="D33" s="19" t="n"/>
-      <c r="E33" s="19" t="n"/>
+      <c r="D33" s="17" t="n"/>
+      <c r="E33" s="18" t="n"/>
     </row>
     <row r="34" ht="44" customHeight="1">
       <c r="A34" s="8" t="inlineStr">
@@ -13008,8 +13326,8 @@
           <t>Required: verified on Ollama, multiple qwen3-vl variants loaded. Lives in 07_Local_Inference LI-03/LI-04 — must be re-proven on whichever runtime replaces Ollama.</t>
         </is>
       </c>
-      <c r="D34" s="19" t="n"/>
-      <c r="E34" s="19" t="n"/>
+      <c r="D34" s="17" t="n"/>
+      <c r="E34" s="18" t="n"/>
     </row>
     <row r="35" ht="44" customHeight="1">
       <c r="A35" s="8" t="inlineStr">
@@ -13027,8 +13345,8 @@
           <t>Required: box up, agent process live. Lives in 01_Core_Runtime CR-01 to CR-03.</t>
         </is>
       </c>
-      <c r="D35" s="19" t="n"/>
-      <c r="E35" s="19" t="n"/>
+      <c r="D35" s="17" t="n"/>
+      <c r="E35" s="18" t="n"/>
     </row>
     <row r="36" ht="44" customHeight="1">
       <c r="A36" s="8" t="inlineStr">
@@ -13046,8 +13364,8 @@
           <t>Required: tunnel + subnet routing, verified end-to-end. Lives in 06_Home_Network_Boundary HN-01/HN-02.</t>
         </is>
       </c>
-      <c r="D36" s="19" t="n"/>
-      <c r="E36" s="19" t="n"/>
+      <c r="D36" s="17" t="n"/>
+      <c r="E36" s="18" t="n"/>
     </row>
     <row r="37" ht="44" customHeight="1">
       <c r="A37" s="8" t="inlineStr">
@@ -13065,8 +13383,8 @@
           <t>Required: native link+code flow, one real coding task. Lives in 03_Model_Routing_Resilience MR-01.</t>
         </is>
       </c>
-      <c r="D37" s="19" t="n"/>
-      <c r="E37" s="19" t="n"/>
+      <c r="D37" s="17" t="n"/>
+      <c r="E37" s="18" t="n"/>
     </row>
     <row r="38" ht="44" customHeight="1">
       <c r="A38" s="8" t="inlineStr">
@@ -13084,8 +13402,8 @@
           <t>Required: Desktop pointed at VPS backend, proven identical from two places. Lives in 08_Interfaces_Access IA-03/IA-04, blocked on 02_Identity_Memory IM-03.</t>
         </is>
       </c>
-      <c r="D38" s="19" t="n"/>
-      <c r="E38" s="19" t="n"/>
+      <c r="D38" s="17" t="n"/>
+      <c r="E38" s="18" t="n"/>
     </row>
     <row r="39" ht="44" customHeight="1">
       <c r="A39" s="8" t="inlineStr">
@@ -13103,8 +13421,8 @@
           <t>Required: a real messaging channel on top of hermes-gateway. Lives in 08_Interfaces_Access IA-05.</t>
         </is>
       </c>
-      <c r="D39" s="19" t="n"/>
-      <c r="E39" s="19" t="n"/>
+      <c r="D39" s="17" t="n"/>
+      <c r="E39" s="18" t="n"/>
     </row>
     <row r="40" ht="44" customHeight="1">
       <c r="A40" s="8" t="inlineStr">
@@ -13122,8 +13440,8 @@
           <t>Required: one prompt stays local, one escalates, both observed. The router-llm-as-judge-rebuild-2026-09-28 catalog entry already shows this happened — update the catalog goal's status field to match.</t>
         </is>
       </c>
-      <c r="D40" s="19" t="n"/>
-      <c r="E40" s="19" t="n"/>
+      <c r="D40" s="17" t="n"/>
+      <c r="E40" s="18" t="n"/>
     </row>
     <row r="41" ht="44" customHeight="1">
       <c r="A41" s="8" t="inlineStr">
@@ -13141,13 +13459,13 @@
           <t>Required: cancel once ChatGPT Plus/Codex covers the same ground. Lives in 11_Cost_Subscriptions CS-03 — the literal finish line.</t>
         </is>
       </c>
-      <c r="D41" s="19" t="n"/>
-      <c r="E41" s="19" t="n"/>
+      <c r="D41" s="17" t="n"/>
+      <c r="E41" s="18" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="18">
+    <mergeCell ref="C36:E36"/>
     <mergeCell ref="C33:E33"/>
-    <mergeCell ref="C36:E36"/>
     <mergeCell ref="A26:E26"/>
     <mergeCell ref="A24:E24"/>
     <mergeCell ref="A2:E2"/>

</xml_diff>

<commit_message>
Research Crons pillar: D4_Crons_System tab, capability-only scope
Verified against primary source (cron/AGENTS.md, scheduler_provider.py,
official cron.md docs) rather than secondary summaries, per the
established verification practice from the Skills pillar pass.

Scoped per explicit instruction: confirm the system CAN schedule work,
don't design actual jobs. Key finding: the one hard prerequisite
(a persistent gateway process, since the ticker runs inside it) is
already satisfied -- CR-03 (hermes-gateway.service) has been Done.
No cron jobs created.

Flagged a real cross-pillar interaction in 02_Identity_Memory IM-05:
cron sessions pass skip_memory=True, so Hindsight will not see or
inform cron job output once deployed.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Hermes_Way.xlsx
+++ b/Hermes_Way.xlsx
@@ -29,6 +29,7 @@
     <sheet name="D1_Vultr_Services_Audit" sheetId="20" state="visible" r:id="rId20"/>
     <sheet name="D2_Providers_And_Deps" sheetId="21" state="visible" r:id="rId21"/>
     <sheet name="D3_Skills_System" sheetId="22" state="visible" r:id="rId22"/>
+    <sheet name="D4_Crons_System" sheetId="23" state="visible" r:id="rId23"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -953,7 +954,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A75"/>
+  <dimension ref="A1:A78"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -1415,40 +1416,61 @@
       </c>
     </row>
     <row r="70">
-      <c r="A70" s="3" t="inlineStr"/>
+      <c r="A70" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  D4_Crons_System              how the Crons pillar actually works (scheduler, config, hardening) -- capability confirmed, no jobs created</t>
+        </is>
+      </c>
     </row>
     <row r="71">
-      <c r="A71" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Found 2026-10-04: Nous's own framing is 'Five Pillars' -- Memory, Skills, Soul, Crons, Self-</t>
-        </is>
-      </c>
+      <c r="A71" s="3" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Improvement. Memory+Soul covered in 02_Identity_Memory. Skills researched 2026-10-04 (see</t>
+          <t xml:space="preserve">  Found 2026-10-04: Nous's own framing is 'Five Pillars' -- Memory, Skills, Soul, Crons, Self-</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">  D3_Skills_System) -- SKILL.md format, bundled/optional catalogs, self-authored creation,</t>
+          <t xml:space="preserve">  Improvement. Memory+Soul covered in 02_Identity_Memory. Skills (D3) and Crons (D4) researched</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">  security scanning all covered; no categories installed yet, still discovery. Crons and Self-</t>
+          <t xml:space="preserve">  and verified against primary source 2026-10-04/05 -- two numeric errors from secondary sources</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Improvement remain real pillars with zero coverage anywhere in this workbook -- not yet researched.</t>
+          <t xml:space="preserve">  caught and fixed in the process (Skills catalog count, Hindsight benchmark figure). Crons</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  capability is confirmed real and its one hard prerequisite (persistent gateway, CR-03) is</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  already Done -- no jobs created, per explicit instruction this stays capability-only. Self-</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Improvement remains the one pillar with zero coverage -- not yet researched.</t>
         </is>
       </c>
     </row>
@@ -12507,6 +12529,343 @@
       <c r="E13" s="8" t="inlineStr">
         <is>
           <t>Open</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A2:E2"/>
+    <mergeCell ref="A1:E1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="008A5A2E"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E14"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="36" customWidth="1" min="2" max="2"/>
+    <col width="50" customWidth="1" min="3" max="3"/>
+    <col width="54" customWidth="1" min="4" max="4"/>
+    <col width="20" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="22" customHeight="1">
+      <c r="A1" s="6" t="inlineStr">
+        <is>
+          <t>Discovery — Crons System (Five Pillars: Crons)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="16" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Researched 2026-10-05, verified against primary source (github.com/NousResearch/hermes-agent cron/AGENTS.md, cron/scheduler_provider.py, website/docs/user-guide/features/cron.md), not secondary summaries. Scope per explicit user instruction: confirm the SYSTEM CAN schedule work, not design actual cron jobs -- no jobs created, still discovery.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="7" t="inlineStr">
+        <is>
+          <t>Topic</t>
+        </is>
+      </c>
+      <c r="B4" s="7" t="inlineStr">
+        <is>
+          <t>What it is</t>
+        </is>
+      </c>
+      <c r="C4" s="7" t="inlineStr">
+        <is>
+          <t>Options found</t>
+        </is>
+      </c>
+      <c r="D4" s="7" t="inlineStr">
+        <is>
+          <t>Recommendation / dependency detail</t>
+        </is>
+      </c>
+      <c r="E4" s="7" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="8" t="inlineStr">
+        <is>
+          <t>What cron is</t>
+        </is>
+      </c>
+      <c r="B5" s="8" t="inlineStr">
+        <is>
+          <t>Hermes's built-in scheduler -- the pillar answering 'can it work without being summoned.'</t>
+        </is>
+      </c>
+      <c r="C5" s="8" t="inlineStr">
+        <is>
+          <t>cron/jobs.py (job store) + cron/scheduler.py (tick loop) + scheduler_*.py siblings. Users: `hermes cron &lt;verb&gt;` or `/cron`. Agents: the `cronjob` tool. A genuinely mature subsystem -- the internal dev notes (cron/AGENTS.md) cite specific hardening fixes by bug number (#107485, #114587, #122222), not a thin wrapper.</t>
+        </is>
+      </c>
+      <c r="D5" s="8" t="inlineStr">
+        <is>
+          <t>Treat as production-grade, not experimental -- the only EXPERIMENTAL-labeled piece is the pluggable external-provider interface (scheduler_provider.py), not the builtin scheduler itself.</t>
+        </is>
+      </c>
+      <c r="E5" s="8" t="inlineStr">
+        <is>
+          <t>Verified real</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="8" t="inlineStr">
+        <is>
+          <t>Hard prerequisite: persistent gateway</t>
+        </is>
+      </c>
+      <c r="B6" s="8" t="inlineStr">
+        <is>
+          <t>Cron jobs are ticked by a loop that runs INSIDE the gateway process -- no gateway process running means no cron ever fires.</t>
+        </is>
+      </c>
+      <c r="C6" s="8" t="inlineStr">
+        <is>
+          <t>`hermes gateway install` (user service) / `sudo hermes gateway install --system` (boot-time) / `hermes gateway` (foreground). The ticker is a SupervisedTickerThread started on gateway boot. One host gateway process ticks EVERY served profile's store -- relevant if CR-15 (sister's separate Hermes) ever shares infra.</t>
+        </is>
+      </c>
+      <c r="D6" s="8" t="inlineStr">
+        <is>
+          <t>ALREADY SATISFIED on hermes-vps -- cross-ref 01_Core_Runtime CR-03 'hermes-gateway running persistently', status Done, evidence hermes-gateway.service (systemd). This is the one thing this pillar actually needed built, and it already is.</t>
+        </is>
+      </c>
+      <c r="E6" s="8" t="inlineStr">
+        <is>
+          <t>Done (via CR-03) -- confirmed, not re-tracked here</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="8" t="inlineStr">
+        <is>
+          <t>Schedule formats</t>
+        </is>
+      </c>
+      <c r="B7" s="8" t="inlineStr">
+        <is>
+          <t>What a job's timing can be expressed as.</t>
+        </is>
+      </c>
+      <c r="C7" s="8" t="inlineStr">
+        <is>
+          <t>Relative one-shot (`in 30m`, `in 2h`, `in 1d`); recurring interval (`every 30m`, `every 2h`); natural recurring (`every monday 9am`, `weekdays at 9am`, `daily at 7am`); 5-field cron expressions (`0 9 * * *`); ISO one-shot timestamps.</t>
+        </is>
+      </c>
+      <c r="D7" s="8" t="inlineStr">
+        <is>
+          <t>No decision needed here -- this is a format reference for whenever a real job gets created, not a choice to lock in now.</t>
+        </is>
+      </c>
+      <c r="E7" s="8" t="inlineStr">
+        <is>
+          <t>Understood, not used</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="8" t="inlineStr">
+        <is>
+          <t>Per-job capabilities</t>
+        </is>
+      </c>
+      <c r="B8" s="8" t="inlineStr">
+        <is>
+          <t>What a single cron job definition can actually do, beyond 'run a prompt on a timer.'</t>
+        </is>
+      </c>
+      <c r="C8" s="8" t="inlineStr">
+        <is>
+          <t>Fields: `skills` (attach specific skills to the run), `model`/`provider` override, `script` (pre-run data-collection script piped into the prompt), `--no-agent` (script output delivered verbatim, skips the LLM entirely -- a watchdog pattern), `context_from` (chain job A's last output into job B's prompt), `workdir` (loads that directory's AGENTS.md/CLAUDE.md), multi-platform delivery targets.</t>
+        </is>
+      </c>
+      <c r="D8" s="8" t="inlineStr">
+        <is>
+          <t>The --no-agent script-only mode is the right fit for cheap health-check-style jobs (e.g. monitoring hermes-vps resource headroom, CR-12) once that's wanted -- no LLM cost, verbatim script stdout delivered only when non-empty.</t>
+        </is>
+      </c>
+      <c r="E8" s="8" t="inlineStr">
+        <is>
+          <t>Understood, not used</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="8" t="inlineStr">
+        <is>
+          <t>Delivery</t>
+        </is>
+      </c>
+      <c r="B9" s="8" t="inlineStr">
+        <is>
+          <t>Where a job's output actually goes once it runs.</t>
+        </is>
+      </c>
+      <c r="C9" s="8" t="inlineStr">
+        <is>
+          <t>`origin` (back to the creating chat, platform default), `local` (~/.hermes/cron/output/, CLI default), `telegram`/`telegram:&lt;chat_id&gt;`, `discord`, `slack`, `email`, `sms`, `all` (every connected home channel), comma-separated multiple targets, `bot-chat`.</t>
+        </is>
+      </c>
+      <c r="D9" s="8" t="inlineStr">
+        <is>
+          <t>Telegram delivery directly reuses the IA-05 gateway decision already locked -- no new dependency once that bot token exists.</t>
+        </is>
+      </c>
+      <c r="E9" s="8" t="inlineStr">
+        <is>
+          <t>Understood, not used</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="8" t="inlineStr">
+        <is>
+          <t>Config keys</t>
+        </is>
+      </c>
+      <c r="B10" s="8" t="inlineStr">
+        <is>
+          <t>What config.yaml controls for the whole cron subsystem.</t>
+        </is>
+      </c>
+      <c r="C10" s="8" t="inlineStr">
+        <is>
+          <t>`cron.model`/`model_provider` (default for unpinned jobs), `preflight` (validate before run), `wrap_response`, `catch_up_missed` (re-run once on restart if a fire was missed), `failure_nudge_threshold`, `retry_unreachable` (auto-retry transient network errors at 5/15/30min), `failure_repeat_alert_hours`, `allow_agent_scheduling` (default false -- cron-run sessions cannot recursively create more cron jobs unless this is on), `max_parallel_jobs` (default 10), `script_timeout_seconds` (default 3600), `cron.provider` (external scheduler override, defaults to builtin).</t>
+        </is>
+      </c>
+      <c r="D10" s="8" t="inlineStr">
+        <is>
+          <t>`allow_agent_scheduling: false` (the default) is the right posture to keep -- matches the same 'review before autonomy' stance already applied to skill write_approval and the Obscura plugin.</t>
+        </is>
+      </c>
+      <c r="E10" s="8" t="inlineStr">
+        <is>
+          <t>Understood, not configured</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="8" t="inlineStr">
+        <is>
+          <t>Storage</t>
+        </is>
+      </c>
+      <c r="B11" s="8" t="inlineStr">
+        <is>
+          <t>Where cron state physically lives.</t>
+        </is>
+      </c>
+      <c r="C11" s="8" t="inlineStr">
+        <is>
+          <t>Job definitions: ~/.hermes/cron/jobs.json. Run outputs: ~/.hermes/cron/output/{job_id}/{timestamp}.md. Execution history: ~/.hermes/cron/executions.db.</t>
+        </is>
+      </c>
+      <c r="D11" s="8" t="inlineStr">
+        <is>
+          <t>All on-box, no external dependency -- consistent with the hermes-vps self-sufficiency rule.</t>
+        </is>
+      </c>
+      <c r="E11" s="8" t="inlineStr">
+        <is>
+          <t>Understood, not used</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="8" t="inlineStr">
+        <is>
+          <t>Hardening (why this isn't a toy scheduler)</t>
+        </is>
+      </c>
+      <c r="B12" s="8" t="inlineStr">
+        <is>
+          <t>Failure modes the system already guards against, per cron/AGENTS.md.</t>
+        </is>
+      </c>
+      <c r="C12" s="8" t="inlineStr">
+        <is>
+          <t>Inactivity watchdog on cron sessions (default 600s idle via HERMES_CRON_TIMEOUT, separate from script_timeout_seconds); catch-up window for missed one-shots (120s grace); per-home tick lock file prevents duplicate ticks across processes; restart-safe external worker processes under systemd; at-most-once accounting across a mid-run crash (next_run_at advances before dispatch).</t>
+        </is>
+      </c>
+      <c r="D12" s="8" t="inlineStr">
+        <is>
+          <t>No action needed -- flagging so a future session doesn't assume this needs building when it's already handled.</t>
+        </is>
+      </c>
+      <c r="E12" s="8" t="inlineStr">
+        <is>
+          <t>Verified real, nothing to build</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="8" t="inlineStr">
+        <is>
+          <t>Cross-pillar interaction: memory does NOT run during cron</t>
+        </is>
+      </c>
+      <c r="B13" s="8" t="inlineStr">
+        <is>
+          <t>A real gotcha found while verifying, not mentioned in any secondary source.</t>
+        </is>
+      </c>
+      <c r="C13" s="8" t="inlineStr">
+        <is>
+          <t>Direct quote, cron/AGENTS.md: 'Cron sessions pass skip_memory=True; memory providers intentionally do not run during cron.'</t>
+        </is>
+      </c>
+      <c r="D13" s="8" t="inlineStr">
+        <is>
+          <t>Worth a Notes/Next-Action flag on IM-05 (Hindsight) once memory is actually deployed: a cron job's output won't be written to or informed by extended memory unless something explicitly changes that. Not a blocker, just don't assume cron jobs get the same memory context an interactive chat gets.</t>
+        </is>
+      </c>
+      <c r="E13" s="8" t="inlineStr">
+        <is>
+          <t>Flagged — see 02_Identity_Memory IM-05</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="8" t="inlineStr">
+        <is>
+          <t>Adjacent but out of scope: Kanban</t>
+        </is>
+      </c>
+      <c r="B14" s="8" t="inlineStr">
+        <is>
+          <t>A related multi-agent work-queue system documented in the same source file as cron, easy to conflate with it.</t>
+        </is>
+      </c>
+      <c r="C14" s="8" t="inlineStr">
+        <is>
+          <t>SQLite-backed board for multiple profiles/workers to collaborate (hermes kanban &lt;verb&gt;). Separate feature, separate toolset, not part of the Five Pillars.</t>
+        </is>
+      </c>
+      <c r="D14" s="8" t="inlineStr">
+        <is>
+          <t>Noting its existence only so it isn't mistaken for part of Crons later -- not pursued in this discovery pass.</t>
+        </is>
+      </c>
+      <c r="E14" s="8" t="inlineStr">
+        <is>
+          <t>Noted, not researched</t>
         </is>
       </c>
     </row>
@@ -15146,7 +15505,7 @@
       </c>
       <c r="J9" s="8" t="inlineStr">
         <is>
-          <t>Decided, not yet deployed. Depends on SV-15 landing first for the shared-database option</t>
+          <t>Decided, not yet deployed. Depends on SV-15 landing first for the shared-database option Found 2026-10-05 (see D4_Crons_System): cron-run sessions pass skip_memory=True -- Hindsight will NOT see or inform cron job output unless that changes. Not a blocker, just dont assume cron jobs get interactive-chat memory context.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Research Self-Improvement pillar; Five Pillars discovery now complete
Verified against primary source (agent/background_review.py,
agent/curator.py, agent/AGENTS.md, skills/AGENTS.md) rather than
secondary summaries, same discipline as Skills/Crons.

Three real mechanisms, not one feature: per-turn background review
(forks the agent, writes memory/skills directly, configurable model
routing that overlaps the existing router decision), skill Curator
(lifecycle management restricted to self-authored skills only, never
touches bundled/hub-installed), and free FTS5 cross-session search.

All five pillars (Memory, Soul, Skills, Crons, Self-Improvement) are
now researched and verified. Discovery only -- nothing configured.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Hermes_Way.xlsx
+++ b/Hermes_Way.xlsx
@@ -30,6 +30,7 @@
     <sheet name="D2_Providers_And_Deps" sheetId="21" state="visible" r:id="rId21"/>
     <sheet name="D3_Skills_System" sheetId="22" state="visible" r:id="rId22"/>
     <sheet name="D4_Crons_System" sheetId="23" state="visible" r:id="rId23"/>
+    <sheet name="D5_Self_Improvement" sheetId="24" state="visible" r:id="rId24"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -954,7 +955,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A78"/>
+  <dimension ref="A1:A79"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -1423,54 +1424,61 @@
       </c>
     </row>
     <row r="71">
-      <c r="A71" s="3" t="inlineStr"/>
+      <c r="A71" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  D5_Self_Improvement          how the Self-Improvement pillar actually works (background review, Curator, session search)</t>
+        </is>
+      </c>
     </row>
     <row r="72">
-      <c r="A72" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Found 2026-10-04: Nous's own framing is 'Five Pillars' -- Memory, Skills, Soul, Crons, Self-</t>
-        </is>
-      </c>
+      <c r="A72" s="3" t="inlineStr"/>
     </row>
     <row r="73">
       <c r="A73" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Improvement. Memory+Soul covered in 02_Identity_Memory. Skills (D3) and Crons (D4) researched</t>
+          <t xml:space="preserve">  Found 2026-10-04: Nous's own framing is 'Five Pillars' -- Memory, Skills, Soul, Crons, Self-</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">  and verified against primary source 2026-10-04/05 -- two numeric errors from secondary sources</t>
+          <t xml:space="preserve">  Improvement. ALL FIVE now researched and verified against primary source as of 2026-10-05</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">  caught and fixed in the process (Skills catalog count, Hindsight benchmark figure). Crons</t>
+          <t xml:space="preserve">  (02_Identity_Memory for Memory/Soul; D3/D4/D5 for Skills/Crons/Self-Improvement). Two</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">  capability is confirmed real and its one hard prerequisite (persistent gateway, CR-03) is</t>
+          <t xml:space="preserve">  numeric errors from secondary sources caught and fixed along the way (Skills catalog count,</t>
         </is>
       </c>
     </row>
     <row r="77">
-      <c r="A77" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  already Done -- no jobs created, per explicit instruction this stays capability-only. Self-</t>
+      <c r="A77" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Hindsight benchmark figure). Crons and Self-Improvement capability both confirmed real and</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Improvement remains the one pillar with zero coverage -- not yet researched.</t>
+          <t xml:space="preserve">  largely already satisfied by existing infra (CR-03 gateway) or built into hermes-agent itself</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  -- no jobs/configuration actually created for either, per explicit discovery-only instruction.</t>
         </is>
       </c>
     </row>
@@ -12866,6 +12874,289 @@
       <c r="E14" s="8" t="inlineStr">
         <is>
           <t>Noted, not researched</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A2:E2"/>
+    <mergeCell ref="A1:E1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="008A5A2E"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E12"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="36" customWidth="1" min="2" max="2"/>
+    <col width="50" customWidth="1" min="3" max="3"/>
+    <col width="54" customWidth="1" min="4" max="4"/>
+    <col width="20" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="22" customHeight="1">
+      <c r="A1" s="6" t="inlineStr">
+        <is>
+          <t>Discovery — Self-Improvement System (Five Pillars: Self-Improvement)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="16" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Researched 2026-10-05, verified against primary source (github.com/NousResearch/hermes-agent agent/background_review.py, agent/curator.py, agent/AGENTS.md, skills/AGENTS.md, and the official memory.md / curator.md docs) before writing anything here. Last of the Five Pillars -- none of Memory/Soul/Skills/Crons/Self-Improvement remain unresearched after this tab.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="7" t="inlineStr">
+        <is>
+          <t>Topic</t>
+        </is>
+      </c>
+      <c r="B4" s="7" t="inlineStr">
+        <is>
+          <t>What it is</t>
+        </is>
+      </c>
+      <c r="C4" s="7" t="inlineStr">
+        <is>
+          <t>Options found</t>
+        </is>
+      </c>
+      <c r="D4" s="7" t="inlineStr">
+        <is>
+          <t>Recommendation / dependency detail</t>
+        </is>
+      </c>
+      <c r="E4" s="7" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="8" t="inlineStr">
+        <is>
+          <t>What self-improvement actually is</t>
+        </is>
+      </c>
+      <c r="B5" s="8" t="inlineStr">
+        <is>
+          <t>Not one feature -- three distinct mechanisms working together: a per-turn background review, a skill lifecycle manager (Curator), and free cross-session search.</t>
+        </is>
+      </c>
+      <c r="C5" s="8" t="inlineStr">
+        <is>
+          <t>agent/background_review.py (+ review_engine.py, review_idle_queue.py), agent/curator.py (+ curator_backup.py), tools/session_search_tool.py. All three confirmed real and substantial in source, not a marketing label over something thin.</t>
+        </is>
+      </c>
+      <c r="D5" s="8" t="inlineStr">
+        <is>
+          <t>The 'work -&gt; learn -&gt; save to memory/skills -&gt; search past sessions' framing from the earlier session summary is directionally right but understates it -- there's a whole skill-lifecycle subsystem (Curator) that framing didn't mention at all.</t>
+        </is>
+      </c>
+      <c r="E5" s="8" t="inlineStr">
+        <is>
+          <t>Verified real</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="8" t="inlineStr">
+        <is>
+          <t>Background review (the actual learning loop)</t>
+        </is>
+      </c>
+      <c r="B6" s="8" t="inlineStr">
+        <is>
+          <t>After every conversation turn, Hermes forks itself to ask 'should anything here be saved as a memory or a skill' -- and writes directly if so.</t>
+        </is>
+      </c>
+      <c r="C6" s="8" t="inlineStr">
+        <is>
+          <t>Direct quote, agent/background_review.py: 'Background memory/skill review — fork the agent to evaluate the turn... asks "should any skill/memory be saved or updated?". Writes go straight to the memory + skill stores; the main conversation and prompt cache are never touched.' Runs as a daemon thread, inherits the parent's live runtime (provider/model/credentials/cached system prompt) so it hits the same prompt-cache prefix, and runs under a restricted tool whitelist.</t>
+        </is>
+      </c>
+      <c r="D6" s="8" t="inlineStr">
+        <is>
+          <t>This is the mechanism that would actually act on this project's 'memory upkeep is Claude's job, not the user's' ground rule, once ported to Hermes itself -- it's architecturally the same idea (passive capture, not waiting to be asked), already built-in rather than something to design from scratch.</t>
+        </is>
+      </c>
+      <c r="E6" s="8" t="inlineStr">
+        <is>
+          <t>Verified real</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="8" t="inlineStr">
+        <is>
+          <t>Background review: model routing</t>
+        </is>
+      </c>
+      <c r="B7" s="8" t="inlineStr">
+        <is>
+          <t>Which model does the per-turn review -- doesn't have to be the expensive main model.</t>
+        </is>
+      </c>
+      <c r="C7" s="8" t="inlineStr">
+        <is>
+          <t>Config: `auxiliary.background_review.provider` / `.model` (e.g. route to a cheaper model like google/gemini-3-flash via openrouter), `.max_input_tokens` (cost cap), `.defer` (e.g. `auto` -- queues the review instead of running it immediately when a local GPU model is busy).</t>
+        </is>
+      </c>
+      <c r="D7" s="8" t="inlineStr">
+        <is>
+          <t>Directly overlaps the local-model-as-tool-tier / Codex-as-thinking-tier routing decision already made for this project (03_Model_Routing_Resilience) and the economic LLM-as-judge router. Background review is a THIRD consumer of that same routing logic, not a new concept -- check whether it can just plug into the existing router instead of getting separately configured.</t>
+        </is>
+      </c>
+      <c r="E7" s="8" t="inlineStr">
+        <is>
+          <t>Needs cross-check against 03_Model_Routing_Resilience once hermes-vps exists</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="8" t="inlineStr">
+        <is>
+          <t>Background review: approval gating</t>
+        </is>
+      </c>
+      <c r="B8" s="8" t="inlineStr">
+        <is>
+          <t>Whether a human reviews what gets auto-saved, same question already asked for Skills (write_approval).</t>
+        </is>
+      </c>
+      <c r="C8" s="8" t="inlineStr">
+        <is>
+          <t>`memory.write_approval` (default false) -- when true, background writes stage via `/memory pending` / `/memory approve` instead of applying directly; foreground (in-conversation) writes prompt inline instead.</t>
+        </is>
+      </c>
+      <c r="D8" s="8" t="inlineStr">
+        <is>
+          <t>Recommend `write_approval: true` initially -- same 'review before trust' posture already applied to skills.write_approval and the Obscura plugin. This is the memory-side twin of that same decision, should probably be set together, not separately.</t>
+        </is>
+      </c>
+      <c r="E8" s="8" t="inlineStr">
+        <is>
+          <t>Not yet configured</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="8" t="inlineStr">
+        <is>
+          <t>Skill Curator (lifecycle management)</t>
+        </is>
+      </c>
+      <c r="B9" s="8" t="inlineStr">
+        <is>
+          <t>Background maintenance that keeps self-authored skills from piling up as stale cruft -- the 'does it get better with use, or just bigger' question.</t>
+        </is>
+      </c>
+      <c r="C9" s="8" t="inlineStr">
+        <is>
+          <t>Deterministic auto-transitions (no LLM cost): active -&gt; stale (14d unused, configurable via `stale_after_days`) -&gt; archived (30d, `archive_after_days`) -&gt; `~/.hermes/skills/.archive/` (restorable, never hard-deleted). Optional LLM consolidation pass (`curator.consolidate`, off by default, token cost) can merge overlapping skills or patch drift. Runs on an inactivity schedule (default 7 days since last run + 2h agent idle, `min_idle_hours`), not on a cron timer. Pre-run tar.gz backups + rollback. CLI: `hermes curator status|run|pause|resume|pin|unpin|archive|restore|prune|backup|rollback`.</t>
+        </is>
+      </c>
+      <c r="D9" s="8" t="inlineStr">
+        <is>
+          <t>CONFIRMED (source, not docs page): Curator only ever touches skills with `created_by: "agent"` -- bundled and hub-installed skills are permanently off-limits to it, even with `prune_builtins` on for the deterministic walk. This is a real safety boundary worth knowing before assuming Curator could ever 'clean up' something you installed yourself.</t>
+        </is>
+      </c>
+      <c r="E9" s="8" t="inlineStr">
+        <is>
+          <t>Verified real</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="8" t="inlineStr">
+        <is>
+          <t>Cross-session search</t>
+        </is>
+      </c>
+      <c r="B10" s="8" t="inlineStr">
+        <is>
+          <t>How the agent finds something from a conversation weeks ago without it being in the 2,200-char MEMORY.md snapshot.</t>
+        </is>
+      </c>
+      <c r="C10" s="8" t="inlineStr">
+        <is>
+          <t>tools/session_search_tool.py queries `~/.hermes/state.db` (SQLite, FTS5 full-text index) across all CLI and messaging sessions. Returns actual past messages, no summarization/truncation, ~20ms, zero LLM cost.</t>
+        </is>
+      </c>
+      <c r="D10" s="8" t="inlineStr">
+        <is>
+          <t>This plus MEMORY.md are complementary, not redundant: MEMORY.md is the always-loaded curated snapshot (~1,300 tokens/session), session_search is free on-demand lookup for anything NOT curated into that snapshot. Matches the IM-07 retention policy already found (facts persisted aggressively, curation forces a filter) -- session_search is the safety net for what curation leaves out.</t>
+        </is>
+      </c>
+      <c r="E10" s="8" t="inlineStr">
+        <is>
+          <t>Verified real</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="8" t="inlineStr">
+        <is>
+          <t>Learning visibility (Desktop only)</t>
+        </is>
+      </c>
+      <c r="B11" s="8" t="inlineStr">
+        <is>
+          <t>A way for a human to actually SEE what the agent has learned, not just trust it happened.</t>
+        </is>
+      </c>
+      <c r="C11" s="8" t="inlineStr">
+        <is>
+          <t>agent/learning_graph.py assembles a graph for the Desktop app: skill nodes (agent-created/used) + MEMORY.md/USER.md chunks as nodes, linked via declared `related_skills` and lexical overlap. Visualization only, not a reasoning mechanism.</t>
+        </is>
+      </c>
+      <c r="D11" s="8" t="inlineStr">
+        <is>
+          <t>Relevant to 09_Observability ('health signals a human can actually see') once the Desktop interface (08_Interfaces_Access) is in use -- this is a built-in answer to 'how do I know self-improvement is actually doing anything,' not something to build custom.</t>
+        </is>
+      </c>
+      <c r="E11" s="8" t="inlineStr">
+        <is>
+          <t>Verified real, Desktop-dependent</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="8" t="inlineStr">
+        <is>
+          <t>Open question for next session</t>
+        </is>
+      </c>
+      <c r="B12" s="8" t="inlineStr">
+        <is>
+          <t>What this pass did NOT resolve.</t>
+        </is>
+      </c>
+      <c r="C12" s="8" t="inlineStr">
+        <is>
+          <t>Whether background_review still fires during a cron-run session (cron confirmed to skip memory PROVIDERS via skip_memory=True, per D4 -- unconfirmed whether the separate background_review/Curator mechanisms are also suppressed, since they write to MEMORY.md/skills directly rather than through a memory provider). Whether memory.write_approval and skills.write_approval need to be set together or are independent toggles in practice.</t>
+        </is>
+      </c>
+      <c r="D12" s="8" t="inlineStr">
+        <is>
+          <t>Answer by reading agent/review_engine.py's cron-session handling directly, or by testing once hermes-vps exists -- don't assume either way from the docs alone.</t>
+        </is>
+      </c>
+      <c r="E12" s="8" t="inlineStr">
+        <is>
+          <t>Open</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Close CR-03: verify gateway survives an actual reboot
Confirmed hermes-gateway.service is a system-level systemd unit
(/etc/systemd/system, multi-user.target.wants), not a --user service,
so loginctl Linger was never actually load-bearing for it (enabled
anyway, harmless). Performed a real reboot of hermes-vps; the gateway
came back active with zero login sessions and the dashboard responded.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Hermes_Way.xlsx
+++ b/Hermes_Way.xlsx
@@ -1506,7 +1506,6 @@
         </is>
       </c>
     </row>
-    <row r="83"/>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
@@ -15988,6 +15987,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="7" t="inlineStr">
         <is>
@@ -16158,7 +16158,7 @@
       </c>
       <c r="F7" s="8" t="inlineStr">
         <is>
-          <t>hermes-gateway.service</t>
+          <t>hermes-gateway.service (system-level unit, /etc/systemd/system, multi-user.target.wants) + real reboot 2026-10-05 17:5x UTC: active again at 17:57:00 with no login session (who=empty), dashboard HTTP 302 reachable</t>
         </is>
       </c>
       <c r="G7" s="8" t="n">
@@ -16175,7 +16175,7 @@
       </c>
       <c r="J7" s="8" t="inlineStr">
         <is>
-          <t>VERIFY 2026-10-05: 'Done' here needs re-checking against loginctl show-user $USER -p Linger (must read Linger=yes) -- a systemd --user service without linger survives logout but NOT an actual reboot. Confirm with a real reboot test, not just systemctl status. See D8_Advanced_Reference.</t>
+          <t>VERIFIED 2026-10-05: confirmed it's a system-level unit (not systemctl --user), so Linger was not actually load-bearing here (enabled it anyway on hermes user, harmless). Performed a real `reboot` of hermes-vps; service came back active automatically with zero logged-in sessions, dashboard responded post-boot. Reboot survival genuinely confirmed, not just systemctl status.</t>
         </is>
       </c>
     </row>
@@ -17300,6 +17300,7 @@
       <c r="I52" s="8" t="n"/>
       <c r="J52" s="8" t="n"/>
     </row>
+    <row r="53"/>
     <row r="54">
       <c r="B54" s="20" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Close CR-17: apply Docker terminal backend with safe memory cap
Set terminal.backend=docker and terminal.container_memory=1024 (the
5120MB default exceeds this box's 4GB RAM). Also fixed a docker-group
permission gap hermes doctor surfaced: the hermes user wasn't in the
docker group, so the daemon was unreachable until usermod -aG docker
hermes + a gateway restart.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Hermes_Way.xlsx
+++ b/Hermes_Way.xlsx
@@ -16779,12 +16779,12 @@
       </c>
       <c r="E21" s="8" t="inlineStr">
         <is>
-          <t>Partial</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F21" s="8" t="inlineStr">
         <is>
-          <t>hermes-five-provider-choices-locked-2026-10-04</t>
+          <t>config.yaml: terminal.backend=docker, terminal.container_memory=1024 (box is 3.8GiB total); hermes user added to docker group, gateway restarted, 'hermes doctor' confirms Docker (daemon running)</t>
         </is>
       </c>
       <c r="G21" s="8" t="n">
@@ -16801,7 +16801,7 @@
       </c>
       <c r="J21" s="8" t="inlineStr">
         <is>
-          <t>Decided, not yet applied to config.yaml Found 2026-10-05: terminal.container_memory defaults to 5120MB (5GB) -- hermes-vps only has 4GB total RAM. MUST be set lower explicitly or Docker-backed commands risk OOM. See D8_Advanced_Reference.</t>
+          <t>APPLIED 2026-10-05: set terminal.backend=docker and terminal.container_memory=1024 (down from the 5120 default that exceeded the box's 4GB RAM). hermes doctor flagged Docker as unreachable after the config change -- root cause was the hermes user not being in the docker group (permission denied on /var/run/docker.sock). Fixed with usermod -aG docker hermes + systemctl restart hermes-gateway to pick up the new group membership. Re-ran hermes doctor: Docker (daemon running) now green.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Close IM-01/IM-02/IM-09: commit SOUL.md/USER.md/MEMORY.md to hermes-vps
hermes chat --query-file (having Hermes write its own identity files)
failed three times: twice on protected_instruction_files approval
timeout in non-interactive mode, then once with a hallucinated
success report (claimed byte counts for files that were never
written, verified via filesystem search). Wrote the files directly
and verified with wc -c on the box.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Hermes_Way.xlsx
+++ b/Hermes_Way.xlsx
@@ -7186,7 +7186,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="7" t="inlineStr">
         <is>
@@ -8049,7 +8048,6 @@
       <c r="I42" s="8" t="n"/>
       <c r="J42" s="8" t="n"/>
     </row>
-    <row r="43"/>
     <row r="44">
       <c r="B44" s="20" t="inlineStr">
         <is>
@@ -17395,6 +17393,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="7" t="inlineStr">
         <is>
@@ -17470,12 +17469,12 @@
       </c>
       <c r="E5" s="8" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F5" s="8" t="inlineStr">
         <is>
-          <t>hermes-agent docs: user-guide/features/personality</t>
+          <t>SOUL.md committed 2026-10-06 (1660 bytes), verified via wc -c on hermes-vps.</t>
         </is>
       </c>
       <c r="G5" s="8" t="n">
@@ -17515,12 +17514,12 @@
       </c>
       <c r="E6" s="8" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F6" s="8" t="inlineStr">
         <is>
-          <t>hermes-vps filesystem</t>
+          <t>USER.md committed 2026-10-06 (1015 bytes), verified via wc -c on hermes-vps.</t>
         </is>
       </c>
       <c r="G6" s="8" t="n">
@@ -17826,12 +17825,12 @@
       </c>
       <c r="E13" s="8" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F13" s="8" t="inlineStr">
         <is>
-          <t>hermes-agent docs: persistent memory</t>
+          <t>MEMORY.md committed 2026-10-06 (1872 bytes), verified via wc -c on hermes-vps.</t>
         </is>
       </c>
       <c r="G13" s="8" t="n">
@@ -18298,6 +18297,7 @@
       <c r="I43" s="8" t="n"/>
       <c r="J43" s="8" t="n"/>
     </row>
+    <row r="44"/>
     <row r="45">
       <c r="B45" s="20" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Close CR-09/10/11/12/13/14/18: Core Runtime batch
- CR-09: registered hermes-vps + 5 services (gateway, complexity-router,
  Caddy, Dokploy, WireGuard) in the catalog hosts/services tables
- CR-18: confirmed the hermes-vps-ssh vault entry satisfies this
- CR-13: confirmed hermes config set/get is the safe edit method in
  practice (used throughout tonight, never raw YAML parse+dump)
- CR-10: unattended-upgrades already enabled by default on the Vultr
  image - verified, not built
- CR-11: wrote the upgrade trigger/test policy
- CR-12: deployed hermes-memcheck.timer, a 15-min systemd check that
  logs when available memory drops below 500MB (headroom is genuinely
  tight right now: 257MB free, 600MB already in swap)
- CR-14: confirmed hermes checkpoints (shadow-git auto-snapshot before
  writes) satisfies staged-config-change safety without custom tooling

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Hermes_Way.xlsx
+++ b/Hermes_Way.xlsx
@@ -16003,6 +16003,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="7" t="inlineStr">
         <is>
@@ -16442,12 +16443,12 @@
       </c>
       <c r="E13" s="8" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F13" s="8" t="inlineStr">
         <is>
-          <t>catalog hosts/services tables — missing</t>
+          <t>catalog host id 7 (hermes-vps) + 5 service rows (hermes-gateway, complexity-router, Caddy, Dokploy, WireGuard wg0) added 2026-10-06</t>
         </is>
       </c>
       <c r="G13" s="8" t="n">
@@ -16464,7 +16465,7 @@
       </c>
       <c r="J13" s="8" t="inlineStr">
         <is>
-          <t>Add hermes-vps as a host row, Caddy/Dokploy/gateway/router as service rows</t>
+          <t>Registered via PostgREST. Dokploy service row notes CR-06 as the remaining gap (admin credential not recoverable from docker env/logs).</t>
         </is>
       </c>
     </row>
@@ -16491,10 +16492,14 @@
       </c>
       <c r="E14" s="8" t="inlineStr">
         <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F14" s="8" t="inlineStr"/>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F14" s="8" t="inlineStr">
+        <is>
+          <t>systemctl is-enabled unattended-upgrades = enabled; /etc/apt/apt.conf.d/20auto-upgrades has Update-Package-Lists=1, Unattended-Upgrade=1</t>
+        </is>
+      </c>
       <c r="G14" s="8" t="n">
         <v>5</v>
       </c>
@@ -16507,7 +16512,11 @@
           <t>Platform/SRE</t>
         </is>
       </c>
-      <c r="J14" s="8" t="inlineStr"/>
+      <c r="J14" s="8" t="inlineStr">
+        <is>
+          <t>Already active on the Vultr image by default - verified 2026-10-06, not something that needed building.</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="8" t="inlineStr">
@@ -16532,10 +16541,14 @@
       </c>
       <c r="E15" s="8" t="inlineStr">
         <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F15" s="8" t="inlineStr"/>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F15" s="8" t="inlineStr">
+        <is>
+          <t>policy logged to catalog 2026-10-06</t>
+        </is>
+      </c>
       <c r="G15" s="8" t="n">
         <v>5</v>
       </c>
@@ -16548,7 +16561,11 @@
           <t>Platform/SRE</t>
         </is>
       </c>
-      <c r="J15" s="8" t="inlineStr"/>
+      <c r="J15" s="8" t="inlineStr">
+        <is>
+          <t>POLICY: upgrade is manual, triggered only when a specific needed fix/feature requires it (not merely 'commits behind'). After hermes update: re-run hermes doctor + hermes security audit, confirm hermes-gateway and complexity-router still active, before considering the upgrade final.</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="8" t="inlineStr">
@@ -16573,10 +16590,14 @@
       </c>
       <c r="E16" s="8" t="inlineStr">
         <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F16" s="8" t="inlineStr"/>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F16" s="8" t="inlineStr">
+        <is>
+          <t>hermes-memcheck.timer + .service (systemd, every 15min, logs via logger if available memory &lt;500MB). Current baseline 2026-10-06: 257MB free / 1.7GB available of 3.8GB total, 600MB already in swap.</t>
+        </is>
+      </c>
       <c r="G16" s="8" t="n">
         <v>5</v>
       </c>
@@ -16589,7 +16610,11 @@
           <t>Platform/SRE</t>
         </is>
       </c>
-      <c r="J16" s="8" t="inlineStr"/>
+      <c r="J16" s="8" t="inlineStr">
+        <is>
+          <t>Lightweight ceiling check, not full alerting (that's OB-02's job - cross-referenced). Headroom is confirmed genuinely tight, not hypothetical.</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="8" t="inlineStr">
@@ -16614,12 +16639,12 @@
       </c>
       <c r="E17" s="8" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F17" s="8" t="inlineStr">
         <is>
-          <t>scripts/ — no helper exists yet</t>
+          <t>hermes config set/get used exclusively throughout 2026-10-05/06 session (CR-17, SH-04, security.protected_instruction_files toggle) - never a raw PyYAML parse+dump</t>
         </is>
       </c>
       <c r="G17" s="8" t="n">
@@ -16636,7 +16661,7 @@
       </c>
       <c r="J17" s="8" t="inlineStr">
         <is>
-          <t>config-yaml-comments-stripped-2026-09-30 incident</t>
+          <t>Confirmed in practice: hermes's own config CLI is the safe method, sidesteps the comment-stripping incident entirely since it's not a full-file parse+rewrite.</t>
         </is>
       </c>
     </row>
@@ -16663,10 +16688,14 @@
       </c>
       <c r="E18" s="8" t="inlineStr">
         <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F18" s="8" t="inlineStr"/>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F18" s="8" t="inlineStr">
+        <is>
+          <t>hermes checkpoints status confirmed real: shadow git repo auto-snapshots before write_file/patch/terminal calls (/home/hermes/.hermes/checkpoints)</t>
+        </is>
+      </c>
       <c r="G18" s="8" t="n">
         <v>5</v>
       </c>
@@ -16679,7 +16708,11 @@
           <t>Hermes Design Specialist</t>
         </is>
       </c>
-      <c r="J18" s="8" t="inlineStr"/>
+      <c r="J18" s="8" t="inlineStr">
+        <is>
+          <t>Built-in mechanism satisfies this without custom tooling, per the D6_Web_Dashboard lead. hermes checkpoints list/status/prune available for recovery.</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="8" t="inlineStr">
@@ -16843,10 +16876,14 @@
       </c>
       <c r="E22" s="8" t="inlineStr">
         <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F22" s="8" t="n"/>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F22" s="8" t="inlineStr">
+        <is>
+          <t>vault secret hermes-vps-ssh (root@207.148.2.224, same key as default ~/.ssh/id_ed25519)</t>
+        </is>
+      </c>
       <c r="G22" s="8" t="n">
         <v>5</v>
       </c>
@@ -16861,7 +16898,7 @@
       </c>
       <c r="J22" s="8" t="inlineStr">
         <is>
-          <t>Blocking the execution phase kickoff -- vault it the moment it exists, never leave it in plaintext.</t>
+          <t>Vaulted 2026-10-05 before any execution work began. SSH tested and used continuously since.</t>
         </is>
       </c>
     </row>
@@ -17315,6 +17352,7 @@
       <c r="I52" s="8" t="n"/>
       <c r="J52" s="8" t="n"/>
     </row>
+    <row r="53"/>
     <row r="54">
       <c r="B54" s="20" t="inlineStr">
         <is>
@@ -17393,7 +17431,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="7" t="inlineStr">
         <is>
@@ -18297,7 +18334,6 @@
       <c r="I43" s="8" t="n"/>
       <c r="J43" s="8" t="n"/>
     </row>
-    <row r="44"/>
     <row r="45">
       <c r="B45" s="20" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
IM-02: separate general USER.md from project-specific facts
Established principle: SOUL.md/memories/USER.md/MEMORY.md are general
to Hermes as a whole, never project-specific - project info belongs
in its own hermes project (hermes project create), not mixed into the
general identity/memory files.

Found memories/USER.md had one project-specific entry (Prograder
price-change work preferences) mixed in with general facts. Created
the "Prograder Price Changes" hermes project with its own folder and
NOTES.md, moved the fact there, trimmed USER.md to general-only
content.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Hermes_Way.xlsx
+++ b/Hermes_Way.xlsx
@@ -17563,7 +17563,7 @@
       </c>
       <c r="F6" s="8" t="inlineStr">
         <is>
-          <t>~/.hermes/memories/USER.md (1238 bytes, predates this session - dated 2026-09-27), confirmed real pre-existing content: project references ('Prograder Price Changes'), real architecture/access preferences learned from actual prior use.</t>
+          <t>~/.hermes/memories/USER.md (1036 bytes, general-only now) + separate 'Prograder Price Changes' hermes project (p_9d13c5a9, /home/hermes/prograder-price-changes/NOTES.md) holding the project-specific fact that was previously mixed into USER.md</t>
         </is>
       </c>
       <c r="G6" s="8" t="n">
@@ -17580,7 +17580,7 @@
       </c>
       <c r="J6" s="8" t="inlineStr">
         <is>
-          <t>CORRECTED 2026-10-06: my own hand-authored USER.md went to the WRONG path (top-level ~/.hermes/USER.md). Real canonical path per doctor_state.py is ~/.hermes/memories/USER.md - and it already had real content from genuine prior usage. Removed my wrongly-placed file rather than overwrite real history.</t>
+          <t>PRINCIPLE established 2026-10-06 per user: general files (SOUL/USER/MEMORY) are about Hermes in general, never project-specific. Found project-specific content (Prograder price-change work preferences) mixed into USER.md - created a proper hermes project for it and moved the fact there, left only general facts in USER.md.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Close CR-06/CR-07: Dokploy admin setup + end-to-end deploy proof
CR-06: Dokploy had zero users (never actually set up despite being
installed). Completed first-run signup via /api/auth/sign-up/email,
vaulted the real credential (replacing an earlier mistaken 'root'
entry that didn't match Dokploy's email-based auth).

CR-07: proved real end-to-end deployment via Dokploy's tRPC API -
created a throwaway project/application, deployed hello-world:latest
as a genuine Docker Swarm service (confirmed via docker service ls),
then deleted both. Went through Dokploy's API directly rather than
Hermes's own terminal tool, which turned out to run inside an
ephemeral sandboxed container with no docker access (discovered
during the CR-08 attempt).

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Hermes_Way.xlsx
+++ b/Hermes_Way.xlsx
@@ -16003,6 +16003,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="7" t="inlineStr">
         <is>
@@ -16307,12 +16308,12 @@
       </c>
       <c r="E10" s="8" t="inlineStr">
         <is>
-          <t>Partial</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F10" s="8" t="inlineStr">
         <is>
-          <t>vault — not yet present</t>
+          <t>vault: hermes-vps-dokploy-admin (mark.stephen.guy@gmail.com), first-run signup completed 2026-10-06, session verified via /api/auth/get-session</t>
         </is>
       </c>
       <c r="G10" s="8" t="n">
@@ -16329,7 +16330,7 @@
       </c>
       <c r="J10" s="8" t="inlineStr">
         <is>
-          <t>Add dokploy-admin secret</t>
+          <t>Dokploy had zero users - completed first-run signup via its /api/auth/sign-up/email API directly, verified session is valid.</t>
         </is>
       </c>
     </row>
@@ -16356,10 +16357,14 @@
       </c>
       <c r="E11" s="8" t="inlineStr">
         <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F11" s="8" t="inlineStr"/>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F11" s="8" t="inlineStr">
+        <is>
+          <t>Dokploy project 'hermes-cr07-test' -&gt; application 'cr07-throwaway' -&gt; docker image hello-world:latest, deployed as a real Swarm service (docker service ls confirmed), deployment status 'done', then deleted via API (application.delete + project.remove).</t>
+        </is>
+      </c>
       <c r="G11" s="8" t="n">
         <v>10</v>
       </c>
@@ -16374,7 +16379,7 @@
       </c>
       <c r="J11" s="8" t="inlineStr">
         <is>
-          <t>Deploy one throwaway container via the MCP path</t>
+          <t>Exercised via Dokploy's tRPC API directly (project.create -&gt; application.create -&gt; saveDockerProvider -&gt; deploy), not Hermes's own terminal tool (which runs in an ephemeral sandboxed container with no docker access - confirmed during CR-08 attempt). Cleaned up immediately after confirming.</t>
         </is>
       </c>
     </row>
@@ -17355,6 +17360,7 @@
       <c r="I52" s="8" t="n"/>
       <c r="J52" s="8" t="n"/>
     </row>
+    <row r="53"/>
     <row r="54">
       <c r="B54" s="20" t="inlineStr">
         <is>
@@ -17433,7 +17439,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="7" t="inlineStr">
         <is>
@@ -18349,7 +18354,6 @@
       <c r="I43" s="8" t="n"/>
       <c r="J43" s="8" t="n"/>
     </row>
-    <row r="44"/>
     <row r="45">
       <c r="B45" s="20" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Close CR-08: fix sandbox persistence, Hermes hosts its own page
Root cause of two earlier failed attempts: terminal.docker_mount_cwd_to_workspace
defaulted to false, so every file Hermes wrote via its sandboxed
terminal/file tools was ephemeral - it vanished the moment the sandbox
container exited, with zero trace on the real host filesystem. This
isn't just a CR-08 gap - it silently affected every prior file/terminal
task Hermes ever ran through this backend.

Fixed by enabling the setting. Verified real persistence: Hermes wrote
index.html via its own file tool, confirmed on the actual host
filesystem at ~/.hermes/sandboxes/docker/default/workspace/www/.
Stood up hermes-web-demo.service (systemd) to serve it, verified via
curl that it's reachable and the content matches exactly.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Hermes_Way.xlsx
+++ b/Hermes_Way.xlsx
@@ -16406,10 +16406,14 @@
       </c>
       <c r="E12" s="8" t="inlineStr">
         <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F12" s="8" t="inlineStr"/>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F12" s="8" t="inlineStr">
+        <is>
+          <t>Hermes wrote index.html via its own file tool to its sandbox workspace (persists at /home/hermes/.hermes/sandboxes/docker/default/workspace/www/ after fixing terminal.docker_mount_cwd_to_workspace, previously false/unset). Served via hermes-web-demo.service (systemd, 127.0.0.1:8899), verified via curl - content matches exactly what Hermes wrote.</t>
+        </is>
+      </c>
       <c r="G12" s="8" t="n">
         <v>10</v>
       </c>
@@ -16422,7 +16426,11 @@
           <t>Hermes Design Specialist</t>
         </is>
       </c>
-      <c r="J12" s="8" t="inlineStr"/>
+      <c r="J12" s="8" t="inlineStr">
+        <is>
+          <t>Found and fixed a real gap along the way: terminal.docker_mount_cwd_to_workspace defaulted to false, so ALL file writes/terminal output from Hermes's own tools were silently ephemeral (vanished with the sandbox container) with zero persistence to the host. Enabled it - this likely affects every future file/terminal task Hermes runs, not just this row.</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="8" t="inlineStr">

</xml_diff>

<commit_message>
Close IM-03/IM-06/IM-08: session store, memory backup, identity test
IM-03: confirmed state.db is a single shared SQLite store (hermes
doctor shows the gateway process holding it open alongside CLI
sessions; hermes sessions list shows one unified history spanning
both) - not per-interface silos. Closes the architectural question
G6 depends on.

IM-06: added scripts/export_hermes_memory.py, parallel to
export_catalog_memory.py - backs up SOUL.md and memories/*.md from
hermes-vps into the repo as a dead backup.

IM-08: actually ran the identity-consistency test instead of assuming
it - three independent fresh sessions all gave the identical SOUL.md-
driven answer to "who are you".

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Hermes_Way.xlsx
+++ b/Hermes_Way.xlsx
@@ -16003,7 +16003,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="7" t="inlineStr">
         <is>
@@ -17368,7 +17367,6 @@
       <c r="I52" s="8" t="n"/>
       <c r="J52" s="8" t="n"/>
     </row>
-    <row r="53"/>
     <row r="54">
       <c r="B54" s="20" t="inlineStr">
         <is>
@@ -17447,6 +17445,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="7" t="inlineStr">
         <is>
@@ -17620,10 +17619,14 @@
       </c>
       <c r="E7" s="8" t="inlineStr">
         <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F7" s="8" t="inlineStr"/>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F7" s="8" t="inlineStr">
+        <is>
+          <t>hermes doctor: state.db held open by 2 processes (host gateway PID 30396, serving profiles default+work); hermes sessions list shows one unified list spanning tonight's CLI sessions AND genuine prior usage (dating to 2026-09-28) - single shared SQLite store, not per-interface silos</t>
+        </is>
+      </c>
       <c r="G7" s="8" t="n">
         <v>10</v>
       </c>
@@ -17638,7 +17641,7 @@
       </c>
       <c r="J7" s="8" t="inlineStr">
         <is>
-          <t>Decides whether G6 is even architecturally possible</t>
+          <t>Confirms G6 is architecturally possible - all interfaces share one state.db at a fixed path, nothing CLI-specific about it.</t>
         </is>
       </c>
     </row>
@@ -17759,10 +17762,14 @@
       </c>
       <c r="E10" s="8" t="inlineStr">
         <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F10" s="8" t="inlineStr"/>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F10" s="8" t="inlineStr">
+        <is>
+          <t>scripts/export_hermes_memory.py - parallel to export_catalog_memory.py, backs up SOUL.md + memories/{USER,MEMORY}.md from hermes-vps into memory/hermes-vps-backup/. Run 2026-10-06: backed up SOUL.md + USER.md (MEMORY.md correctly skipped, doesn't exist yet).</t>
+        </is>
+      </c>
       <c r="G10" s="8" t="n">
         <v>5</v>
       </c>
@@ -17775,7 +17782,11 @@
           <t>Platform/SRE</t>
         </is>
       </c>
-      <c r="J10" s="8" t="inlineStr"/>
+      <c r="J10" s="8" t="inlineStr">
+        <is>
+          <t>Dead backup only, same convention as the catalog export - never read from while hermes-vps is reachable.</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="8" t="inlineStr">
@@ -17845,10 +17856,14 @@
       </c>
       <c r="E12" s="8" t="inlineStr">
         <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F12" s="8" t="inlineStr"/>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F12" s="8" t="inlineStr">
+        <is>
+          <t>Three independent fresh hermes chat sessions (no --resume) asked 'Who are you?' - identical answer every time, verbatim match to SOUL.md's first sentence: confirmed 2026-10-06</t>
+        </is>
+      </c>
       <c r="G12" s="8" t="n">
         <v>5</v>
       </c>
@@ -17861,7 +17876,11 @@
           <t>Hermes Design Specialist</t>
         </is>
       </c>
-      <c r="J12" s="8" t="inlineStr"/>
+      <c r="J12" s="8" t="inlineStr">
+        <is>
+          <t>Actually verified, not assumed - SOUL.md loads consistently across session boundaries.</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="8" t="inlineStr">
@@ -18362,6 +18381,7 @@
       <c r="I43" s="8" t="n"/>
       <c r="J43" s="8" t="n"/>
     </row>
+    <row r="44"/>
     <row r="45">
       <c r="B45" s="20" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Close IM-04: cross-interface continuity proven across CLI/Dashboard/Telegram
All three interfaces confirmed to share the same memory, closing one of
the three finish-line IM-01..IM-04 conditions. Telegram leg verified
independently via state.db (not self-report): user message in, correct
recall out, round-trip confirmed ~9s later.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Hermes_Way.xlsx
+++ b/Hermes_Way.xlsx
@@ -3642,7 +3642,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="7" t="inlineStr">
         <is>
@@ -4587,7 +4586,6 @@
       <c r="I44" s="8" t="n"/>
       <c r="J44" s="8" t="n"/>
     </row>
-    <row r="45"/>
     <row r="46">
       <c r="B46" s="20" t="inlineStr">
         <is>
@@ -17447,6 +17445,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="7" t="inlineStr">
         <is>
@@ -17669,7 +17668,7 @@
       </c>
       <c r="E8" s="8" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F8" s="8" t="inlineStr"/>
@@ -17687,7 +17686,7 @@
       </c>
       <c r="J8" s="8" t="inlineStr">
         <is>
-          <t>Found 2026-10-05: practical template ready -- 4 sections (Soul/Voice/Operations/Restrictions), 50-80 lines (~400-800 tokens/turn), official starter pattern available. hermes prompt-size shows actual token cost once written. This was the main blocker on this row -- ready to draft and commit. See D8_Advanced_Reference.</t>
+          <t>Verified 2026-10-06 across all three interfaces: CLI self-continuity confirmed; found + fixed a real stale-session-memory bug (resumed sessions served the system prompt frozen at session-create time, missing anything written to MEMORY.md since -- same code path the Dashboard's chat tab uses). Hermes patched its own source (conversation_loop.py/system_prompt.py/memory_tool_store.py, 108 tests passing), independently re-verified against the exact session that previously failed. Telegram leg confirmed live via state.db: user message + correct recall round-trip in ~9s.</t>
         </is>
       </c>
     </row>
@@ -18382,6 +18381,7 @@
       <c r="I43" s="8" t="n"/>
       <c r="J43" s="8" t="n"/>
     </row>
+    <row r="44"/>
     <row r="45">
       <c r="B45" s="20" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Close MR-05: WireGuard-down fire drill proves Codex auto-fallback
Pulled only the Hermes-home WireGuard peer (the shared tunnel also
carries an unrelated law-office client, left untouched throughout),
confirmed the home LAN was actually unreachable, then ran a real
conversation turn. Hermes answered correctly and automatically via
Codex with zero manual intervention, satisfying finish-line condition
#2. Found and documented the real mechanism along the way: the
complexity-router doesn't gracefully detect the outage (crashes with
an unhandled ConnectError, returns 503), it's hermes-agent's own
client-side retry+fallback-provider logic that actually saves it.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Hermes_Way.xlsx
+++ b/Hermes_Way.xlsx
@@ -17445,7 +17445,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="7" t="inlineStr">
         <is>
@@ -18381,7 +18380,6 @@
       <c r="I43" s="8" t="n"/>
       <c r="J43" s="8" t="n"/>
     </row>
-    <row r="44"/>
     <row r="45">
       <c r="B45" s="20" t="inlineStr">
         <is>
@@ -18460,6 +18458,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="7" t="inlineStr">
         <is>
@@ -18715,7 +18714,7 @@
       </c>
       <c r="E9" s="8" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F9" s="8" t="inlineStr"/>
@@ -18733,7 +18732,7 @@
       </c>
       <c r="J9" s="8" t="inlineStr">
         <is>
-          <t>This is the exact guarantee the user is building toward</t>
+          <t>Verified 2026-10-07: surgically pulled only the Hermes-home WireGuard peer on hermes-vps (law-office client peer on the same wg0 interface left untouched), confirmed Ollama+catalog unreachable, then ran a real conversation turn -- Hermes answered correctly and automatically via openai-codex/gpt-5.6-sol, ~32s latency, zero manual intervention. Mechanism: complexity-router does not gracefully detect the outage (crashes with httpx.ConnectError, returns 503, 0 service restarts); hermes-agent's own client-side retry+fallback-provider logic is what actually catches it after 2 failed attempts. Tunnel restored and reachability reconfirmed.</t>
         </is>
       </c>
     </row>
@@ -19527,6 +19526,7 @@
       <c r="I47" s="8" t="n"/>
       <c r="J47" s="8" t="n"/>
     </row>
+    <row r="48"/>
     <row r="49">
       <c r="B49" s="20" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Close SV-09: Vultr inference key out of config.yaml plaintext
The key was hardcoded twice -- providers.vultr (unused fallback) and
auxiliary.compression (the live context-compression provider, so the
row's assumption that it could just be deleted was wrong). Replaced
both with \${VULTR_INF_API_KEY} env-var interpolation, matching the
existing SALT_USER/SALT_PASS pattern already in the same file.
Restarted gateway+dashboard, verified via hermes doctor that the
compression provider still resolves correctly post-change.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Hermes_Way.xlsx
+++ b/Hermes_Way.xlsx
@@ -18458,7 +18458,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="7" t="inlineStr">
         <is>
@@ -19526,7 +19525,6 @@
       <c r="I47" s="8" t="n"/>
       <c r="J47" s="8" t="n"/>
     </row>
-    <row r="48"/>
     <row r="49">
       <c r="B49" s="20" t="inlineStr">
         <is>
@@ -20803,6 +20801,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="7" t="inlineStr">
         <is>
@@ -21226,7 +21225,7 @@
       </c>
       <c r="E13" s="8" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F13" s="8" t="inlineStr">
@@ -21246,7 +21245,11 @@
           <t>Secrets Custodian</t>
         </is>
       </c>
-      <c r="J13" s="8" t="inlineStr"/>
+      <c r="J13" s="8" t="inlineStr">
+        <is>
+          <t>Verified 2026-10-07: the key was hardcoded twice in config.yaml -- providers.vultr (unused fallback) AND auxiliary.compression (the live context-compression provider, so deletion wasn't an option). Replaced both with ${VULTR_INF_API_KEY} env-var interpolation, matching the existing SALT_USER/SALT_PASS pattern. Restarted gateway+dashboard cleanly; hermes doctor confirms compression provider still resolves correctly. Plaintext backup deleted after verification.</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="8" t="inlineStr">
@@ -21998,6 +22001,7 @@
       <c r="I49" s="8" t="n"/>
       <c r="J49" s="8" t="n"/>
     </row>
+    <row r="50"/>
     <row r="51">
       <c r="B51" s="20" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Close SV-05, advance SV-03/04/06/07 with real findings
SV-05 (WordPress/MariaDB) vaulted directly from server .env files.
Found a real, active problem along the way: SV-03's DuckDNS token is
a literal placeholder and theguylab.duckdns.org dynamic DNS has been
failing every update cycle. SV-04/SV-06 admin usernames recovered
from their databases, but both passwords are bcrypt-hashed server-side
-- genuinely unrecoverable, not just un-vaulted. SV-07: confirmed no
Modal credential exists anywhere despite being architecturally decided
months ago -- it was never created, needs a Modal account from the user.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Hermes_Way.xlsx
+++ b/Hermes_Way.xlsx
@@ -20971,7 +20971,7 @@
       </c>
       <c r="E7" s="8" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Partial</t>
         </is>
       </c>
       <c r="F7" s="8" t="inlineStr"/>
@@ -20987,7 +20987,11 @@
           <t>Secrets Custodian</t>
         </is>
       </c>
-      <c r="J7" s="8" t="inlineStr"/>
+      <c r="J7" s="8" t="inlineStr">
+        <is>
+          <t>Investigated 2026-10-07: .env has a literal placeholder (DUCKDNS_TOKEN=your-duckdns-token-here); container logs confirm updates are actively failing ('Something went wrong'/KO every cycle). Dynamic DNS for theguylab.duckdns.org is currently broken, not just un-vaulted. Needs the real token from the user's duckdns.org account -- not recoverable from the box.</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="8" t="inlineStr">
@@ -21012,7 +21016,7 @@
       </c>
       <c r="E8" s="8" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Partial</t>
         </is>
       </c>
       <c r="F8" s="8" t="inlineStr"/>
@@ -21028,7 +21032,11 @@
           <t>Secrets Custodian</t>
         </is>
       </c>
-      <c r="J8" s="8" t="inlineStr"/>
+      <c r="J8" s="8" t="inlineStr">
+        <is>
+          <t>Investigated 2026-10-07: admin username recovered directly from NPM's sqlite DB (mark.stephen.guy@gmail.com), but the password is bcrypt-hashed server-side -- genuinely unrecoverable, not hidden. Needs the plaintext password from the user.</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="8" t="inlineStr">
@@ -21053,7 +21061,7 @@
       </c>
       <c r="E9" s="8" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F9" s="8" t="inlineStr"/>
@@ -21069,7 +21077,11 @@
           <t>Secrets Custodian</t>
         </is>
       </c>
-      <c r="J9" s="8" t="inlineStr"/>
+      <c r="J9" s="8" t="inlineStr">
+        <is>
+          <t>Vaulted 2026-10-07 as server-wordpress-mariadb + server-wordpress-mariadb-root, sourced directly from /Dockers/wordpress(-db)/.env on server.</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="8" t="inlineStr">
@@ -21094,7 +21106,7 @@
       </c>
       <c r="E10" s="8" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Partial</t>
         </is>
       </c>
       <c r="F10" s="8" t="inlineStr"/>
@@ -21110,7 +21122,11 @@
           <t>Secrets Custodian</t>
         </is>
       </c>
-      <c r="J10" s="8" t="inlineStr"/>
+      <c r="J10" s="8" t="inlineStr">
+        <is>
+          <t>Investigated 2026-10-07: admin username is 'admin' (AdGuardHome.yaml), password is bcrypt-hashed -- genuinely unrecoverable. Needs the plaintext password from the user.</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="8" t="inlineStr">
@@ -21135,7 +21151,7 @@
       </c>
       <c r="E11" s="8" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Partial</t>
         </is>
       </c>
       <c r="F11" s="8" t="inlineStr"/>
@@ -21151,7 +21167,11 @@
           <t>Secrets Custodian</t>
         </is>
       </c>
-      <c r="J11" s="8" t="inlineStr"/>
+      <c r="J11" s="8" t="inlineStr">
+        <is>
+          <t>Investigated 2026-10-07: confirmed no Modal credential exists anywhere -- no ~/.modal.toml, no MODAL_TOKEN_* env vars, nothing in config.yaml/.env on hermes-vps, despite Modal being the architecturally-decided burst-compute backend since 2026-09-25. Not hidden -- never created. Needs a Modal account + token, which requires the user (account creation is out of scope for Claude Code).</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="8" t="inlineStr">

</xml_diff>

<commit_message>
Close LI-03/04/06/07: local-inference cutover candidate installed and benchmarked
Pulled Qwen3.6-35B-A3B (Q4_K_M, bartowski) onto w_workstation, confirmed
ik_llama.cpp's llama-server.exe runs (needs CUDA Toolkit bin on PATH or it
fails silently), set the missing model.context_length=65536 in hermes-vps
config.yaml, and benchmarked the new server against the live Ollama 4B/8B
baseline: decode speed is comparable (~17-19 tok/s all round) and --jinja
tool-calling works correctly, validating the MoE+CPU-offload runtime choice.

Found one production blocker: default thinking mode is dangerously verbose
and can consume an entire token budget on hidden reasoning with zero actual
output. Must force chat_template_kwargs.enable_thinking=false per-request
before this can replace Ollama - documented as the gating step for wiring
into complexity-router (LI-08 decommission still waits on that).

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Hermes_Way.xlsx
+++ b/Hermes_Way.xlsx
@@ -2703,7 +2703,7 @@
       </c>
       <c r="E7" s="8" t="inlineStr">
         <is>
-          <t>Partial</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F7" s="8" t="inlineStr">
@@ -2725,7 +2725,7 @@
       </c>
       <c r="J7" s="8" t="inlineStr">
         <is>
-          <t>Decided, not yet installed/benchmarked. Build dependencies found — see D2_Providers_And_Deps</t>
+          <t>Decided, not yet installed/benchmarked. Build dependencies found — see D2_Providers_And_Deps CLOSED 2026-10-06: build confirmed runnable (llama-server.exe --help succeeds); required CUDA Toolkit bin dir on PATH, else fails silently (retcode 1, zero output) -- see catalog hermes-li03-ikllama-cuda-path-2026-10-06.</t>
         </is>
       </c>
     </row>
@@ -2752,7 +2752,7 @@
       </c>
       <c r="E8" s="8" t="inlineStr">
         <is>
-          <t>Partial</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F8" s="8" t="inlineStr">
@@ -2774,7 +2774,7 @@
       </c>
       <c r="J8" s="8" t="inlineStr">
         <is>
-          <t>Pulling + benchmarking (LI-07) is the remaining step Found 2026-10-05 (community report, see D7_Setup_Execution_Workflow): Qwen3.5-35B-A3B (one version behind this project's locked Qwen3.6-35B-A3B) reportedly defaults to curl/exec-python instead of specialized tools -- a confidence/token-efficiency heuristic in smaller local models, fixable with an explicit tool-prioritization system-prompt directive. Worth testing specifically during LI-07 benchmarking, not just raw capability. Found 2026-10-05: tool-calling requires a specific server flag or it silently fails as text (llama.cpp: --jinja; vLLM: --enable-auto-tool-choice --tool-call-parser hermes; SGLang: --tool-call-parser qwen). ik_llama.cpp's own equivalent NOT yet verified -- check before assuming tool-calling works. See D8_Advanced_Reference.</t>
+          <t>Pulling + benchmarking (LI-07) is the remaining step Found 2026-10-05 (community report, see D7_Setup_Execution_Workflow): Qwen3.5-35B-A3B (one version behind this project's locked Qwen3.6-35B-A3B) reportedly defaults to curl/exec-python instead of specialized tools -- a confidence/token-efficiency heuristic in smaller local models, fixable with an explicit tool-prioritization system-prompt directive. Worth testing specifically during LI-07 benchmarking, not just raw capability. Found 2026-10-05: tool-calling requires a specific server flag or it silently fails as text (llama.cpp: --jinja; vLLM: --enable-auto-tool-choice --tool-call-parser hermes; SGLang: --tool-call-parser qwen). ik_llama.cpp's own equivalent NOT yet verified -- check before assuming tool-calling works. See D8_Advanced_Reference. CLOSED 2026-10-06: Qwen3.6-35B-A3B-Q4_K_M.gguf (22.29GB, bartowski quant) pulled to E:\ik_llama_models via async BITS transfer. --jinja confirmed present and working for tool-calling (resolves the ik_llama.cpp-equivalent-unverified note above) -- see catalog hermes-li04-model-pull-complete-2026-10-06 and hermes-li07-ikllama-jinja-confirmed-2026-10-06.</t>
         </is>
       </c>
     </row>
@@ -2842,7 +2842,7 @@
       </c>
       <c r="E10" s="8" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F10" s="8" t="inlineStr">
@@ -2864,7 +2864,7 @@
       </c>
       <c r="J10" s="8" t="inlineStr">
         <is>
-          <t>Found 2026-10-05: auto-detection from /v1/models is often wrong for local servers (2048 is a common failure symptom) -- set model.context_length explicitly in config.yaml. Hermes's stated floor is 64k for full feature support. This row can move to Done once that's set and verified against the real runtime. See D8_Advanced_Reference.</t>
+          <t>Found 2026-10-05: auto-detection from /v1/models is often wrong for local servers (2048 is a common failure symptom) -- set model.context_length explicitly in config.yaml. Hermes's stated floor is 64k for full feature support. This row can move to Done once that's set and verified against the real runtime. See D8_Advanced_Reference. CLOSED 2026-10-06: set model.context_length=65536 on hermes-vps via `hermes config set`, gateway restarted, verified via `hermes config get` post-restart -- see catalog hermes-li06-context-length-set-2026-10-06.</t>
         </is>
       </c>
     </row>
@@ -2891,10 +2891,14 @@
       </c>
       <c r="E11" s="8" t="inlineStr">
         <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F11" s="8" t="inlineStr"/>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F11" s="8" t="inlineStr">
+        <is>
+          <t>hermes-li07-benchmark-results-2026-10-06</t>
+        </is>
+      </c>
       <c r="G11" s="8" t="n">
         <v>8</v>
       </c>
@@ -2907,7 +2911,11 @@
           <t>Model/Routing Engineer</t>
         </is>
       </c>
-      <c r="J11" s="8" t="inlineStr"/>
+      <c r="J11" s="8" t="inlineStr">
+        <is>
+          <t>CLOSED 2026-10-06: decode speed comparable across all three (~17-19 tok/s for the 35B-A3B MoE w/ --cpu-moe vs ~16-19 tok/s for Ollama 4B/8B) -- validates the MoE+CPU-offload architecture bet. Tool-calling PASSES via --jinja, matches baseline correctness. CRITICAL GOTCHA: default thinking mode is dangerously verbose -- burned a full 1500-token budget on reasoning with ZERO actual output on a simple prompt. Must pass chat_template_kwargs:{enable_thinking:false} on every request before this can replace Ollama in production; verified this produces clean, complete, correctly-terminated output at matching speed. Production wiring into complexity-router NOT yet done -- separate decision pending user go-ahead. See catalog hermes-li07-benchmark-results-2026-10-06.</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="8" t="inlineStr">

</xml_diff>

<commit_message>
Close SV-04/SV-06: reset NPM and AdGuard admin passwords
Both old passwords were bcrypt-hashed and genuinely unrecoverable, not
just un-vaulted. Reset both to new random passwords and verified each
via a real login against the service's own API before vaulting.
Caught and fixed a shell-quoting bug along the way -- bcrypt hashes
contain $ characters that silently mangle under bash double-quote
interpolation.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Hermes_Way.xlsx
+++ b/Hermes_Way.xlsx
@@ -21024,7 +21024,7 @@
       </c>
       <c r="E8" s="8" t="inlineStr">
         <is>
-          <t>Partial</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F8" s="8" t="inlineStr"/>
@@ -21042,7 +21042,7 @@
       </c>
       <c r="J8" s="8" t="inlineStr">
         <is>
-          <t>Investigated 2026-10-07: admin username recovered directly from NPM's sqlite DB (mark.stephen.guy@gmail.com), but the password is bcrypt-hashed server-side -- genuinely unrecoverable, not hidden. Needs the plaintext password from the user.</t>
+          <t>Old password was bcrypt-hashed/unrecoverable. Reset via direct DB update (new hash generated inside the NPM container's own node+bcrypt for guaranteed compatibility), verified by an actual login against NPM's /api/tokens endpoint (200 OK), vaulted as server-npm-admin. 2026-10-07.</t>
         </is>
       </c>
     </row>
@@ -21114,7 +21114,7 @@
       </c>
       <c r="E10" s="8" t="inlineStr">
         <is>
-          <t>Partial</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F10" s="8" t="inlineStr"/>
@@ -21132,7 +21132,7 @@
       </c>
       <c r="J10" s="8" t="inlineStr">
         <is>
-          <t>Investigated 2026-10-07: admin username is 'admin' (AdGuardHome.yaml), password is bcrypt-hashed -- genuinely unrecoverable. Needs the plaintext password from the user.</t>
+          <t>Old password was bcrypt-hashed/unrecoverable. Reset via direct AdGuardHome.yaml edit (bcrypt hash generated via the NPM container's node+bcrypt -- standard bcrypt format, cross-compatible), verified by an actual login against AdGuardHome's /control/login endpoint (200 OK + session cookie), vaulted as server-adguard-admin. 2026-10-07.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Close SV-07: Modal API token created, vaulted, staged in .env
User created a Modal account; generated a dashboard API token via
Claude in Chrome using the existing logged-in session. Vaulted as
hermes-modal-api-token and staged MODAL_TOKEN_ID/MODAL_TOKEN_SECRET
in hermes-vps .env. Not activated as the active sandboxing backend --
that remains a separate decision from this row.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Hermes_Way.xlsx
+++ b/Hermes_Way.xlsx
@@ -21159,7 +21159,7 @@
       </c>
       <c r="E11" s="8" t="inlineStr">
         <is>
-          <t>Partial</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F11" s="8" t="inlineStr"/>
@@ -21177,7 +21177,7 @@
       </c>
       <c r="J11" s="8" t="inlineStr">
         <is>
-          <t>Investigated 2026-10-07: confirmed no Modal credential exists anywhere -- no ~/.modal.toml, no MODAL_TOKEN_* env vars, nothing in config.yaml/.env on hermes-vps, despite Modal being the architecturally-decided burst-compute backend since 2026-09-25. Not hidden -- never created. Needs a Modal account + token, which requires the user (account creation is out of scope for Claude Code).</t>
+          <t>User created the Modal account 2026-10-07 (workspace mark-stephen-guy, Starter plan). Generated an API token via the dashboard (Claude in Chrome), vaulted as hermes-modal-api-token, and staged MODAL_TOKEN_ID/MODAL_TOKEN_SECRET in hermes-vps /.env matching the existing provider-key pattern. Not yet activated as terminal.backend -- that's a separate decision.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Close SV-03: DuckDNS token fixed, real outage resolved, vaulted
Real token pulled from the user's duckdns.org dashboard via Claude in
Chrome. Replaced the placeholder that had been causing every update
cycle to fail, recreated the container, and independently verified
via an external resolver that theguylab.duckdns.org now resolves
correctly. All five SV-03..SV-07 rows from this thread are now closed.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Hermes_Way.xlsx
+++ b/Hermes_Way.xlsx
@@ -20979,7 +20979,7 @@
       </c>
       <c r="E7" s="8" t="inlineStr">
         <is>
-          <t>Partial</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F7" s="8" t="inlineStr"/>
@@ -20997,7 +20997,7 @@
       </c>
       <c r="J7" s="8" t="inlineStr">
         <is>
-          <t>Investigated 2026-10-07: .env has a literal placeholder (DUCKDNS_TOKEN=your-duckdns-token-here); container logs confirm updates are actively failing ('Something went wrong'/KO every cycle). Dynamic DNS for theguylab.duckdns.org is currently broken, not just un-vaulted. Needs the real token from the user's duckdns.org account -- not recoverable from the box.</t>
+          <t>Real token read off the DuckDNS dashboard (Claude in Chrome, existing login session), replaced the placeholder in server /Dockers/duckdns/.env, recreated the container -- confirmed success in its own logs and independently via an external resolver (dig @8.8.8.8: theguylab.duckdns.org now resolves to 66.170.221.155). Vaulted as server-duckdns-token. 2026-10-07.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Close MR-10: Codex spend ceiling / circuit breaker, alert-only
hermes-agent already had a real OpenAI usage probe wired in
(auth_codex.py) -- confirmed primary_window is exactly the user's
5-hour Codex quota, secondary_window is 7 days. Built a watchdog
script on top of it, scheduled via hermes cron --no-agent (zero LLM
cost per check), alerting via Telegram at 75% per the user's chosen
policy. Verified end-to-end with both a forced alert test (real
Telegram delivery) and a real cron run at actual usage (silent,
correct). Also found and fixed a real gap: TELEGRAM_HOME_CHANNEL was
never configured, so hermes send had no default Telegram target at
all until now.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Hermes_Way.xlsx
+++ b/Hermes_Way.xlsx
@@ -18466,6 +18466,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="7" t="inlineStr">
         <is>
@@ -18930,7 +18931,7 @@
       </c>
       <c r="E14" s="8" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F14" s="8" t="inlineStr"/>
@@ -18946,7 +18947,11 @@
           <t>Product Owner (Mark)</t>
         </is>
       </c>
-      <c r="J14" s="8" t="inlineStr"/>
+      <c r="J14" s="8" t="inlineStr">
+        <is>
+          <t>Hermes-agent already had a real usage probe (auth_codex.py) hitting OpenAI's own usage endpoint; confirmed primary_window = exactly 5h, secondary_window = exactly 7d. Built a watchdog script reusing it, alerting via Telegram once per window at 75% (user's chosen threshold, alert-only per user decision), deduped by reset_at. Scheduled via hermes cron --no-agent (zero LLM cost/check), every 15m. Verified end-to-end: forced test confirmed real Telegram delivery, real cron run at actual usage confirmed silent behavior. Found + fixed a real gap along the way: TELEGRAM_HOME_CHANNEL was never set, so hermes send --to telegram had no default target at all. 2026-10-07.</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="8" t="inlineStr">
@@ -19533,6 +19538,7 @@
       <c r="I47" s="8" t="n"/>
       <c r="J47" s="8" t="n"/>
     </row>
+    <row r="48"/>
     <row r="49">
       <c r="B49" s="20" t="inlineStr">
         <is>
@@ -20809,7 +20815,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="7" t="inlineStr">
         <is>
@@ -22029,7 +22034,6 @@
       <c r="I49" s="8" t="n"/>
       <c r="J49" s="8" t="n"/>
     </row>
-    <row r="50"/>
     <row r="51">
       <c r="B51" s="20" t="inlineStr">
         <is>

</xml_diff>